<commit_message>
Orari: giornate intere e mezze giornate come nello schema del negozio, Laura alterna mattine e pomeriggi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RgW8tUpL59m5j1P2CKTdxn
</commit_message>
<xml_diff>
--- a/orari/Orari_12-18_ottobre_2026.xlsx
+++ b/orari/Orari_12-18_ottobre_2026.xlsx
@@ -107,10 +107,10 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -885,21 +885,25 @@
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="7" t="n">
+      <c r="G6" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="K6" s="7" t="n"/>
+      <c r="L6" s="7" t="n"/>
+      <c r="M6" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="J6" s="7" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="K6" s="6" t="n"/>
-      <c r="L6" s="6" t="n"/>
-      <c r="M6" s="7" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="N6" s="7" t="n">
-        <v>0.8333333333333334</v>
+      <c r="N6" s="6" t="n">
+        <v>0.75</v>
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
@@ -909,35 +913,39 @@
       <c r="P6" s="5" t="n"/>
       <c r="Q6" s="5" t="n"/>
       <c r="R6" s="5" t="n"/>
-      <c r="S6" s="6" t="n"/>
-      <c r="T6" s="6" t="n"/>
-      <c r="U6" s="7" t="n">
+      <c r="S6" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="T6" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="U6" s="6" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="V6" s="6" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="W6" s="7" t="n"/>
+      <c r="X6" s="7" t="n"/>
+      <c r="Y6" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="V6" s="7" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="W6" s="7" t="n">
-        <v>0.4583333333333333</v>
-      </c>
-      <c r="X6" s="7" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="Y6" s="6" t="n"/>
-      <c r="Z6" s="6" t="n"/>
-      <c r="AA6" s="6" t="n"/>
-      <c r="AB6" s="6" t="n"/>
-      <c r="AC6" s="7" t="n">
+      <c r="Z6" s="6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AA6" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="AB6" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="AD6" s="7" t="n">
-        <v>0.8333333333333334</v>
-      </c>
+      <c r="AC6" s="7" t="n"/>
+      <c r="AD6" s="7" t="n"/>
       <c r="AE6" s="8">
         <f>ROUND(24*(N(D6)-N(C6)+N(F6)-N(E6)+N(H6)-N(G6)+N(J6)-N(I6)+N(L6)-N(K6)+N(N6)-N(M6)+N(P6)-N(O6)+N(R6)-N(Q6)+N(T6)-N(S6)+N(V6)-N(U6)+N(X6)-N(W6)+N(Z6)-N(Y6)+N(AB6)-N(AA6)+N(AD6)-N(AC6)),2)</f>
         <v/>
       </c>
-      <c r="AF6" s="6" t="n">
+      <c r="AF6" s="7" t="n">
         <v>30</v>
       </c>
     </row>
@@ -952,17 +960,17 @@
           <t>Vicedirettore</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>0.5416666666666666</v>
-      </c>
-      <c r="E7" s="7" t="n">
+      <c r="C7" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="D7" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="F7" s="7" t="n">
-        <v>0.7083333333333334</v>
+      <c r="E7" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>0.875</v>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
@@ -972,52 +980,48 @@
       <c r="H7" s="5" t="n"/>
       <c r="I7" s="5" t="n"/>
       <c r="J7" s="5" t="n"/>
-      <c r="K7" s="7" t="n">
+      <c r="K7" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="O7" s="6" t="n">
         <v>0.4166666666666667</v>
       </c>
-      <c r="L7" s="7" t="n">
+      <c r="P7" s="6" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="M7" s="7" t="n">
+      <c r="Q7" s="6" t="n">
         <v>0.7083333333333334</v>
       </c>
-      <c r="N7" s="7" t="n">
+      <c r="R7" s="6" t="n">
         <v>0.875</v>
       </c>
-      <c r="O7" s="7" t="n">
+      <c r="S7" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="P7" s="7" t="n">
-        <v>0.5416666666666666</v>
-      </c>
-      <c r="Q7" s="7" t="n">
+      <c r="T7" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="U7" s="7" t="n"/>
+      <c r="V7" s="7" t="n"/>
+      <c r="W7" s="6" t="n">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="X7" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="R7" s="7" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="S7" s="7" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="T7" s="7" t="n">
+      <c r="Y7" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="U7" s="7" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="V7" s="7" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="W7" s="7" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="X7" s="7" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="Y7" s="7" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="Z7" s="7" t="n">
+      <c r="Z7" s="6" t="n">
         <v>0.875</v>
       </c>
       <c r="AA7" s="5" t="inlineStr">
@@ -1032,7 +1036,7 @@
         <f>ROUND(24*(N(D7)-N(C7)+N(F7)-N(E7)+N(H7)-N(G7)+N(J7)-N(I7)+N(L7)-N(K7)+N(N7)-N(M7)+N(P7)-N(O7)+N(R7)-N(Q7)+N(T7)-N(S7)+N(V7)-N(U7)+N(X7)-N(W7)+N(Z7)-N(Y7)+N(AB7)-N(AA7)+N(AD7)-N(AC7)),2)</f>
         <v/>
       </c>
-      <c r="AF7" s="6" t="inlineStr">
+      <c r="AF7" s="7" t="inlineStr">
         <is>
           <t>44-45</t>
         </is>
@@ -1049,29 +1053,25 @@
           <t>Addetto vendite</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="F8" s="7" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="G8" s="7" t="n">
+      <c r="C8" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="D8" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="H8" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="I8" s="7" t="n">
+      <c r="I8" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="J8" s="7" t="n">
-        <v>0.75</v>
+      <c r="J8" s="6" t="n">
+        <v>0.7916666666666666</v>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
@@ -1081,17 +1081,17 @@
       <c r="L8" s="5" t="n"/>
       <c r="M8" s="5" t="n"/>
       <c r="N8" s="5" t="n"/>
-      <c r="O8" s="7" t="n">
+      <c r="O8" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="P8" s="6" t="n">
         <v>0.5</v>
       </c>
-      <c r="P8" s="7" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="Q8" s="7" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="R8" s="7" t="n">
-        <v>0.875</v>
+      <c r="Q8" s="6" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="R8" s="6" t="n">
+        <v>0.7916666666666666</v>
       </c>
       <c r="S8" s="5" t="inlineStr">
         <is>
@@ -1101,35 +1101,31 @@
       <c r="T8" s="5" t="n"/>
       <c r="U8" s="5" t="n"/>
       <c r="V8" s="5" t="n"/>
-      <c r="W8" s="7" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="X8" s="7" t="n">
+      <c r="W8" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="X8" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="Y8" s="7" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="Z8" s="7" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="AA8" s="7" t="n">
+      <c r="Y8" s="7" t="n"/>
+      <c r="Z8" s="7" t="n"/>
+      <c r="AA8" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="AB8" s="7" t="n">
+      <c r="AB8" s="6" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="AC8" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="AC8" s="7" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="AD8" s="7" t="n">
-        <v>0.75</v>
+      <c r="AD8" s="6" t="n">
+        <v>0.8333333333333334</v>
       </c>
       <c r="AE8" s="8">
         <f>ROUND(24*(N(D8)-N(C8)+N(F8)-N(E8)+N(H8)-N(G8)+N(J8)-N(I8)+N(L8)-N(K8)+N(N8)-N(M8)+N(P8)-N(O8)+N(R8)-N(Q8)+N(T8)-N(S8)+N(V8)-N(U8)+N(X8)-N(W8)+N(Z8)-N(Y8)+N(AB8)-N(AA8)+N(AD8)-N(AC8)),2)</f>
         <v/>
       </c>
-      <c r="AF8" s="6" t="n">
+      <c r="AF8" s="7" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1144,17 +1140,17 @@
           <t>Addetto vendite</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="6" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="F9" s="7" t="n">
-        <v>0.7083333333333334</v>
+      <c r="F9" s="6" t="n">
+        <v>0.8333333333333334</v>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
@@ -1164,17 +1160,17 @@
       <c r="H9" s="5" t="n"/>
       <c r="I9" s="5" t="n"/>
       <c r="J9" s="5" t="n"/>
-      <c r="K9" s="7" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="L9" s="7" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="M9" s="7" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="N9" s="7" t="n">
-        <v>0.7916666666666666</v>
+      <c r="K9" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>0.875</v>
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
@@ -1184,47 +1180,39 @@
       <c r="P9" s="5" t="n"/>
       <c r="Q9" s="5" t="n"/>
       <c r="R9" s="5" t="n"/>
-      <c r="S9" s="7" t="n">
+      <c r="S9" s="7" t="n"/>
+      <c r="T9" s="7" t="n"/>
+      <c r="U9" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="V9" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="W9" s="7" t="n"/>
+      <c r="X9" s="7" t="n"/>
+      <c r="Y9" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="Z9" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="AA9" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="T9" s="7" t="n">
+      <c r="AB9" s="6" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="U9" s="7" t="n">
+      <c r="AC9" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="V9" s="7" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="W9" s="7" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="X9" s="7" t="n">
-        <v>0.5416666666666666</v>
-      </c>
-      <c r="Y9" s="7" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="Z9" s="7" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="AA9" s="7" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="AB9" s="7" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="AC9" s="7" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="AD9" s="7" t="n">
-        <v>0.875</v>
+      <c r="AD9" s="6" t="n">
+        <v>0.8333333333333334</v>
       </c>
       <c r="AE9" s="8">
         <f>ROUND(24*(N(D9)-N(C9)+N(F9)-N(E9)+N(H9)-N(G9)+N(J9)-N(I9)+N(L9)-N(K9)+N(N9)-N(M9)+N(P9)-N(O9)+N(R9)-N(Q9)+N(T9)-N(S9)+N(V9)-N(U9)+N(X9)-N(W9)+N(Z9)-N(Y9)+N(AB9)-N(AA9)+N(AD9)-N(AC9)),2)</f>
         <v/>
       </c>
-      <c r="AF9" s="6" t="n">
+      <c r="AF9" s="7" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1239,28 +1227,24 @@
           <t>Addetto vendite</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D10" s="7" t="n">
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="H10" s="6" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="I10" s="6" t="n">
         <v>0.7083333333333334</v>
       </c>
-      <c r="F10" s="7" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="G10" s="7" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="H10" s="7" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="I10" s="7" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="J10" s="7" t="n">
+      <c r="J10" s="6" t="n">
         <v>0.875</v>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -1271,55 +1255,51 @@
       <c r="L10" s="5" t="n"/>
       <c r="M10" s="5" t="n"/>
       <c r="N10" s="5" t="n"/>
-      <c r="O10" s="7" t="n">
+      <c r="O10" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="P10" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="Q10" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="R10" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="S10" s="7" t="n"/>
+      <c r="T10" s="7" t="n"/>
+      <c r="U10" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="V10" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="W10" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="P10" s="7" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="Q10" s="7" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="R10" s="7" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="S10" s="7" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="T10" s="7" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="U10" s="7" t="n">
+      <c r="X10" s="6" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="V10" s="7" t="n">
+      <c r="Y10" s="7" t="n"/>
+      <c r="Z10" s="7" t="n"/>
+      <c r="AA10" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="AB10" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="AC10" s="6" t="n">
         <v>0.7083333333333334</v>
       </c>
-      <c r="W10" s="7" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="X10" s="7" t="n">
-        <v>0.5416666666666666</v>
-      </c>
-      <c r="Y10" s="7" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="Z10" s="7" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="AA10" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="AB10" s="5" t="n"/>
-      <c r="AC10" s="5" t="n"/>
-      <c r="AD10" s="5" t="n"/>
+      <c r="AD10" s="6" t="n">
+        <v>0.875</v>
+      </c>
       <c r="AE10" s="8">
         <f>ROUND(24*(N(D10)-N(C10)+N(F10)-N(E10)+N(H10)-N(G10)+N(J10)-N(I10)+N(L10)-N(K10)+N(N10)-N(M10)+N(P10)-N(O10)+N(R10)-N(Q10)+N(T10)-N(S10)+N(V10)-N(U10)+N(X10)-N(W10)+N(Z10)-N(Y10)+N(AB10)-N(AA10)+N(AD10)-N(AC10)),2)</f>
         <v/>
       </c>
-      <c r="AF10" s="6" t="n">
+      <c r="AF10" s="7" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1342,29 +1322,29 @@
       <c r="D11" s="5" t="n"/>
       <c r="E11" s="5" t="n"/>
       <c r="F11" s="5" t="n"/>
-      <c r="G11" s="7" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H11" s="7" t="n">
+      <c r="G11" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="H11" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="I11" s="7" t="n">
+      <c r="I11" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="J11" s="7" t="n">
+      <c r="J11" s="6" t="n">
         <v>0.875</v>
       </c>
-      <c r="K11" s="7" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="L11" s="7" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="M11" s="7" t="n">
-        <v>0.5416666666666666</v>
-      </c>
-      <c r="N11" s="7" t="n">
-        <v>0.7083333333333334</v>
+      <c r="K11" s="6" t="n">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>0.875</v>
       </c>
       <c r="O11" s="5" t="inlineStr">
         <is>
@@ -1374,47 +1354,39 @@
       <c r="P11" s="5" t="n"/>
       <c r="Q11" s="5" t="n"/>
       <c r="R11" s="5" t="n"/>
-      <c r="S11" s="7" t="n">
+      <c r="S11" s="6" t="n">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="T11" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="U11" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="V11" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="W11" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="T11" s="7" t="n">
+      <c r="X11" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="U11" s="7" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="V11" s="7" t="n">
-        <v>0.7916666666666666</v>
-      </c>
-      <c r="W11" s="7" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="X11" s="7" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Y11" s="7" t="n">
-        <v>0.5416666666666666</v>
-      </c>
-      <c r="Z11" s="7" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="AA11" s="7" t="n">
-        <v>0.4583333333333333</v>
-      </c>
-      <c r="AB11" s="7" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="AC11" s="7" t="n">
+      <c r="Y11" s="7" t="n"/>
+      <c r="Z11" s="7" t="n"/>
+      <c r="AA11" s="7" t="n"/>
+      <c r="AB11" s="7" t="n"/>
+      <c r="AC11" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="AD11" s="7" t="n">
+      <c r="AD11" s="6" t="n">
         <v>0.875</v>
       </c>
       <c r="AE11" s="8">
         <f>ROUND(24*(N(D11)-N(C11)+N(F11)-N(E11)+N(H11)-N(G11)+N(J11)-N(I11)+N(L11)-N(K11)+N(N11)-N(M11)+N(P11)-N(O11)+N(R11)-N(Q11)+N(T11)-N(S11)+N(V11)-N(U11)+N(X11)-N(W11)+N(Z11)-N(Y11)+N(AB11)-N(AA11)+N(AD11)-N(AC11)),2)</f>
         <v/>
       </c>
-      <c r="AF11" s="6" t="n">
+      <c r="AF11" s="7" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1429,22 +1401,22 @@
           <t>Cassiera</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="7" t="n">
+      <c r="C12" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="D12" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="F12" s="7" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="n"/>
-      <c r="J12" s="5" t="n"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="I12" s="7" t="n"/>
+      <c r="J12" s="7" t="n"/>
       <c r="K12" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
@@ -1453,13 +1425,13 @@
       <c r="L12" s="5" t="n"/>
       <c r="M12" s="5" t="n"/>
       <c r="N12" s="5" t="n"/>
-      <c r="O12" s="6" t="n"/>
-      <c r="P12" s="6" t="n"/>
-      <c r="Q12" s="7" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="R12" s="7" t="n">
-        <v>0.875</v>
+      <c r="O12" s="7" t="n"/>
+      <c r="P12" s="7" t="n"/>
+      <c r="Q12" s="6" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="R12" s="6" t="n">
+        <v>0.7916666666666666</v>
       </c>
       <c r="S12" s="5" t="inlineStr">
         <is>
@@ -1469,27 +1441,27 @@
       <c r="T12" s="5" t="n"/>
       <c r="U12" s="5" t="n"/>
       <c r="V12" s="5" t="n"/>
-      <c r="W12" s="6" t="n"/>
-      <c r="X12" s="6" t="n"/>
-      <c r="Y12" s="7" t="n">
+      <c r="W12" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="X12" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="Z12" s="7" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="AA12" s="7" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="AB12" s="7" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="AC12" s="6" t="n"/>
-      <c r="AD12" s="6" t="n"/>
+      <c r="Y12" s="7" t="n"/>
+      <c r="Z12" s="7" t="n"/>
+      <c r="AA12" s="5" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="AB12" s="5" t="n"/>
+      <c r="AC12" s="5" t="n"/>
+      <c r="AD12" s="5" t="n"/>
       <c r="AE12" s="8">
         <f>ROUND(24*(N(D12)-N(C12)+N(F12)-N(E12)+N(H12)-N(G12)+N(J12)-N(I12)+N(L12)-N(K12)+N(N12)-N(M12)+N(P12)-N(O12)+N(R12)-N(Q12)+N(T12)-N(S12)+N(V12)-N(U12)+N(X12)-N(W12)+N(Z12)-N(Y12)+N(AB12)-N(AA12)+N(AD12)-N(AC12)),2)</f>
         <v/>
       </c>
-      <c r="AF12" s="6" t="n">
+      <c r="AF12" s="7" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1504,14 +1476,14 @@
           <t>Cassiera</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="D13" s="7" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
       <c r="G13" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
@@ -1520,38 +1492,38 @@
       <c r="H13" s="5" t="n"/>
       <c r="I13" s="5" t="n"/>
       <c r="J13" s="5" t="n"/>
-      <c r="K13" s="6" t="n"/>
-      <c r="L13" s="6" t="n"/>
-      <c r="M13" s="7" t="n">
+      <c r="K13" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="L13" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="N13" s="7" t="n">
+      <c r="M13" s="7" t="n"/>
+      <c r="N13" s="7" t="n"/>
+      <c r="O13" s="7" t="n"/>
+      <c r="P13" s="7" t="n"/>
+      <c r="Q13" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="R13" s="6" t="n">
         <v>0.875</v>
       </c>
-      <c r="O13" s="7" t="n">
+      <c r="S13" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="P13" s="7" t="n">
+      <c r="T13" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="Q13" s="6" t="n"/>
-      <c r="R13" s="6" t="n"/>
-      <c r="S13" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="T13" s="5" t="n"/>
-      <c r="U13" s="5" t="n"/>
-      <c r="V13" s="5" t="n"/>
-      <c r="W13" s="7" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="X13" s="7" t="n">
+      <c r="U13" s="7" t="n"/>
+      <c r="V13" s="7" t="n"/>
+      <c r="W13" s="7" t="n"/>
+      <c r="X13" s="7" t="n"/>
+      <c r="Y13" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="Y13" s="6" t="n"/>
-      <c r="Z13" s="6" t="n"/>
+      <c r="Z13" s="6" t="n">
+        <v>0.875</v>
+      </c>
       <c r="AA13" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
@@ -1564,7 +1536,7 @@
         <f>ROUND(24*(N(D13)-N(C13)+N(F13)-N(E13)+N(H13)-N(G13)+N(J13)-N(I13)+N(L13)-N(K13)+N(N13)-N(M13)+N(P13)-N(O13)+N(R13)-N(Q13)+N(T13)-N(S13)+N(V13)-N(U13)+N(X13)-N(W13)+N(Z13)-N(Y13)+N(AB13)-N(AA13)+N(AD13)-N(AC13)),2)</f>
         <v/>
       </c>
-      <c r="AF13" s="6" t="n">
+      <c r="AF13" s="7" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1579,67 +1551,67 @@
           <t>Cassiera</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="7" t="n">
+      <c r="H14" s="5" t="n"/>
+      <c r="I14" s="5" t="n"/>
+      <c r="J14" s="5" t="n"/>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="n"/>
+      <c r="M14" s="5" t="n"/>
+      <c r="N14" s="5" t="n"/>
+      <c r="O14" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="H14" s="7" t="n">
+      <c r="P14" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="I14" s="6" t="n"/>
-      <c r="J14" s="6" t="n"/>
-      <c r="K14" s="7" t="n">
+      <c r="Q14" s="7" t="n"/>
+      <c r="R14" s="7" t="n"/>
+      <c r="S14" s="5" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="T14" s="5" t="n"/>
+      <c r="U14" s="5" t="n"/>
+      <c r="V14" s="5" t="n"/>
+      <c r="W14" s="7" t="n"/>
+      <c r="X14" s="7" t="n"/>
+      <c r="Y14" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="Z14" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="AA14" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="L14" s="7" t="n">
+      <c r="AB14" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="M14" s="6" t="n"/>
-      <c r="N14" s="6" t="n"/>
-      <c r="O14" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="P14" s="5" t="n"/>
-      <c r="Q14" s="5" t="n"/>
-      <c r="R14" s="5" t="n"/>
-      <c r="S14" s="6" t="n"/>
-      <c r="T14" s="6" t="n"/>
-      <c r="U14" s="7" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="V14" s="7" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="W14" s="6" t="n"/>
-      <c r="X14" s="6" t="n"/>
-      <c r="Y14" s="7" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="Z14" s="7" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="AA14" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="AB14" s="5" t="n"/>
-      <c r="AC14" s="5" t="n"/>
-      <c r="AD14" s="5" t="n"/>
+      <c r="AC14" s="7" t="n"/>
+      <c r="AD14" s="7" t="n"/>
       <c r="AE14" s="8">
         <f>ROUND(24*(N(D14)-N(C14)+N(F14)-N(E14)+N(H14)-N(G14)+N(J14)-N(I14)+N(L14)-N(K14)+N(N14)-N(M14)+N(P14)-N(O14)+N(R14)-N(Q14)+N(T14)-N(S14)+N(V14)-N(U14)+N(X14)-N(W14)+N(Z14)-N(Y14)+N(AB14)-N(AA14)+N(AD14)-N(AC14)),2)</f>
         <v/>
       </c>
-      <c r="AF14" s="6" t="n">
+      <c r="AF14" s="7" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1654,64 +1626,64 @@
           <t>Magazziniere</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="6" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="E15" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="F15" s="7" t="n">
+      <c r="F15" s="6" t="n">
         <v>0.75</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="G15" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="H15" s="7" t="n">
+      <c r="H15" s="6" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="I15" s="7" t="n">
+      <c r="I15" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="J15" s="7" t="n">
+      <c r="J15" s="6" t="n">
         <v>0.75</v>
       </c>
-      <c r="K15" s="7" t="n">
+      <c r="K15" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="L15" s="7" t="n">
+      <c r="L15" s="6" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="M15" s="7" t="n">
+      <c r="M15" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="N15" s="7" t="n">
+      <c r="N15" s="6" t="n">
         <v>0.75</v>
       </c>
-      <c r="O15" s="7" t="n">
+      <c r="O15" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="P15" s="7" t="n">
+      <c r="P15" s="6" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="Q15" s="7" t="n">
+      <c r="Q15" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="R15" s="7" t="n">
+      <c r="R15" s="6" t="n">
         <v>0.75</v>
       </c>
-      <c r="S15" s="7" t="n">
+      <c r="S15" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="T15" s="7" t="n">
+      <c r="T15" s="6" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="U15" s="7" t="n">
+      <c r="U15" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="V15" s="7" t="n">
+      <c r="V15" s="6" t="n">
         <v>0.75</v>
       </c>
       <c r="W15" s="5" t="inlineStr">
@@ -1734,7 +1706,7 @@
         <f>ROUND(24*(N(D15)-N(C15)+N(F15)-N(E15)+N(H15)-N(G15)+N(J15)-N(I15)+N(L15)-N(K15)+N(N15)-N(M15)+N(P15)-N(O15)+N(R15)-N(Q15)+N(T15)-N(S15)+N(V15)-N(U15)+N(X15)-N(W15)+N(Z15)-N(Y15)+N(AB15)-N(AA15)+N(AD15)-N(AC15)),2)</f>
         <v/>
       </c>
-      <c r="AF15" s="6" t="n">
+      <c r="AF15" s="7" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1770,29 +1742,28 @@
   <mergeCells count="48">
     <mergeCell ref="W4:X4"/>
     <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="K14:N14"/>
     <mergeCell ref="AA3:AD3"/>
     <mergeCell ref="O11:R11"/>
+    <mergeCell ref="AA12:AD12"/>
     <mergeCell ref="K10:N10"/>
-    <mergeCell ref="O14:R14"/>
     <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C13:F13"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="G9:J9"/>
     <mergeCell ref="C3:F3"/>
-    <mergeCell ref="AA14:AD14"/>
     <mergeCell ref="K3:N3"/>
+    <mergeCell ref="G14:J14"/>
     <mergeCell ref="O3:R3"/>
-    <mergeCell ref="G12:J12"/>
     <mergeCell ref="C6:F6"/>
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="S12:V12"/>
     <mergeCell ref="O6:R6"/>
     <mergeCell ref="O4:P4"/>
-    <mergeCell ref="AA10:AD10"/>
+    <mergeCell ref="W15:Z15"/>
     <mergeCell ref="AA4:AB4"/>
     <mergeCell ref="Q4:R4"/>
-    <mergeCell ref="C14:F14"/>
     <mergeCell ref="AC4:AD4"/>
-    <mergeCell ref="W15:Z15"/>
     <mergeCell ref="AF3:AF5"/>
     <mergeCell ref="O9:R9"/>
     <mergeCell ref="AA13:AD13"/>
@@ -1800,13 +1771,14 @@
     <mergeCell ref="S8:V8"/>
     <mergeCell ref="AE3:AE5"/>
     <mergeCell ref="G7:J7"/>
+    <mergeCell ref="C10:F10"/>
     <mergeCell ref="AA15:AD15"/>
+    <mergeCell ref="S14:V14"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="G13:J13"/>
     <mergeCell ref="I4:J4"/>
     <mergeCell ref="W3:Z3"/>
     <mergeCell ref="G3:J3"/>
-    <mergeCell ref="S13:V13"/>
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="K12:N12"/>
     <mergeCell ref="K8:N8"/>
@@ -1933,51 +1905,51 @@
           <t>lunedì 12 ottobre 2026</t>
         </is>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(9,30,0))*(Orari!$D$6:$D$15&gt;TIME(9,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(9,30,0))*(Orari!$F$6:$F$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(10,30,0))*(Orari!$D$6:$D$15&gt;TIME(10,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(10,30,0))*(Orari!$F$6:$F$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(11,30,0))*(Orari!$D$6:$D$15&gt;TIME(11,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(11,30,0))*(Orari!$F$6:$F$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(12,30,0))*(Orari!$D$6:$D$15&gt;TIME(12,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(12,30,0))*(Orari!$F$6:$F$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(13,30,0))*(Orari!$D$6:$D$15&gt;TIME(13,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(13,30,0))*(Orari!$F$6:$F$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(14,30,0))*(Orari!$D$6:$D$15&gt;TIME(14,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(14,30,0))*(Orari!$F$6:$F$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H5" s="6">
+      <c r="H5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(15,30,0))*(Orari!$D$6:$D$15&gt;TIME(15,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(15,30,0))*(Orari!$F$6:$F$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I5" s="6">
+      <c r="I5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(16,30,0))*(Orari!$D$6:$D$15&gt;TIME(16,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(16,30,0))*(Orari!$F$6:$F$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J5" s="6">
+      <c r="J5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(17,30,0))*(Orari!$D$6:$D$15&gt;TIME(17,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(17,30,0))*(Orari!$F$6:$F$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K5" s="6">
+      <c r="K5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(18,30,0))*(Orari!$D$6:$D$15&gt;TIME(18,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(18,30,0))*(Orari!$F$6:$F$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L5" s="6">
+      <c r="L5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(19,30,0))*(Orari!$D$6:$D$15&gt;TIME(19,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(19,30,0))*(Orari!$F$6:$F$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M5" s="6">
+      <c r="M5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(20,30,0))*(Orari!$D$6:$D$15&gt;TIME(20,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(20,30,0))*(Orari!$F$6:$F$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -1988,51 +1960,51 @@
           <t>martedì 13 ottobre 2026</t>
         </is>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(9,30,0))*(Orari!$H$6:$H$15&gt;TIME(9,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(9,30,0))*(Orari!$J$6:$J$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(10,30,0))*(Orari!$H$6:$H$15&gt;TIME(10,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(10,30,0))*(Orari!$J$6:$J$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(11,30,0))*(Orari!$H$6:$H$15&gt;TIME(11,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(11,30,0))*(Orari!$J$6:$J$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(12,30,0))*(Orari!$H$6:$H$15&gt;TIME(12,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(12,30,0))*(Orari!$J$6:$J$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(13,30,0))*(Orari!$H$6:$H$15&gt;TIME(13,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(13,30,0))*(Orari!$J$6:$J$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G6" s="6">
+      <c r="G6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(14,30,0))*(Orari!$H$6:$H$15&gt;TIME(14,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(14,30,0))*(Orari!$J$6:$J$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(15,30,0))*(Orari!$H$6:$H$15&gt;TIME(15,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(15,30,0))*(Orari!$J$6:$J$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I6" s="6">
+      <c r="I6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(16,30,0))*(Orari!$H$6:$H$15&gt;TIME(16,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(16,30,0))*(Orari!$J$6:$J$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J6" s="6">
+      <c r="J6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(17,30,0))*(Orari!$H$6:$H$15&gt;TIME(17,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(17,30,0))*(Orari!$J$6:$J$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K6" s="6">
+      <c r="K6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(18,30,0))*(Orari!$H$6:$H$15&gt;TIME(18,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(18,30,0))*(Orari!$J$6:$J$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L6" s="6">
+      <c r="L6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(19,30,0))*(Orari!$H$6:$H$15&gt;TIME(19,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(19,30,0))*(Orari!$J$6:$J$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M6" s="6">
+      <c r="M6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(20,30,0))*(Orari!$H$6:$H$15&gt;TIME(20,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(20,30,0))*(Orari!$J$6:$J$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2043,51 +2015,51 @@
           <t>mercoledì 14 ottobre 2026</t>
         </is>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(9,30,0))*(Orari!$L$6:$L$15&gt;TIME(9,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(9,30,0))*(Orari!$N$6:$N$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(10,30,0))*(Orari!$L$6:$L$15&gt;TIME(10,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(10,30,0))*(Orari!$N$6:$N$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(11,30,0))*(Orari!$L$6:$L$15&gt;TIME(11,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(11,30,0))*(Orari!$N$6:$N$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(12,30,0))*(Orari!$L$6:$L$15&gt;TIME(12,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(12,30,0))*(Orari!$N$6:$N$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(13,30,0))*(Orari!$L$6:$L$15&gt;TIME(13,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(13,30,0))*(Orari!$N$6:$N$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(14,30,0))*(Orari!$L$6:$L$15&gt;TIME(14,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(14,30,0))*(Orari!$N$6:$N$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(15,30,0))*(Orari!$L$6:$L$15&gt;TIME(15,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(15,30,0))*(Orari!$N$6:$N$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I7" s="6">
+      <c r="I7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(16,30,0))*(Orari!$L$6:$L$15&gt;TIME(16,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(16,30,0))*(Orari!$N$6:$N$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J7" s="6">
+      <c r="J7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(17,30,0))*(Orari!$L$6:$L$15&gt;TIME(17,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(17,30,0))*(Orari!$N$6:$N$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K7" s="6">
+      <c r="K7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(18,30,0))*(Orari!$L$6:$L$15&gt;TIME(18,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(18,30,0))*(Orari!$N$6:$N$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L7" s="6">
+      <c r="L7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(19,30,0))*(Orari!$L$6:$L$15&gt;TIME(19,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(19,30,0))*(Orari!$N$6:$N$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M7" s="6">
+      <c r="M7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(20,30,0))*(Orari!$L$6:$L$15&gt;TIME(20,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(20,30,0))*(Orari!$N$6:$N$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2098,51 +2070,51 @@
           <t>giovedì 15 ottobre 2026</t>
         </is>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(9,30,0))*(Orari!$P$6:$P$15&gt;TIME(9,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(9,30,0))*(Orari!$R$6:$R$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(10,30,0))*(Orari!$P$6:$P$15&gt;TIME(10,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(10,30,0))*(Orari!$R$6:$R$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(11,30,0))*(Orari!$P$6:$P$15&gt;TIME(11,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(11,30,0))*(Orari!$R$6:$R$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(12,30,0))*(Orari!$P$6:$P$15&gt;TIME(12,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(12,30,0))*(Orari!$R$6:$R$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(13,30,0))*(Orari!$P$6:$P$15&gt;TIME(13,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(13,30,0))*(Orari!$R$6:$R$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(14,30,0))*(Orari!$P$6:$P$15&gt;TIME(14,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(14,30,0))*(Orari!$R$6:$R$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(15,30,0))*(Orari!$P$6:$P$15&gt;TIME(15,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(15,30,0))*(Orari!$R$6:$R$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I8" s="6">
+      <c r="I8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(16,30,0))*(Orari!$P$6:$P$15&gt;TIME(16,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(16,30,0))*(Orari!$R$6:$R$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J8" s="6">
+      <c r="J8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(17,30,0))*(Orari!$P$6:$P$15&gt;TIME(17,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(17,30,0))*(Orari!$R$6:$R$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K8" s="6">
+      <c r="K8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(18,30,0))*(Orari!$P$6:$P$15&gt;TIME(18,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(18,30,0))*(Orari!$R$6:$R$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L8" s="6">
+      <c r="L8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(19,30,0))*(Orari!$P$6:$P$15&gt;TIME(19,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(19,30,0))*(Orari!$R$6:$R$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M8" s="6">
+      <c r="M8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(20,30,0))*(Orari!$P$6:$P$15&gt;TIME(20,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(20,30,0))*(Orari!$R$6:$R$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2153,51 +2125,51 @@
           <t>venerdì 16 ottobre 2026</t>
         </is>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(9,30,0))*(Orari!$T$6:$T$15&gt;TIME(9,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(9,30,0))*(Orari!$V$6:$V$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(10,30,0))*(Orari!$T$6:$T$15&gt;TIME(10,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(10,30,0))*(Orari!$V$6:$V$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(11,30,0))*(Orari!$T$6:$T$15&gt;TIME(11,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(11,30,0))*(Orari!$V$6:$V$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(12,30,0))*(Orari!$T$6:$T$15&gt;TIME(12,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(12,30,0))*(Orari!$V$6:$V$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(13,30,0))*(Orari!$T$6:$T$15&gt;TIME(13,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(13,30,0))*(Orari!$V$6:$V$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G9" s="6">
+      <c r="G9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(14,30,0))*(Orari!$T$6:$T$15&gt;TIME(14,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(14,30,0))*(Orari!$V$6:$V$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H9" s="6">
+      <c r="H9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(15,30,0))*(Orari!$T$6:$T$15&gt;TIME(15,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(15,30,0))*(Orari!$V$6:$V$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I9" s="6">
+      <c r="I9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(16,30,0))*(Orari!$T$6:$T$15&gt;TIME(16,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(16,30,0))*(Orari!$V$6:$V$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J9" s="6">
+      <c r="J9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(17,30,0))*(Orari!$T$6:$T$15&gt;TIME(17,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(17,30,0))*(Orari!$V$6:$V$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K9" s="6">
+      <c r="K9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(18,30,0))*(Orari!$T$6:$T$15&gt;TIME(18,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(18,30,0))*(Orari!$V$6:$V$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L9" s="6">
+      <c r="L9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(19,30,0))*(Orari!$T$6:$T$15&gt;TIME(19,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(19,30,0))*(Orari!$V$6:$V$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M9" s="6">
+      <c r="M9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(20,30,0))*(Orari!$T$6:$T$15&gt;TIME(20,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(20,30,0))*(Orari!$V$6:$V$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2208,51 +2180,51 @@
           <t>sabato 17 ottobre 2026</t>
         </is>
       </c>
-      <c r="B10" s="6">
+      <c r="B10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(9,30,0))*(Orari!$X$6:$X$15&gt;TIME(9,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(9,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(10,30,0))*(Orari!$X$6:$X$15&gt;TIME(10,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(10,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(11,30,0))*(Orari!$X$6:$X$15&gt;TIME(11,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(11,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(12,30,0))*(Orari!$X$6:$X$15&gt;TIME(12,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(12,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(13,30,0))*(Orari!$X$6:$X$15&gt;TIME(13,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(13,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G10" s="6">
+      <c r="G10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(14,30,0))*(Orari!$X$6:$X$15&gt;TIME(14,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(14,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H10" s="6">
+      <c r="H10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(15,30,0))*(Orari!$X$6:$X$15&gt;TIME(15,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(15,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I10" s="6">
+      <c r="I10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(16,30,0))*(Orari!$X$6:$X$15&gt;TIME(16,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(16,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J10" s="6">
+      <c r="J10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(17,30,0))*(Orari!$X$6:$X$15&gt;TIME(17,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(17,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K10" s="6">
+      <c r="K10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(18,30,0))*(Orari!$X$6:$X$15&gt;TIME(18,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(18,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L10" s="6">
+      <c r="L10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(19,30,0))*(Orari!$X$6:$X$15&gt;TIME(19,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(19,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M10" s="6">
+      <c r="M10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(20,30,0))*(Orari!$X$6:$X$15&gt;TIME(20,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(20,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2263,51 +2235,51 @@
           <t>domenica 18 ottobre 2026</t>
         </is>
       </c>
-      <c r="B11" s="6">
+      <c r="B11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(9,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(9,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(9,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(10,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(10,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(10,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(11,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(11,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(11,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(12,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(12,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(12,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(13,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(13,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(13,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G11" s="6">
+      <c r="G11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(14,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(14,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(14,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H11" s="6">
+      <c r="H11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(15,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(15,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(15,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I11" s="6">
+      <c r="I11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(16,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(16,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(16,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J11" s="6">
+      <c r="J11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(17,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(17,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(17,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K11" s="6">
+      <c r="K11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(18,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(18,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(18,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L11" s="6">
+      <c r="L11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(19,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(19,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(19,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M11" s="6">
+      <c r="M11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(20,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(20,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(20,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2392,51 +2364,51 @@
           <t>lunedì 12 ottobre 2026</t>
         </is>
       </c>
-      <c r="B15" s="6">
+      <c r="B15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(9,30,0))*(Orari!$D$6:$D$15&gt;TIME(9,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(9,30,0))*(Orari!$F$6:$F$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C15" s="6">
+      <c r="C15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(10,30,0))*(Orari!$D$6:$D$15&gt;TIME(10,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(10,30,0))*(Orari!$F$6:$F$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(11,30,0))*(Orari!$D$6:$D$15&gt;TIME(11,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(11,30,0))*(Orari!$F$6:$F$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(12,30,0))*(Orari!$D$6:$D$15&gt;TIME(12,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(12,30,0))*(Orari!$F$6:$F$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F15" s="6">
+      <c r="F15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(13,30,0))*(Orari!$D$6:$D$15&gt;TIME(13,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(13,30,0))*(Orari!$F$6:$F$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G15" s="6">
+      <c r="G15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(14,30,0))*(Orari!$D$6:$D$15&gt;TIME(14,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(14,30,0))*(Orari!$F$6:$F$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H15" s="6">
+      <c r="H15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(15,30,0))*(Orari!$D$6:$D$15&gt;TIME(15,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(15,30,0))*(Orari!$F$6:$F$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I15" s="6">
+      <c r="I15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(16,30,0))*(Orari!$D$6:$D$15&gt;TIME(16,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(16,30,0))*(Orari!$F$6:$F$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J15" s="6">
+      <c r="J15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(17,30,0))*(Orari!$D$6:$D$15&gt;TIME(17,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(17,30,0))*(Orari!$F$6:$F$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K15" s="6">
+      <c r="K15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(18,30,0))*(Orari!$D$6:$D$15&gt;TIME(18,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(18,30,0))*(Orari!$F$6:$F$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L15" s="6">
+      <c r="L15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(19,30,0))*(Orari!$D$6:$D$15&gt;TIME(19,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(19,30,0))*(Orari!$F$6:$F$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M15" s="6">
+      <c r="M15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(20,30,0))*(Orari!$D$6:$D$15&gt;TIME(20,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(20,30,0))*(Orari!$F$6:$F$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2447,51 +2419,51 @@
           <t>martedì 13 ottobre 2026</t>
         </is>
       </c>
-      <c r="B16" s="6">
+      <c r="B16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(9,30,0))*(Orari!$H$6:$H$15&gt;TIME(9,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(9,30,0))*(Orari!$J$6:$J$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C16" s="6">
+      <c r="C16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(10,30,0))*(Orari!$H$6:$H$15&gt;TIME(10,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(10,30,0))*(Orari!$J$6:$J$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(11,30,0))*(Orari!$H$6:$H$15&gt;TIME(11,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(11,30,0))*(Orari!$J$6:$J$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E16" s="6">
+      <c r="E16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(12,30,0))*(Orari!$H$6:$H$15&gt;TIME(12,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(12,30,0))*(Orari!$J$6:$J$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F16" s="6">
+      <c r="F16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(13,30,0))*(Orari!$H$6:$H$15&gt;TIME(13,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(13,30,0))*(Orari!$J$6:$J$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G16" s="6">
+      <c r="G16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(14,30,0))*(Orari!$H$6:$H$15&gt;TIME(14,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(14,30,0))*(Orari!$J$6:$J$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H16" s="6">
+      <c r="H16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(15,30,0))*(Orari!$H$6:$H$15&gt;TIME(15,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(15,30,0))*(Orari!$J$6:$J$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I16" s="6">
+      <c r="I16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(16,30,0))*(Orari!$H$6:$H$15&gt;TIME(16,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(16,30,0))*(Orari!$J$6:$J$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J16" s="6">
+      <c r="J16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(17,30,0))*(Orari!$H$6:$H$15&gt;TIME(17,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(17,30,0))*(Orari!$J$6:$J$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K16" s="6">
+      <c r="K16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(18,30,0))*(Orari!$H$6:$H$15&gt;TIME(18,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(18,30,0))*(Orari!$J$6:$J$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L16" s="6">
+      <c r="L16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(19,30,0))*(Orari!$H$6:$H$15&gt;TIME(19,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(19,30,0))*(Orari!$J$6:$J$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M16" s="6">
+      <c r="M16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(20,30,0))*(Orari!$H$6:$H$15&gt;TIME(20,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(20,30,0))*(Orari!$J$6:$J$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2502,51 +2474,51 @@
           <t>mercoledì 14 ottobre 2026</t>
         </is>
       </c>
-      <c r="B17" s="6">
+      <c r="B17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(9,30,0))*(Orari!$L$6:$L$15&gt;TIME(9,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(9,30,0))*(Orari!$N$6:$N$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C17" s="6">
+      <c r="C17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(10,30,0))*(Orari!$L$6:$L$15&gt;TIME(10,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(10,30,0))*(Orari!$N$6:$N$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(11,30,0))*(Orari!$L$6:$L$15&gt;TIME(11,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(11,30,0))*(Orari!$N$6:$N$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(12,30,0))*(Orari!$L$6:$L$15&gt;TIME(12,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(12,30,0))*(Orari!$N$6:$N$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F17" s="6">
+      <c r="F17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(13,30,0))*(Orari!$L$6:$L$15&gt;TIME(13,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(13,30,0))*(Orari!$N$6:$N$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G17" s="6">
+      <c r="G17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(14,30,0))*(Orari!$L$6:$L$15&gt;TIME(14,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(14,30,0))*(Orari!$N$6:$N$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H17" s="6">
+      <c r="H17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(15,30,0))*(Orari!$L$6:$L$15&gt;TIME(15,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(15,30,0))*(Orari!$N$6:$N$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I17" s="6">
+      <c r="I17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(16,30,0))*(Orari!$L$6:$L$15&gt;TIME(16,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(16,30,0))*(Orari!$N$6:$N$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J17" s="6">
+      <c r="J17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(17,30,0))*(Orari!$L$6:$L$15&gt;TIME(17,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(17,30,0))*(Orari!$N$6:$N$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K17" s="6">
+      <c r="K17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(18,30,0))*(Orari!$L$6:$L$15&gt;TIME(18,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(18,30,0))*(Orari!$N$6:$N$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L17" s="6">
+      <c r="L17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(19,30,0))*(Orari!$L$6:$L$15&gt;TIME(19,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(19,30,0))*(Orari!$N$6:$N$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M17" s="6">
+      <c r="M17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(20,30,0))*(Orari!$L$6:$L$15&gt;TIME(20,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(20,30,0))*(Orari!$N$6:$N$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2557,51 +2529,51 @@
           <t>giovedì 15 ottobre 2026</t>
         </is>
       </c>
-      <c r="B18" s="6">
+      <c r="B18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(9,30,0))*(Orari!$P$6:$P$15&gt;TIME(9,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(9,30,0))*(Orari!$R$6:$R$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C18" s="6">
+      <c r="C18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(10,30,0))*(Orari!$P$6:$P$15&gt;TIME(10,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(10,30,0))*(Orari!$R$6:$R$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(11,30,0))*(Orari!$P$6:$P$15&gt;TIME(11,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(11,30,0))*(Orari!$R$6:$R$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(12,30,0))*(Orari!$P$6:$P$15&gt;TIME(12,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(12,30,0))*(Orari!$R$6:$R$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F18" s="6">
+      <c r="F18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(13,30,0))*(Orari!$P$6:$P$15&gt;TIME(13,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(13,30,0))*(Orari!$R$6:$R$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G18" s="6">
+      <c r="G18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(14,30,0))*(Orari!$P$6:$P$15&gt;TIME(14,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(14,30,0))*(Orari!$R$6:$R$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H18" s="6">
+      <c r="H18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(15,30,0))*(Orari!$P$6:$P$15&gt;TIME(15,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(15,30,0))*(Orari!$R$6:$R$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I18" s="6">
+      <c r="I18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(16,30,0))*(Orari!$P$6:$P$15&gt;TIME(16,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(16,30,0))*(Orari!$R$6:$R$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J18" s="6">
+      <c r="J18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(17,30,0))*(Orari!$P$6:$P$15&gt;TIME(17,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(17,30,0))*(Orari!$R$6:$R$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K18" s="6">
+      <c r="K18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(18,30,0))*(Orari!$P$6:$P$15&gt;TIME(18,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(18,30,0))*(Orari!$R$6:$R$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L18" s="6">
+      <c r="L18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(19,30,0))*(Orari!$P$6:$P$15&gt;TIME(19,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(19,30,0))*(Orari!$R$6:$R$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M18" s="6">
+      <c r="M18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(20,30,0))*(Orari!$P$6:$P$15&gt;TIME(20,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(20,30,0))*(Orari!$R$6:$R$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2612,51 +2584,51 @@
           <t>venerdì 16 ottobre 2026</t>
         </is>
       </c>
-      <c r="B19" s="6">
+      <c r="B19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(9,30,0))*(Orari!$T$6:$T$15&gt;TIME(9,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(9,30,0))*(Orari!$V$6:$V$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C19" s="6">
+      <c r="C19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(10,30,0))*(Orari!$T$6:$T$15&gt;TIME(10,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(10,30,0))*(Orari!$V$6:$V$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(11,30,0))*(Orari!$T$6:$T$15&gt;TIME(11,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(11,30,0))*(Orari!$V$6:$V$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E19" s="6">
+      <c r="E19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(12,30,0))*(Orari!$T$6:$T$15&gt;TIME(12,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(12,30,0))*(Orari!$V$6:$V$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F19" s="6">
+      <c r="F19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(13,30,0))*(Orari!$T$6:$T$15&gt;TIME(13,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(13,30,0))*(Orari!$V$6:$V$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G19" s="6">
+      <c r="G19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(14,30,0))*(Orari!$T$6:$T$15&gt;TIME(14,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(14,30,0))*(Orari!$V$6:$V$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H19" s="6">
+      <c r="H19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(15,30,0))*(Orari!$T$6:$T$15&gt;TIME(15,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(15,30,0))*(Orari!$V$6:$V$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I19" s="6">
+      <c r="I19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(16,30,0))*(Orari!$T$6:$T$15&gt;TIME(16,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(16,30,0))*(Orari!$V$6:$V$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J19" s="6">
+      <c r="J19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(17,30,0))*(Orari!$T$6:$T$15&gt;TIME(17,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(17,30,0))*(Orari!$V$6:$V$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K19" s="6">
+      <c r="K19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(18,30,0))*(Orari!$T$6:$T$15&gt;TIME(18,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(18,30,0))*(Orari!$V$6:$V$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L19" s="6">
+      <c r="L19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(19,30,0))*(Orari!$T$6:$T$15&gt;TIME(19,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(19,30,0))*(Orari!$V$6:$V$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M19" s="6">
+      <c r="M19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(20,30,0))*(Orari!$T$6:$T$15&gt;TIME(20,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(20,30,0))*(Orari!$V$6:$V$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2667,51 +2639,51 @@
           <t>sabato 17 ottobre 2026</t>
         </is>
       </c>
-      <c r="B20" s="6">
+      <c r="B20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(9,30,0))*(Orari!$X$6:$X$15&gt;TIME(9,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(9,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C20" s="6">
+      <c r="C20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(10,30,0))*(Orari!$X$6:$X$15&gt;TIME(10,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(10,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D20" s="6">
+      <c r="D20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(11,30,0))*(Orari!$X$6:$X$15&gt;TIME(11,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(11,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E20" s="6">
+      <c r="E20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(12,30,0))*(Orari!$X$6:$X$15&gt;TIME(12,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(12,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F20" s="6">
+      <c r="F20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(13,30,0))*(Orari!$X$6:$X$15&gt;TIME(13,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(13,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G20" s="6">
+      <c r="G20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(14,30,0))*(Orari!$X$6:$X$15&gt;TIME(14,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(14,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H20" s="6">
+      <c r="H20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(15,30,0))*(Orari!$X$6:$X$15&gt;TIME(15,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(15,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I20" s="6">
+      <c r="I20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(16,30,0))*(Orari!$X$6:$X$15&gt;TIME(16,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(16,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J20" s="6">
+      <c r="J20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(17,30,0))*(Orari!$X$6:$X$15&gt;TIME(17,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(17,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K20" s="6">
+      <c r="K20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(18,30,0))*(Orari!$X$6:$X$15&gt;TIME(18,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(18,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L20" s="6">
+      <c r="L20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(19,30,0))*(Orari!$X$6:$X$15&gt;TIME(19,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(19,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M20" s="6">
+      <c r="M20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(20,30,0))*(Orari!$X$6:$X$15&gt;TIME(20,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(20,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2722,51 +2694,51 @@
           <t>domenica 18 ottobre 2026</t>
         </is>
       </c>
-      <c r="B21" s="6">
+      <c r="B21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(9,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(9,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(9,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(10,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(10,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(10,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(11,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(11,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(11,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E21" s="6">
+      <c r="E21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(12,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(12,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(12,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F21" s="6">
+      <c r="F21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(13,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(13,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(13,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G21" s="6">
+      <c r="G21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(14,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(14,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(14,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H21" s="6">
+      <c r="H21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(15,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(15,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(15,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I21" s="6">
+      <c r="I21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(16,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(16,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(16,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J21" s="6">
+      <c r="J21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(17,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(17,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(17,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K21" s="6">
+      <c r="K21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(18,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(18,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(18,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L21" s="6">
+      <c r="L21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(19,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(19,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(19,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M21" s="6">
+      <c r="M21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(20,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(20,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(20,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2851,51 +2823,51 @@
           <t>lunedì 12 ottobre 2026</t>
         </is>
       </c>
-      <c r="B25" s="6">
+      <c r="B25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(9,30,0))*(Orari!$D$6:$D$15&gt;TIME(9,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(9,30,0))*(Orari!$F$6:$F$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C25" s="6">
+      <c r="C25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(10,30,0))*(Orari!$D$6:$D$15&gt;TIME(10,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(10,30,0))*(Orari!$F$6:$F$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D25" s="6">
+      <c r="D25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(11,30,0))*(Orari!$D$6:$D$15&gt;TIME(11,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(11,30,0))*(Orari!$F$6:$F$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E25" s="6">
+      <c r="E25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(12,30,0))*(Orari!$D$6:$D$15&gt;TIME(12,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(12,30,0))*(Orari!$F$6:$F$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F25" s="6">
+      <c r="F25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(13,30,0))*(Orari!$D$6:$D$15&gt;TIME(13,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(13,30,0))*(Orari!$F$6:$F$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G25" s="6">
+      <c r="G25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(14,30,0))*(Orari!$D$6:$D$15&gt;TIME(14,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(14,30,0))*(Orari!$F$6:$F$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H25" s="6">
+      <c r="H25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(15,30,0))*(Orari!$D$6:$D$15&gt;TIME(15,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(15,30,0))*(Orari!$F$6:$F$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I25" s="6">
+      <c r="I25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(16,30,0))*(Orari!$D$6:$D$15&gt;TIME(16,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(16,30,0))*(Orari!$F$6:$F$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J25" s="6">
+      <c r="J25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(17,30,0))*(Orari!$D$6:$D$15&gt;TIME(17,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(17,30,0))*(Orari!$F$6:$F$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K25" s="6">
+      <c r="K25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(18,30,0))*(Orari!$D$6:$D$15&gt;TIME(18,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(18,30,0))*(Orari!$F$6:$F$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L25" s="6">
+      <c r="L25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(19,30,0))*(Orari!$D$6:$D$15&gt;TIME(19,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(19,30,0))*(Orari!$F$6:$F$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M25" s="6">
+      <c r="M25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(20,30,0))*(Orari!$D$6:$D$15&gt;TIME(20,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(20,30,0))*(Orari!$F$6:$F$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2906,51 +2878,51 @@
           <t>martedì 13 ottobre 2026</t>
         </is>
       </c>
-      <c r="B26" s="6">
+      <c r="B26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(9,30,0))*(Orari!$H$6:$H$15&gt;TIME(9,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(9,30,0))*(Orari!$J$6:$J$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C26" s="6">
+      <c r="C26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(10,30,0))*(Orari!$H$6:$H$15&gt;TIME(10,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(10,30,0))*(Orari!$J$6:$J$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D26" s="6">
+      <c r="D26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(11,30,0))*(Orari!$H$6:$H$15&gt;TIME(11,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(11,30,0))*(Orari!$J$6:$J$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E26" s="6">
+      <c r="E26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(12,30,0))*(Orari!$H$6:$H$15&gt;TIME(12,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(12,30,0))*(Orari!$J$6:$J$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F26" s="6">
+      <c r="F26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(13,30,0))*(Orari!$H$6:$H$15&gt;TIME(13,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(13,30,0))*(Orari!$J$6:$J$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G26" s="6">
+      <c r="G26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(14,30,0))*(Orari!$H$6:$H$15&gt;TIME(14,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(14,30,0))*(Orari!$J$6:$J$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H26" s="6">
+      <c r="H26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(15,30,0))*(Orari!$H$6:$H$15&gt;TIME(15,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(15,30,0))*(Orari!$J$6:$J$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I26" s="6">
+      <c r="I26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(16,30,0))*(Orari!$H$6:$H$15&gt;TIME(16,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(16,30,0))*(Orari!$J$6:$J$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J26" s="6">
+      <c r="J26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(17,30,0))*(Orari!$H$6:$H$15&gt;TIME(17,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(17,30,0))*(Orari!$J$6:$J$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K26" s="6">
+      <c r="K26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(18,30,0))*(Orari!$H$6:$H$15&gt;TIME(18,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(18,30,0))*(Orari!$J$6:$J$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L26" s="6">
+      <c r="L26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(19,30,0))*(Orari!$H$6:$H$15&gt;TIME(19,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(19,30,0))*(Orari!$J$6:$J$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M26" s="6">
+      <c r="M26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(20,30,0))*(Orari!$H$6:$H$15&gt;TIME(20,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(20,30,0))*(Orari!$J$6:$J$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2961,51 +2933,51 @@
           <t>mercoledì 14 ottobre 2026</t>
         </is>
       </c>
-      <c r="B27" s="6">
+      <c r="B27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(9,30,0))*(Orari!$L$6:$L$15&gt;TIME(9,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(9,30,0))*(Orari!$N$6:$N$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C27" s="6">
+      <c r="C27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(10,30,0))*(Orari!$L$6:$L$15&gt;TIME(10,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(10,30,0))*(Orari!$N$6:$N$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D27" s="6">
+      <c r="D27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(11,30,0))*(Orari!$L$6:$L$15&gt;TIME(11,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(11,30,0))*(Orari!$N$6:$N$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E27" s="6">
+      <c r="E27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(12,30,0))*(Orari!$L$6:$L$15&gt;TIME(12,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(12,30,0))*(Orari!$N$6:$N$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F27" s="6">
+      <c r="F27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(13,30,0))*(Orari!$L$6:$L$15&gt;TIME(13,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(13,30,0))*(Orari!$N$6:$N$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G27" s="6">
+      <c r="G27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(14,30,0))*(Orari!$L$6:$L$15&gt;TIME(14,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(14,30,0))*(Orari!$N$6:$N$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H27" s="6">
+      <c r="H27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(15,30,0))*(Orari!$L$6:$L$15&gt;TIME(15,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(15,30,0))*(Orari!$N$6:$N$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I27" s="6">
+      <c r="I27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(16,30,0))*(Orari!$L$6:$L$15&gt;TIME(16,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(16,30,0))*(Orari!$N$6:$N$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J27" s="6">
+      <c r="J27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(17,30,0))*(Orari!$L$6:$L$15&gt;TIME(17,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(17,30,0))*(Orari!$N$6:$N$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K27" s="6">
+      <c r="K27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(18,30,0))*(Orari!$L$6:$L$15&gt;TIME(18,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(18,30,0))*(Orari!$N$6:$N$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L27" s="6">
+      <c r="L27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(19,30,0))*(Orari!$L$6:$L$15&gt;TIME(19,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(19,30,0))*(Orari!$N$6:$N$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M27" s="6">
+      <c r="M27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(20,30,0))*(Orari!$L$6:$L$15&gt;TIME(20,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(20,30,0))*(Orari!$N$6:$N$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -3016,51 +2988,51 @@
           <t>giovedì 15 ottobre 2026</t>
         </is>
       </c>
-      <c r="B28" s="6">
+      <c r="B28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(9,30,0))*(Orari!$P$6:$P$15&gt;TIME(9,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(9,30,0))*(Orari!$R$6:$R$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C28" s="6">
+      <c r="C28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(10,30,0))*(Orari!$P$6:$P$15&gt;TIME(10,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(10,30,0))*(Orari!$R$6:$R$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D28" s="6">
+      <c r="D28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(11,30,0))*(Orari!$P$6:$P$15&gt;TIME(11,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(11,30,0))*(Orari!$R$6:$R$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E28" s="6">
+      <c r="E28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(12,30,0))*(Orari!$P$6:$P$15&gt;TIME(12,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(12,30,0))*(Orari!$R$6:$R$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F28" s="6">
+      <c r="F28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(13,30,0))*(Orari!$P$6:$P$15&gt;TIME(13,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(13,30,0))*(Orari!$R$6:$R$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G28" s="6">
+      <c r="G28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(14,30,0))*(Orari!$P$6:$P$15&gt;TIME(14,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(14,30,0))*(Orari!$R$6:$R$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H28" s="6">
+      <c r="H28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(15,30,0))*(Orari!$P$6:$P$15&gt;TIME(15,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(15,30,0))*(Orari!$R$6:$R$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I28" s="6">
+      <c r="I28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(16,30,0))*(Orari!$P$6:$P$15&gt;TIME(16,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(16,30,0))*(Orari!$R$6:$R$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J28" s="6">
+      <c r="J28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(17,30,0))*(Orari!$P$6:$P$15&gt;TIME(17,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(17,30,0))*(Orari!$R$6:$R$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K28" s="6">
+      <c r="K28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(18,30,0))*(Orari!$P$6:$P$15&gt;TIME(18,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(18,30,0))*(Orari!$R$6:$R$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L28" s="6">
+      <c r="L28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(19,30,0))*(Orari!$P$6:$P$15&gt;TIME(19,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(19,30,0))*(Orari!$R$6:$R$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M28" s="6">
+      <c r="M28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(20,30,0))*(Orari!$P$6:$P$15&gt;TIME(20,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(20,30,0))*(Orari!$R$6:$R$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -3071,51 +3043,51 @@
           <t>venerdì 16 ottobre 2026</t>
         </is>
       </c>
-      <c r="B29" s="6">
+      <c r="B29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(9,30,0))*(Orari!$T$6:$T$15&gt;TIME(9,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(9,30,0))*(Orari!$V$6:$V$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C29" s="6">
+      <c r="C29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(10,30,0))*(Orari!$T$6:$T$15&gt;TIME(10,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(10,30,0))*(Orari!$V$6:$V$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D29" s="6">
+      <c r="D29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(11,30,0))*(Orari!$T$6:$T$15&gt;TIME(11,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(11,30,0))*(Orari!$V$6:$V$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E29" s="6">
+      <c r="E29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(12,30,0))*(Orari!$T$6:$T$15&gt;TIME(12,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(12,30,0))*(Orari!$V$6:$V$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F29" s="6">
+      <c r="F29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(13,30,0))*(Orari!$T$6:$T$15&gt;TIME(13,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(13,30,0))*(Orari!$V$6:$V$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G29" s="6">
+      <c r="G29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(14,30,0))*(Orari!$T$6:$T$15&gt;TIME(14,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(14,30,0))*(Orari!$V$6:$V$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H29" s="6">
+      <c r="H29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(15,30,0))*(Orari!$T$6:$T$15&gt;TIME(15,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(15,30,0))*(Orari!$V$6:$V$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I29" s="6">
+      <c r="I29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(16,30,0))*(Orari!$T$6:$T$15&gt;TIME(16,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(16,30,0))*(Orari!$V$6:$V$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J29" s="6">
+      <c r="J29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(17,30,0))*(Orari!$T$6:$T$15&gt;TIME(17,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(17,30,0))*(Orari!$V$6:$V$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K29" s="6">
+      <c r="K29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(18,30,0))*(Orari!$T$6:$T$15&gt;TIME(18,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(18,30,0))*(Orari!$V$6:$V$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L29" s="6">
+      <c r="L29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(19,30,0))*(Orari!$T$6:$T$15&gt;TIME(19,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(19,30,0))*(Orari!$V$6:$V$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M29" s="6">
+      <c r="M29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(20,30,0))*(Orari!$T$6:$T$15&gt;TIME(20,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(20,30,0))*(Orari!$V$6:$V$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -3126,51 +3098,51 @@
           <t>sabato 17 ottobre 2026</t>
         </is>
       </c>
-      <c r="B30" s="6">
+      <c r="B30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(9,30,0))*(Orari!$X$6:$X$15&gt;TIME(9,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(9,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C30" s="6">
+      <c r="C30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(10,30,0))*(Orari!$X$6:$X$15&gt;TIME(10,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(10,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D30" s="6">
+      <c r="D30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(11,30,0))*(Orari!$X$6:$X$15&gt;TIME(11,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(11,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E30" s="6">
+      <c r="E30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(12,30,0))*(Orari!$X$6:$X$15&gt;TIME(12,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(12,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F30" s="6">
+      <c r="F30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(13,30,0))*(Orari!$X$6:$X$15&gt;TIME(13,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(13,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G30" s="6">
+      <c r="G30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(14,30,0))*(Orari!$X$6:$X$15&gt;TIME(14,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(14,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H30" s="6">
+      <c r="H30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(15,30,0))*(Orari!$X$6:$X$15&gt;TIME(15,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(15,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I30" s="6">
+      <c r="I30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(16,30,0))*(Orari!$X$6:$X$15&gt;TIME(16,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(16,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J30" s="6">
+      <c r="J30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(17,30,0))*(Orari!$X$6:$X$15&gt;TIME(17,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(17,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K30" s="6">
+      <c r="K30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(18,30,0))*(Orari!$X$6:$X$15&gt;TIME(18,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(18,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L30" s="6">
+      <c r="L30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(19,30,0))*(Orari!$X$6:$X$15&gt;TIME(19,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(19,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M30" s="6">
+      <c r="M30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(20,30,0))*(Orari!$X$6:$X$15&gt;TIME(20,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(20,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -3181,51 +3153,51 @@
           <t>domenica 18 ottobre 2026</t>
         </is>
       </c>
-      <c r="B31" s="6">
+      <c r="B31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(9,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(9,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(9,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C31" s="6">
+      <c r="C31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(10,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(10,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(10,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D31" s="6">
+      <c r="D31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(11,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(11,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(11,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E31" s="6">
+      <c r="E31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(12,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(12,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(12,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F31" s="6">
+      <c r="F31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(13,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(13,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(13,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G31" s="6">
+      <c r="G31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(14,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(14,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(14,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H31" s="6">
+      <c r="H31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(15,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(15,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(15,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I31" s="6">
+      <c r="I31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(16,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(16,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(16,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J31" s="6">
+      <c r="J31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(17,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(17,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(17,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K31" s="6">
+      <c r="K31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(18,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(18,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(18,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L31" s="6">
+      <c r="L31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(19,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(19,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(19,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M31" s="6">
+      <c r="M31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(20,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(20,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(20,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Orari: sabato giornata intera per tutti, terzo addetto di reparto preferibilmente al pomeriggio
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RgW8tUpL59m5j1P2CKTdxn
</commit_message>
<xml_diff>
--- a/orari/Orari_12-18_ottobre_2026.xlsx
+++ b/orari/Orari_12-18_ottobre_2026.xlsx
@@ -104,13 +104,13 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -877,75 +877,71 @@
           <t>Addetto vendite</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="5" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="6" t="n">
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="7" t="n"/>
+      <c r="J6" s="7" t="n"/>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="6" t="n"/>
+      <c r="M6" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="N6" s="5" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="O6" s="5" t="n">
         <v>0.4166666666666667</v>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="P6" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="I6" s="6" t="n">
+      <c r="Q6" s="6" t="n"/>
+      <c r="R6" s="6" t="n"/>
+      <c r="S6" s="6" t="n"/>
+      <c r="T6" s="6" t="n"/>
+      <c r="U6" s="5" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="V6" s="5" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="W6" s="5" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="X6" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="Y6" s="5" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="J6" s="6" t="n">
+      <c r="Z6" s="5" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="K6" s="7" t="n"/>
-      <c r="L6" s="7" t="n"/>
-      <c r="M6" s="6" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="N6" s="6" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="O6" s="5" t="inlineStr">
+      <c r="AA6" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="P6" s="5" t="n"/>
-      <c r="Q6" s="5" t="n"/>
-      <c r="R6" s="5" t="n"/>
-      <c r="S6" s="6" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="T6" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="U6" s="6" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="V6" s="6" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="W6" s="7" t="n"/>
-      <c r="X6" s="7" t="n"/>
-      <c r="Y6" s="6" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="Z6" s="6" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="AA6" s="6" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="AB6" s="6" t="n">
-        <v>0.5833333333333334</v>
-      </c>
+      <c r="AB6" s="7" t="n"/>
       <c r="AC6" s="7" t="n"/>
       <c r="AD6" s="7" t="n"/>
       <c r="AE6" s="8">
         <f>ROUND(24*(N(D6)-N(C6)+N(F6)-N(E6)+N(H6)-N(G6)+N(J6)-N(I6)+N(L6)-N(K6)+N(N6)-N(M6)+N(P6)-N(O6)+N(R6)-N(Q6)+N(T6)-N(S6)+N(V6)-N(U6)+N(X6)-N(W6)+N(Z6)-N(Y6)+N(AB6)-N(AA6)+N(AD6)-N(AC6)),2)</f>
         <v/>
       </c>
-      <c r="AF6" s="7" t="n">
+      <c r="AF6" s="6" t="n">
         <v>30</v>
       </c>
     </row>
@@ -960,83 +956,83 @@
           <t>Vicedirettore</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="7" t="n"/>
+      <c r="J7" s="7" t="n"/>
+      <c r="K7" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="O7" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="P7" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="Q7" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="R7" s="5" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="S7" s="5" t="n">
         <v>0.4166666666666667</v>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="T7" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="U7" s="5" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="V7" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="W7" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="X7" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="E7" s="6" t="n">
+      <c r="Y7" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="F7" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="Z7" s="5" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="AA7" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="M7" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="N7" s="6" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="O7" s="6" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="Q7" s="6" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="R7" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="S7" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="T7" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="U7" s="7" t="n"/>
-      <c r="V7" s="7" t="n"/>
-      <c r="W7" s="6" t="n">
-        <v>0.4583333333333333</v>
-      </c>
-      <c r="X7" s="6" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="Y7" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="Z7" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="AA7" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="AB7" s="5" t="n"/>
-      <c r="AC7" s="5" t="n"/>
-      <c r="AD7" s="5" t="n"/>
+      <c r="AB7" s="7" t="n"/>
+      <c r="AC7" s="7" t="n"/>
+      <c r="AD7" s="7" t="n"/>
       <c r="AE7" s="8">
         <f>ROUND(24*(N(D7)-N(C7)+N(F7)-N(E7)+N(H7)-N(G7)+N(J7)-N(I7)+N(L7)-N(K7)+N(N7)-N(M7)+N(P7)-N(O7)+N(R7)-N(Q7)+N(T7)-N(S7)+N(V7)-N(U7)+N(X7)-N(W7)+N(Z7)-N(Y7)+N(AB7)-N(AA7)+N(AD7)-N(AC7)),2)</f>
         <v/>
       </c>
-      <c r="AF7" s="7" t="inlineStr">
+      <c r="AF7" s="6" t="inlineStr">
         <is>
           <t>44-45</t>
         </is>
@@ -1053,79 +1049,79 @@
           <t>Addetto vendite</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G8" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="H8" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="H8" s="6" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="I8" s="6" t="n">
+      <c r="I8" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="L8" s="7" t="n"/>
+      <c r="M8" s="7" t="n"/>
+      <c r="N8" s="7" t="n"/>
+      <c r="O8" s="6" t="n"/>
+      <c r="P8" s="6" t="n"/>
+      <c r="Q8" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="J8" s="6" t="n">
-        <v>0.7916666666666666</v>
-      </c>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="R8" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="S8" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="L8" s="5" t="n"/>
-      <c r="M8" s="5" t="n"/>
-      <c r="N8" s="5" t="n"/>
-      <c r="O8" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="P8" s="6" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Q8" s="6" t="n">
-        <v>0.5416666666666666</v>
-      </c>
-      <c r="R8" s="6" t="n">
-        <v>0.7916666666666666</v>
-      </c>
-      <c r="S8" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="T8" s="5" t="n"/>
-      <c r="U8" s="5" t="n"/>
-      <c r="V8" s="5" t="n"/>
-      <c r="W8" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="X8" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="Y8" s="7" t="n"/>
-      <c r="Z8" s="7" t="n"/>
-      <c r="AA8" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="AB8" s="6" t="n">
-        <v>0.5416666666666666</v>
-      </c>
-      <c r="AC8" s="6" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="AD8" s="6" t="n">
-        <v>0.8333333333333334</v>
+      <c r="T8" s="7" t="n"/>
+      <c r="U8" s="7" t="n"/>
+      <c r="V8" s="7" t="n"/>
+      <c r="W8" s="5" t="n">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="X8" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="Y8" s="5" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="Z8" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="AA8" s="5" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="AB8" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="AC8" s="5" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="AD8" s="5" t="n">
+        <v>0.875</v>
       </c>
       <c r="AE8" s="8">
         <f>ROUND(24*(N(D8)-N(C8)+N(F8)-N(E8)+N(H8)-N(G8)+N(J8)-N(I8)+N(L8)-N(K8)+N(N8)-N(M8)+N(P8)-N(O8)+N(R8)-N(Q8)+N(T8)-N(S8)+N(V8)-N(U8)+N(X8)-N(W8)+N(Z8)-N(Y8)+N(AB8)-N(AA8)+N(AD8)-N(AC8)),2)</f>
         <v/>
       </c>
-      <c r="AF8" s="7" t="n">
+      <c r="AF8" s="6" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1140,79 +1136,79 @@
           <t>Addetto vendite</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="n"/>
+      <c r="M9" s="7" t="n"/>
+      <c r="N9" s="7" t="n"/>
+      <c r="O9" s="6" t="n"/>
+      <c r="P9" s="6" t="n"/>
+      <c r="Q9" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="R9" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="S9" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="T9" s="7" t="n"/>
+      <c r="U9" s="7" t="n"/>
+      <c r="V9" s="7" t="n"/>
+      <c r="W9" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="D9" s="6" t="n">
-        <v>0.5416666666666666</v>
-      </c>
-      <c r="E9" s="6" t="n">
+      <c r="X9" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="F9" s="6" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="6" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="L9" s="6" t="n">
+      <c r="Y9" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="Z9" s="5" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="AA9" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="AB9" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="AC9" s="5" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="M9" s="6" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="N9" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="O9" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="P9" s="5" t="n"/>
-      <c r="Q9" s="5" t="n"/>
-      <c r="R9" s="5" t="n"/>
-      <c r="S9" s="7" t="n"/>
-      <c r="T9" s="7" t="n"/>
-      <c r="U9" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="V9" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="W9" s="7" t="n"/>
-      <c r="X9" s="7" t="n"/>
-      <c r="Y9" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="Z9" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="AA9" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="AB9" s="6" t="n">
-        <v>0.5416666666666666</v>
-      </c>
-      <c r="AC9" s="6" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="AD9" s="6" t="n">
-        <v>0.8333333333333334</v>
+      <c r="AD9" s="5" t="n">
+        <v>0.7916666666666666</v>
       </c>
       <c r="AE9" s="8">
         <f>ROUND(24*(N(D9)-N(C9)+N(F9)-N(E9)+N(H9)-N(G9)+N(J9)-N(I9)+N(L9)-N(K9)+N(N9)-N(M9)+N(P9)-N(O9)+N(R9)-N(Q9)+N(T9)-N(S9)+N(V9)-N(U9)+N(X9)-N(W9)+N(Z9)-N(Y9)+N(AB9)-N(AA9)+N(AD9)-N(AC9)),2)</f>
         <v/>
       </c>
-      <c r="AF9" s="7" t="n">
+      <c r="AF9" s="6" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1227,79 +1223,79 @@
           <t>Addetto vendite</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="6" t="n">
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="K10" s="5" t="n">
         <v>0.4166666666666667</v>
       </c>
-      <c r="H10" s="6" t="n">
+      <c r="L10" s="5" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="I10" s="6" t="n">
+      <c r="M10" s="5" t="n">
         <v>0.7083333333333334</v>
       </c>
-      <c r="J10" s="6" t="n">
+      <c r="N10" s="5" t="n">
         <v>0.875</v>
       </c>
-      <c r="K10" s="5" t="inlineStr">
+      <c r="O10" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="L10" s="5" t="n"/>
-      <c r="M10" s="5" t="n"/>
-      <c r="N10" s="5" t="n"/>
-      <c r="O10" s="6" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="P10" s="6" t="n">
+      <c r="P10" s="7" t="n"/>
+      <c r="Q10" s="7" t="n"/>
+      <c r="R10" s="7" t="n"/>
+      <c r="S10" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="T10" s="5" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="U10" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="Q10" s="6" t="n">
+      <c r="V10" s="5" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="W10" s="5" t="n">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="X10" s="5" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="R10" s="6" t="n">
+      <c r="Y10" s="5" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="Z10" s="5" t="n">
         <v>0.875</v>
       </c>
-      <c r="S10" s="7" t="n"/>
-      <c r="T10" s="7" t="n"/>
-      <c r="U10" s="6" t="n">
+      <c r="AA10" s="6" t="n"/>
+      <c r="AB10" s="6" t="n"/>
+      <c r="AC10" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="V10" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="W10" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="X10" s="6" t="n">
-        <v>0.5416666666666666</v>
-      </c>
-      <c r="Y10" s="7" t="n"/>
-      <c r="Z10" s="7" t="n"/>
-      <c r="AA10" s="6" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="AB10" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="AC10" s="6" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="AD10" s="6" t="n">
+      <c r="AD10" s="5" t="n">
         <v>0.875</v>
       </c>
       <c r="AE10" s="8">
         <f>ROUND(24*(N(D10)-N(C10)+N(F10)-N(E10)+N(H10)-N(G10)+N(J10)-N(I10)+N(L10)-N(K10)+N(N10)-N(M10)+N(P10)-N(O10)+N(R10)-N(Q10)+N(T10)-N(S10)+N(V10)-N(U10)+N(X10)-N(W10)+N(Z10)-N(Y10)+N(AB10)-N(AA10)+N(AD10)-N(AC10)),2)</f>
         <v/>
       </c>
-      <c r="AF10" s="7" t="n">
+      <c r="AF10" s="6" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1314,79 +1310,79 @@
           <t>Cassiera</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="6" t="n">
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="5" t="n">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="K11" s="5" t="n">
         <v>0.4166666666666667</v>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="L11" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="I11" s="6" t="n">
+      <c r="M11" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="J11" s="6" t="n">
+      <c r="N11" s="5" t="n">
         <v>0.875</v>
       </c>
-      <c r="K11" s="6" t="n">
+      <c r="O11" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="P11" s="7" t="n"/>
+      <c r="Q11" s="7" t="n"/>
+      <c r="R11" s="7" t="n"/>
+      <c r="S11" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="T11" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="U11" s="6" t="n"/>
+      <c r="V11" s="6" t="n"/>
+      <c r="W11" s="5" t="n">
         <v>0.4583333333333333</v>
       </c>
-      <c r="L11" s="6" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="M11" s="6" t="n">
+      <c r="X11" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="N11" s="6" t="n">
+      <c r="Y11" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="Z11" s="5" t="n">
         <v>0.875</v>
       </c>
-      <c r="O11" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="P11" s="5" t="n"/>
-      <c r="Q11" s="5" t="n"/>
-      <c r="R11" s="5" t="n"/>
-      <c r="S11" s="6" t="n">
-        <v>0.4583333333333333</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="U11" s="6" t="n">
+      <c r="AA11" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="AB11" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="V11" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="W11" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="X11" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="Y11" s="7" t="n"/>
-      <c r="Z11" s="7" t="n"/>
-      <c r="AA11" s="7" t="n"/>
-      <c r="AB11" s="7" t="n"/>
-      <c r="AC11" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="AD11" s="6" t="n">
-        <v>0.875</v>
-      </c>
+      <c r="AC11" s="6" t="n"/>
+      <c r="AD11" s="6" t="n"/>
       <c r="AE11" s="8">
         <f>ROUND(24*(N(D11)-N(C11)+N(F11)-N(E11)+N(H11)-N(G11)+N(J11)-N(I11)+N(L11)-N(K11)+N(N11)-N(M11)+N(P11)-N(O11)+N(R11)-N(Q11)+N(T11)-N(S11)+N(V11)-N(U11)+N(X11)-N(W11)+N(Z11)-N(Y11)+N(AB11)-N(AA11)+N(AD11)-N(AC11)),2)</f>
         <v/>
       </c>
-      <c r="AF11" s="7" t="n">
+      <c r="AF11" s="6" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1401,67 +1397,71 @@
           <t>Cassiera</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="D12" s="6" t="n">
-        <v>0.625</v>
-      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="n"/>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="7" t="n"/>
-      <c r="G12" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="H12" s="6" t="n">
-        <v>0.625</v>
-      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="n"/>
       <c r="I12" s="7" t="n"/>
       <c r="J12" s="7" t="n"/>
-      <c r="K12" s="5" t="inlineStr">
+      <c r="K12" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="L12" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="M12" s="6" t="n"/>
+      <c r="N12" s="6" t="n"/>
+      <c r="O12" s="6" t="n"/>
+      <c r="P12" s="6" t="n"/>
+      <c r="Q12" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="R12" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="S12" s="6" t="n"/>
+      <c r="T12" s="6" t="n"/>
+      <c r="U12" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="V12" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="W12" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="X12" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="Y12" s="5" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="Z12" s="5" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="AA12" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="L12" s="5" t="n"/>
-      <c r="M12" s="5" t="n"/>
-      <c r="N12" s="5" t="n"/>
-      <c r="O12" s="7" t="n"/>
-      <c r="P12" s="7" t="n"/>
-      <c r="Q12" s="6" t="n">
-        <v>0.5416666666666666</v>
-      </c>
-      <c r="R12" s="6" t="n">
-        <v>0.7916666666666666</v>
-      </c>
-      <c r="S12" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="T12" s="5" t="n"/>
-      <c r="U12" s="5" t="n"/>
-      <c r="V12" s="5" t="n"/>
-      <c r="W12" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="X12" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="Y12" s="7" t="n"/>
-      <c r="Z12" s="7" t="n"/>
-      <c r="AA12" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="AB12" s="5" t="n"/>
-      <c r="AC12" s="5" t="n"/>
-      <c r="AD12" s="5" t="n"/>
+      <c r="AB12" s="7" t="n"/>
+      <c r="AC12" s="7" t="n"/>
+      <c r="AD12" s="7" t="n"/>
       <c r="AE12" s="8">
         <f>ROUND(24*(N(D12)-N(C12)+N(F12)-N(E12)+N(H12)-N(G12)+N(J12)-N(I12)+N(L12)-N(K12)+N(N12)-N(M12)+N(P12)-N(O12)+N(R12)-N(Q12)+N(T12)-N(S12)+N(V12)-N(U12)+N(X12)-N(W12)+N(Z12)-N(Y12)+N(AB12)-N(AA12)+N(AD12)-N(AC12)),2)</f>
         <v/>
       </c>
-      <c r="AF12" s="7" t="n">
+      <c r="AF12" s="6" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1476,67 +1476,71 @@
           <t>Cassiera</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="n"/>
+      <c r="K13" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="n"/>
-      <c r="K13" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="L13" s="6" t="n">
-        <v>0.625</v>
-      </c>
+      <c r="L13" s="7" t="n"/>
       <c r="M13" s="7" t="n"/>
       <c r="N13" s="7" t="n"/>
-      <c r="O13" s="7" t="n"/>
-      <c r="P13" s="7" t="n"/>
-      <c r="Q13" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="R13" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="S13" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="T13" s="6" t="n">
-        <v>0.625</v>
-      </c>
+      <c r="O13" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P13" s="5" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="Q13" s="6" t="n"/>
+      <c r="R13" s="6" t="n"/>
+      <c r="S13" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="T13" s="7" t="n"/>
       <c r="U13" s="7" t="n"/>
       <c r="V13" s="7" t="n"/>
-      <c r="W13" s="7" t="n"/>
-      <c r="X13" s="7" t="n"/>
-      <c r="Y13" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="Z13" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="AA13" s="5" t="inlineStr">
+      <c r="W13" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="X13" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Y13" s="5" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="Z13" s="5" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="AA13" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="AB13" s="5" t="n"/>
-      <c r="AC13" s="5" t="n"/>
-      <c r="AD13" s="5" t="n"/>
+      <c r="AB13" s="7" t="n"/>
+      <c r="AC13" s="7" t="n"/>
+      <c r="AD13" s="7" t="n"/>
       <c r="AE13" s="8">
         <f>ROUND(24*(N(D13)-N(C13)+N(F13)-N(E13)+N(H13)-N(G13)+N(J13)-N(I13)+N(L13)-N(K13)+N(N13)-N(M13)+N(P13)-N(O13)+N(R13)-N(Q13)+N(T13)-N(S13)+N(V13)-N(U13)+N(X13)-N(W13)+N(Z13)-N(Y13)+N(AB13)-N(AA13)+N(AD13)-N(AC13)),2)</f>
         <v/>
       </c>
-      <c r="AF13" s="7" t="n">
+      <c r="AF13" s="6" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1551,67 +1555,71 @@
           <t>Cassiera</t>
         </is>
       </c>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="6" t="n">
+      <c r="C14" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="D14" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="F14" s="6" t="n">
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="n"/>
+      <c r="I14" s="7" t="n"/>
+      <c r="J14" s="7" t="n"/>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="L14" s="7" t="n"/>
+      <c r="M14" s="7" t="n"/>
+      <c r="N14" s="7" t="n"/>
+      <c r="O14" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="P14" s="5" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="Q14" s="6" t="n"/>
+      <c r="R14" s="6" t="n"/>
+      <c r="S14" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="T14" s="7" t="n"/>
+      <c r="U14" s="7" t="n"/>
+      <c r="V14" s="7" t="n"/>
+      <c r="W14" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="X14" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Y14" s="5" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="Z14" s="5" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="AA14" s="6" t="n"/>
+      <c r="AB14" s="6" t="n"/>
+      <c r="AC14" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="AD14" s="5" t="n">
         <v>0.875</v>
       </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="5" t="n"/>
-      <c r="J14" s="5" t="n"/>
-      <c r="K14" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="L14" s="5" t="n"/>
-      <c r="M14" s="5" t="n"/>
-      <c r="N14" s="5" t="n"/>
-      <c r="O14" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="P14" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="Q14" s="7" t="n"/>
-      <c r="R14" s="7" t="n"/>
-      <c r="S14" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="T14" s="5" t="n"/>
-      <c r="U14" s="5" t="n"/>
-      <c r="V14" s="5" t="n"/>
-      <c r="W14" s="7" t="n"/>
-      <c r="X14" s="7" t="n"/>
-      <c r="Y14" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="Z14" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="AA14" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="AB14" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="AC14" s="7" t="n"/>
-      <c r="AD14" s="7" t="n"/>
       <c r="AE14" s="8">
         <f>ROUND(24*(N(D14)-N(C14)+N(F14)-N(E14)+N(H14)-N(G14)+N(J14)-N(I14)+N(L14)-N(K14)+N(N14)-N(M14)+N(P14)-N(O14)+N(R14)-N(Q14)+N(T14)-N(S14)+N(V14)-N(U14)+N(X14)-N(W14)+N(Z14)-N(Y14)+N(AB14)-N(AA14)+N(AD14)-N(AC14)),2)</f>
         <v/>
       </c>
-      <c r="AF14" s="7" t="n">
+      <c r="AF14" s="6" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1626,87 +1634,87 @@
           <t>Magazziniere</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="C15" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="D15" s="6" t="n">
+      <c r="D15" s="5" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="E15" s="6" t="n">
+      <c r="E15" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="F15" s="6" t="n">
+      <c r="F15" s="5" t="n">
         <v>0.75</v>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="G15" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="H15" s="6" t="n">
+      <c r="H15" s="5" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="I15" s="6" t="n">
+      <c r="I15" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="J15" s="6" t="n">
+      <c r="J15" s="5" t="n">
         <v>0.75</v>
       </c>
-      <c r="K15" s="6" t="n">
+      <c r="K15" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="L15" s="6" t="n">
+      <c r="L15" s="5" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="M15" s="6" t="n">
+      <c r="M15" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="N15" s="6" t="n">
+      <c r="N15" s="5" t="n">
         <v>0.75</v>
       </c>
-      <c r="O15" s="6" t="n">
+      <c r="O15" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="P15" s="6" t="n">
+      <c r="P15" s="5" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="Q15" s="6" t="n">
+      <c r="Q15" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="R15" s="6" t="n">
+      <c r="R15" s="5" t="n">
         <v>0.75</v>
       </c>
-      <c r="S15" s="6" t="n">
+      <c r="S15" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="T15" s="6" t="n">
+      <c r="T15" s="5" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="U15" s="6" t="n">
+      <c r="U15" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="V15" s="6" t="n">
+      <c r="V15" s="5" t="n">
         <v>0.75</v>
       </c>
-      <c r="W15" s="5" t="inlineStr">
+      <c r="W15" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="X15" s="5" t="n"/>
-      <c r="Y15" s="5" t="n"/>
-      <c r="Z15" s="5" t="n"/>
-      <c r="AA15" s="5" t="inlineStr">
+      <c r="X15" s="7" t="n"/>
+      <c r="Y15" s="7" t="n"/>
+      <c r="Z15" s="7" t="n"/>
+      <c r="AA15" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="AB15" s="5" t="n"/>
-      <c r="AC15" s="5" t="n"/>
-      <c r="AD15" s="5" t="n"/>
+      <c r="AB15" s="7" t="n"/>
+      <c r="AC15" s="7" t="n"/>
+      <c r="AD15" s="7" t="n"/>
       <c r="AE15" s="8">
         <f>ROUND(24*(N(D15)-N(C15)+N(F15)-N(E15)+N(H15)-N(G15)+N(J15)-N(I15)+N(L15)-N(K15)+N(N15)-N(M15)+N(P15)-N(O15)+N(R15)-N(Q15)+N(T15)-N(S15)+N(V15)-N(U15)+N(X15)-N(W15)+N(Z15)-N(Y15)+N(AB15)-N(AA15)+N(AD15)-N(AC15)),2)</f>
         <v/>
       </c>
-      <c r="AF15" s="7" t="n">
+      <c r="AF15" s="6" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1741,46 +1749,46 @@
   </sheetData>
   <mergeCells count="48">
     <mergeCell ref="W4:X4"/>
+    <mergeCell ref="S9:V9"/>
     <mergeCell ref="Y4:Z4"/>
     <mergeCell ref="K14:N14"/>
     <mergeCell ref="AA3:AD3"/>
     <mergeCell ref="O11:R11"/>
     <mergeCell ref="AA12:AD12"/>
-    <mergeCell ref="K10:N10"/>
     <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C13:F13"/>
     <mergeCell ref="E4:F4"/>
-    <mergeCell ref="G9:J9"/>
+    <mergeCell ref="K13:N13"/>
     <mergeCell ref="C3:F3"/>
     <mergeCell ref="K3:N3"/>
     <mergeCell ref="G14:J14"/>
     <mergeCell ref="O3:R3"/>
-    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="G12:J12"/>
     <mergeCell ref="B3:B5"/>
-    <mergeCell ref="S12:V12"/>
-    <mergeCell ref="O6:R6"/>
+    <mergeCell ref="O10:R10"/>
     <mergeCell ref="O4:P4"/>
-    <mergeCell ref="W15:Z15"/>
+    <mergeCell ref="K9:N9"/>
     <mergeCell ref="AA4:AB4"/>
     <mergeCell ref="Q4:R4"/>
+    <mergeCell ref="W15:Z15"/>
     <mergeCell ref="AC4:AD4"/>
     <mergeCell ref="AF3:AF5"/>
-    <mergeCell ref="O9:R9"/>
     <mergeCell ref="AA13:AD13"/>
     <mergeCell ref="S3:V3"/>
     <mergeCell ref="S8:V8"/>
     <mergeCell ref="AE3:AE5"/>
     <mergeCell ref="G7:J7"/>
+    <mergeCell ref="AA6:AD6"/>
     <mergeCell ref="C10:F10"/>
     <mergeCell ref="AA15:AD15"/>
     <mergeCell ref="S14:V14"/>
     <mergeCell ref="G4:H4"/>
-    <mergeCell ref="G13:J13"/>
+    <mergeCell ref="G6:J6"/>
     <mergeCell ref="I4:J4"/>
     <mergeCell ref="W3:Z3"/>
     <mergeCell ref="G3:J3"/>
+    <mergeCell ref="S13:V13"/>
+    <mergeCell ref="C12:F12"/>
     <mergeCell ref="A3:A5"/>
-    <mergeCell ref="K12:N12"/>
     <mergeCell ref="K8:N8"/>
     <mergeCell ref="C11:F11"/>
     <mergeCell ref="K4:L4"/>
@@ -1905,51 +1913,51 @@
           <t>lunedì 12 ottobre 2026</t>
         </is>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(9,30,0))*(Orari!$D$6:$D$15&gt;TIME(9,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(9,30,0))*(Orari!$F$6:$F$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(10,30,0))*(Orari!$D$6:$D$15&gt;TIME(10,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(10,30,0))*(Orari!$F$6:$F$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(11,30,0))*(Orari!$D$6:$D$15&gt;TIME(11,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(11,30,0))*(Orari!$F$6:$F$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(12,30,0))*(Orari!$D$6:$D$15&gt;TIME(12,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(12,30,0))*(Orari!$F$6:$F$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(13,30,0))*(Orari!$D$6:$D$15&gt;TIME(13,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(13,30,0))*(Orari!$F$6:$F$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(14,30,0))*(Orari!$D$6:$D$15&gt;TIME(14,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(14,30,0))*(Orari!$F$6:$F$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(15,30,0))*(Orari!$D$6:$D$15&gt;TIME(15,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(15,30,0))*(Orari!$F$6:$F$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(16,30,0))*(Orari!$D$6:$D$15&gt;TIME(16,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(16,30,0))*(Orari!$F$6:$F$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J5" s="7">
+      <c r="J5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(17,30,0))*(Orari!$D$6:$D$15&gt;TIME(17,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(17,30,0))*(Orari!$F$6:$F$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K5" s="7">
+      <c r="K5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(18,30,0))*(Orari!$D$6:$D$15&gt;TIME(18,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(18,30,0))*(Orari!$F$6:$F$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L5" s="7">
+      <c r="L5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(19,30,0))*(Orari!$D$6:$D$15&gt;TIME(19,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(19,30,0))*(Orari!$F$6:$F$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M5" s="7">
+      <c r="M5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(20,30,0))*(Orari!$D$6:$D$15&gt;TIME(20,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(20,30,0))*(Orari!$F$6:$F$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -1960,51 +1968,51 @@
           <t>martedì 13 ottobre 2026</t>
         </is>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(9,30,0))*(Orari!$H$6:$H$15&gt;TIME(9,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(9,30,0))*(Orari!$J$6:$J$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(10,30,0))*(Orari!$H$6:$H$15&gt;TIME(10,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(10,30,0))*(Orari!$J$6:$J$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(11,30,0))*(Orari!$H$6:$H$15&gt;TIME(11,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(11,30,0))*(Orari!$J$6:$J$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(12,30,0))*(Orari!$H$6:$H$15&gt;TIME(12,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(12,30,0))*(Orari!$J$6:$J$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(13,30,0))*(Orari!$H$6:$H$15&gt;TIME(13,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(13,30,0))*(Orari!$J$6:$J$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(14,30,0))*(Orari!$H$6:$H$15&gt;TIME(14,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(14,30,0))*(Orari!$J$6:$J$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(15,30,0))*(Orari!$H$6:$H$15&gt;TIME(15,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(15,30,0))*(Orari!$J$6:$J$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(16,30,0))*(Orari!$H$6:$H$15&gt;TIME(16,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(16,30,0))*(Orari!$J$6:$J$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J6" s="7">
+      <c r="J6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(17,30,0))*(Orari!$H$6:$H$15&gt;TIME(17,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(17,30,0))*(Orari!$J$6:$J$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K6" s="7">
+      <c r="K6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(18,30,0))*(Orari!$H$6:$H$15&gt;TIME(18,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(18,30,0))*(Orari!$J$6:$J$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L6" s="7">
+      <c r="L6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(19,30,0))*(Orari!$H$6:$H$15&gt;TIME(19,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(19,30,0))*(Orari!$J$6:$J$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M6" s="7">
+      <c r="M6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(20,30,0))*(Orari!$H$6:$H$15&gt;TIME(20,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(20,30,0))*(Orari!$J$6:$J$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2015,51 +2023,51 @@
           <t>mercoledì 14 ottobre 2026</t>
         </is>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(9,30,0))*(Orari!$L$6:$L$15&gt;TIME(9,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(9,30,0))*(Orari!$N$6:$N$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(10,30,0))*(Orari!$L$6:$L$15&gt;TIME(10,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(10,30,0))*(Orari!$N$6:$N$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(11,30,0))*(Orari!$L$6:$L$15&gt;TIME(11,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(11,30,0))*(Orari!$N$6:$N$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(12,30,0))*(Orari!$L$6:$L$15&gt;TIME(12,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(12,30,0))*(Orari!$N$6:$N$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(13,30,0))*(Orari!$L$6:$L$15&gt;TIME(13,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(13,30,0))*(Orari!$N$6:$N$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(14,30,0))*(Orari!$L$6:$L$15&gt;TIME(14,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(14,30,0))*(Orari!$N$6:$N$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H7" s="7">
+      <c r="H7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(15,30,0))*(Orari!$L$6:$L$15&gt;TIME(15,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(15,30,0))*(Orari!$N$6:$N$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I7" s="7">
+      <c r="I7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(16,30,0))*(Orari!$L$6:$L$15&gt;TIME(16,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(16,30,0))*(Orari!$N$6:$N$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J7" s="7">
+      <c r="J7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(17,30,0))*(Orari!$L$6:$L$15&gt;TIME(17,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(17,30,0))*(Orari!$N$6:$N$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K7" s="7">
+      <c r="K7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(18,30,0))*(Orari!$L$6:$L$15&gt;TIME(18,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(18,30,0))*(Orari!$N$6:$N$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L7" s="7">
+      <c r="L7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(19,30,0))*(Orari!$L$6:$L$15&gt;TIME(19,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(19,30,0))*(Orari!$N$6:$N$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M7" s="7">
+      <c r="M7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(20,30,0))*(Orari!$L$6:$L$15&gt;TIME(20,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(20,30,0))*(Orari!$N$6:$N$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2070,51 +2078,51 @@
           <t>giovedì 15 ottobre 2026</t>
         </is>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(9,30,0))*(Orari!$P$6:$P$15&gt;TIME(9,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(9,30,0))*(Orari!$R$6:$R$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(10,30,0))*(Orari!$P$6:$P$15&gt;TIME(10,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(10,30,0))*(Orari!$R$6:$R$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(11,30,0))*(Orari!$P$6:$P$15&gt;TIME(11,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(11,30,0))*(Orari!$R$6:$R$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(12,30,0))*(Orari!$P$6:$P$15&gt;TIME(12,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(12,30,0))*(Orari!$R$6:$R$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(13,30,0))*(Orari!$P$6:$P$15&gt;TIME(13,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(13,30,0))*(Orari!$R$6:$R$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(14,30,0))*(Orari!$P$6:$P$15&gt;TIME(14,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(14,30,0))*(Orari!$R$6:$R$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(15,30,0))*(Orari!$P$6:$P$15&gt;TIME(15,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(15,30,0))*(Orari!$R$6:$R$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(16,30,0))*(Orari!$P$6:$P$15&gt;TIME(16,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(16,30,0))*(Orari!$R$6:$R$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J8" s="7">
+      <c r="J8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(17,30,0))*(Orari!$P$6:$P$15&gt;TIME(17,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(17,30,0))*(Orari!$R$6:$R$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K8" s="7">
+      <c r="K8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(18,30,0))*(Orari!$P$6:$P$15&gt;TIME(18,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(18,30,0))*(Orari!$R$6:$R$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L8" s="7">
+      <c r="L8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(19,30,0))*(Orari!$P$6:$P$15&gt;TIME(19,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(19,30,0))*(Orari!$R$6:$R$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M8" s="7">
+      <c r="M8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(20,30,0))*(Orari!$P$6:$P$15&gt;TIME(20,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(20,30,0))*(Orari!$R$6:$R$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2125,51 +2133,51 @@
           <t>venerdì 16 ottobre 2026</t>
         </is>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(9,30,0))*(Orari!$T$6:$T$15&gt;TIME(9,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(9,30,0))*(Orari!$V$6:$V$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(10,30,0))*(Orari!$T$6:$T$15&gt;TIME(10,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(10,30,0))*(Orari!$V$6:$V$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(11,30,0))*(Orari!$T$6:$T$15&gt;TIME(11,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(11,30,0))*(Orari!$V$6:$V$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(12,30,0))*(Orari!$T$6:$T$15&gt;TIME(12,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(12,30,0))*(Orari!$V$6:$V$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(13,30,0))*(Orari!$T$6:$T$15&gt;TIME(13,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(13,30,0))*(Orari!$V$6:$V$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(14,30,0))*(Orari!$T$6:$T$15&gt;TIME(14,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(14,30,0))*(Orari!$V$6:$V$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H9" s="7">
+      <c r="H9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(15,30,0))*(Orari!$T$6:$T$15&gt;TIME(15,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(15,30,0))*(Orari!$V$6:$V$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(16,30,0))*(Orari!$T$6:$T$15&gt;TIME(16,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(16,30,0))*(Orari!$V$6:$V$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J9" s="7">
+      <c r="J9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(17,30,0))*(Orari!$T$6:$T$15&gt;TIME(17,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(17,30,0))*(Orari!$V$6:$V$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K9" s="7">
+      <c r="K9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(18,30,0))*(Orari!$T$6:$T$15&gt;TIME(18,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(18,30,0))*(Orari!$V$6:$V$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L9" s="7">
+      <c r="L9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(19,30,0))*(Orari!$T$6:$T$15&gt;TIME(19,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(19,30,0))*(Orari!$V$6:$V$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M9" s="7">
+      <c r="M9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(20,30,0))*(Orari!$T$6:$T$15&gt;TIME(20,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(20,30,0))*(Orari!$V$6:$V$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2180,51 +2188,51 @@
           <t>sabato 17 ottobre 2026</t>
         </is>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(9,30,0))*(Orari!$X$6:$X$15&gt;TIME(9,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(9,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(10,30,0))*(Orari!$X$6:$X$15&gt;TIME(10,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(10,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(11,30,0))*(Orari!$X$6:$X$15&gt;TIME(11,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(11,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(12,30,0))*(Orari!$X$6:$X$15&gt;TIME(12,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(12,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F10" s="7">
+      <c r="F10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(13,30,0))*(Orari!$X$6:$X$15&gt;TIME(13,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(13,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G10" s="7">
+      <c r="G10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(14,30,0))*(Orari!$X$6:$X$15&gt;TIME(14,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(14,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H10" s="7">
+      <c r="H10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(15,30,0))*(Orari!$X$6:$X$15&gt;TIME(15,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(15,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I10" s="7">
+      <c r="I10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(16,30,0))*(Orari!$X$6:$X$15&gt;TIME(16,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(16,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J10" s="7">
+      <c r="J10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(17,30,0))*(Orari!$X$6:$X$15&gt;TIME(17,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(17,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K10" s="7">
+      <c r="K10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(18,30,0))*(Orari!$X$6:$X$15&gt;TIME(18,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(18,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L10" s="7">
+      <c r="L10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(19,30,0))*(Orari!$X$6:$X$15&gt;TIME(19,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(19,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M10" s="7">
+      <c r="M10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(20,30,0))*(Orari!$X$6:$X$15&gt;TIME(20,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(20,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2235,51 +2243,51 @@
           <t>domenica 18 ottobre 2026</t>
         </is>
       </c>
-      <c r="B11" s="7">
+      <c r="B11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(9,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(9,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(9,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(10,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(10,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(10,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(11,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(11,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(11,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(12,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(12,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(12,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F11" s="7">
+      <c r="F11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(13,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(13,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(13,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G11" s="7">
+      <c r="G11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(14,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(14,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(14,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H11" s="7">
+      <c r="H11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(15,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(15,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(15,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(16,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(16,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(16,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J11" s="7">
+      <c r="J11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(17,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(17,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(17,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K11" s="7">
+      <c r="K11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(18,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(18,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(18,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L11" s="7">
+      <c r="L11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(19,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(19,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(19,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M11" s="7">
+      <c r="M11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(20,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(20,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(20,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2364,51 +2372,51 @@
           <t>lunedì 12 ottobre 2026</t>
         </is>
       </c>
-      <c r="B15" s="7">
+      <c r="B15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(9,30,0))*(Orari!$D$6:$D$15&gt;TIME(9,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(9,30,0))*(Orari!$F$6:$F$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C15" s="7">
+      <c r="C15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(10,30,0))*(Orari!$D$6:$D$15&gt;TIME(10,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(10,30,0))*(Orari!$F$6:$F$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D15" s="7">
+      <c r="D15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(11,30,0))*(Orari!$D$6:$D$15&gt;TIME(11,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(11,30,0))*(Orari!$F$6:$F$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E15" s="7">
+      <c r="E15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(12,30,0))*(Orari!$D$6:$D$15&gt;TIME(12,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(12,30,0))*(Orari!$F$6:$F$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F15" s="7">
+      <c r="F15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(13,30,0))*(Orari!$D$6:$D$15&gt;TIME(13,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(13,30,0))*(Orari!$F$6:$F$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G15" s="7">
+      <c r="G15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(14,30,0))*(Orari!$D$6:$D$15&gt;TIME(14,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(14,30,0))*(Orari!$F$6:$F$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H15" s="7">
+      <c r="H15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(15,30,0))*(Orari!$D$6:$D$15&gt;TIME(15,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(15,30,0))*(Orari!$F$6:$F$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I15" s="7">
+      <c r="I15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(16,30,0))*(Orari!$D$6:$D$15&gt;TIME(16,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(16,30,0))*(Orari!$F$6:$F$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J15" s="7">
+      <c r="J15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(17,30,0))*(Orari!$D$6:$D$15&gt;TIME(17,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(17,30,0))*(Orari!$F$6:$F$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K15" s="7">
+      <c r="K15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(18,30,0))*(Orari!$D$6:$D$15&gt;TIME(18,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(18,30,0))*(Orari!$F$6:$F$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L15" s="7">
+      <c r="L15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(19,30,0))*(Orari!$D$6:$D$15&gt;TIME(19,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(19,30,0))*(Orari!$F$6:$F$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M15" s="7">
+      <c r="M15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(20,30,0))*(Orari!$D$6:$D$15&gt;TIME(20,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(20,30,0))*(Orari!$F$6:$F$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2419,51 +2427,51 @@
           <t>martedì 13 ottobre 2026</t>
         </is>
       </c>
-      <c r="B16" s="7">
+      <c r="B16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(9,30,0))*(Orari!$H$6:$H$15&gt;TIME(9,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(9,30,0))*(Orari!$J$6:$J$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C16" s="7">
+      <c r="C16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(10,30,0))*(Orari!$H$6:$H$15&gt;TIME(10,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(10,30,0))*(Orari!$J$6:$J$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D16" s="7">
+      <c r="D16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(11,30,0))*(Orari!$H$6:$H$15&gt;TIME(11,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(11,30,0))*(Orari!$J$6:$J$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E16" s="7">
+      <c r="E16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(12,30,0))*(Orari!$H$6:$H$15&gt;TIME(12,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(12,30,0))*(Orari!$J$6:$J$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F16" s="7">
+      <c r="F16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(13,30,0))*(Orari!$H$6:$H$15&gt;TIME(13,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(13,30,0))*(Orari!$J$6:$J$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G16" s="7">
+      <c r="G16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(14,30,0))*(Orari!$H$6:$H$15&gt;TIME(14,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(14,30,0))*(Orari!$J$6:$J$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H16" s="7">
+      <c r="H16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(15,30,0))*(Orari!$H$6:$H$15&gt;TIME(15,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(15,30,0))*(Orari!$J$6:$J$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I16" s="7">
+      <c r="I16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(16,30,0))*(Orari!$H$6:$H$15&gt;TIME(16,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(16,30,0))*(Orari!$J$6:$J$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J16" s="7">
+      <c r="J16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(17,30,0))*(Orari!$H$6:$H$15&gt;TIME(17,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(17,30,0))*(Orari!$J$6:$J$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K16" s="7">
+      <c r="K16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(18,30,0))*(Orari!$H$6:$H$15&gt;TIME(18,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(18,30,0))*(Orari!$J$6:$J$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L16" s="7">
+      <c r="L16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(19,30,0))*(Orari!$H$6:$H$15&gt;TIME(19,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(19,30,0))*(Orari!$J$6:$J$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M16" s="7">
+      <c r="M16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(20,30,0))*(Orari!$H$6:$H$15&gt;TIME(20,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(20,30,0))*(Orari!$J$6:$J$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2474,51 +2482,51 @@
           <t>mercoledì 14 ottobre 2026</t>
         </is>
       </c>
-      <c r="B17" s="7">
+      <c r="B17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(9,30,0))*(Orari!$L$6:$L$15&gt;TIME(9,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(9,30,0))*(Orari!$N$6:$N$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C17" s="7">
+      <c r="C17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(10,30,0))*(Orari!$L$6:$L$15&gt;TIME(10,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(10,30,0))*(Orari!$N$6:$N$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D17" s="7">
+      <c r="D17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(11,30,0))*(Orari!$L$6:$L$15&gt;TIME(11,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(11,30,0))*(Orari!$N$6:$N$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E17" s="7">
+      <c r="E17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(12,30,0))*(Orari!$L$6:$L$15&gt;TIME(12,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(12,30,0))*(Orari!$N$6:$N$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F17" s="7">
+      <c r="F17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(13,30,0))*(Orari!$L$6:$L$15&gt;TIME(13,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(13,30,0))*(Orari!$N$6:$N$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G17" s="7">
+      <c r="G17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(14,30,0))*(Orari!$L$6:$L$15&gt;TIME(14,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(14,30,0))*(Orari!$N$6:$N$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H17" s="7">
+      <c r="H17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(15,30,0))*(Orari!$L$6:$L$15&gt;TIME(15,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(15,30,0))*(Orari!$N$6:$N$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I17" s="7">
+      <c r="I17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(16,30,0))*(Orari!$L$6:$L$15&gt;TIME(16,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(16,30,0))*(Orari!$N$6:$N$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J17" s="7">
+      <c r="J17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(17,30,0))*(Orari!$L$6:$L$15&gt;TIME(17,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(17,30,0))*(Orari!$N$6:$N$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K17" s="7">
+      <c r="K17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(18,30,0))*(Orari!$L$6:$L$15&gt;TIME(18,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(18,30,0))*(Orari!$N$6:$N$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L17" s="7">
+      <c r="L17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(19,30,0))*(Orari!$L$6:$L$15&gt;TIME(19,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(19,30,0))*(Orari!$N$6:$N$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M17" s="7">
+      <c r="M17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(20,30,0))*(Orari!$L$6:$L$15&gt;TIME(20,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(20,30,0))*(Orari!$N$6:$N$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2529,51 +2537,51 @@
           <t>giovedì 15 ottobre 2026</t>
         </is>
       </c>
-      <c r="B18" s="7">
+      <c r="B18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(9,30,0))*(Orari!$P$6:$P$15&gt;TIME(9,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(9,30,0))*(Orari!$R$6:$R$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C18" s="7">
+      <c r="C18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(10,30,0))*(Orari!$P$6:$P$15&gt;TIME(10,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(10,30,0))*(Orari!$R$6:$R$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D18" s="7">
+      <c r="D18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(11,30,0))*(Orari!$P$6:$P$15&gt;TIME(11,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(11,30,0))*(Orari!$R$6:$R$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E18" s="7">
+      <c r="E18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(12,30,0))*(Orari!$P$6:$P$15&gt;TIME(12,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(12,30,0))*(Orari!$R$6:$R$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F18" s="7">
+      <c r="F18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(13,30,0))*(Orari!$P$6:$P$15&gt;TIME(13,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(13,30,0))*(Orari!$R$6:$R$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G18" s="7">
+      <c r="G18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(14,30,0))*(Orari!$P$6:$P$15&gt;TIME(14,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(14,30,0))*(Orari!$R$6:$R$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H18" s="7">
+      <c r="H18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(15,30,0))*(Orari!$P$6:$P$15&gt;TIME(15,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(15,30,0))*(Orari!$R$6:$R$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I18" s="7">
+      <c r="I18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(16,30,0))*(Orari!$P$6:$P$15&gt;TIME(16,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(16,30,0))*(Orari!$R$6:$R$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J18" s="7">
+      <c r="J18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(17,30,0))*(Orari!$P$6:$P$15&gt;TIME(17,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(17,30,0))*(Orari!$R$6:$R$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K18" s="7">
+      <c r="K18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(18,30,0))*(Orari!$P$6:$P$15&gt;TIME(18,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(18,30,0))*(Orari!$R$6:$R$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L18" s="7">
+      <c r="L18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(19,30,0))*(Orari!$P$6:$P$15&gt;TIME(19,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(19,30,0))*(Orari!$R$6:$R$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M18" s="7">
+      <c r="M18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(20,30,0))*(Orari!$P$6:$P$15&gt;TIME(20,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(20,30,0))*(Orari!$R$6:$R$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2584,51 +2592,51 @@
           <t>venerdì 16 ottobre 2026</t>
         </is>
       </c>
-      <c r="B19" s="7">
+      <c r="B19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(9,30,0))*(Orari!$T$6:$T$15&gt;TIME(9,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(9,30,0))*(Orari!$V$6:$V$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C19" s="7">
+      <c r="C19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(10,30,0))*(Orari!$T$6:$T$15&gt;TIME(10,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(10,30,0))*(Orari!$V$6:$V$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D19" s="7">
+      <c r="D19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(11,30,0))*(Orari!$T$6:$T$15&gt;TIME(11,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(11,30,0))*(Orari!$V$6:$V$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E19" s="7">
+      <c r="E19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(12,30,0))*(Orari!$T$6:$T$15&gt;TIME(12,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(12,30,0))*(Orari!$V$6:$V$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F19" s="7">
+      <c r="F19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(13,30,0))*(Orari!$T$6:$T$15&gt;TIME(13,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(13,30,0))*(Orari!$V$6:$V$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G19" s="7">
+      <c r="G19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(14,30,0))*(Orari!$T$6:$T$15&gt;TIME(14,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(14,30,0))*(Orari!$V$6:$V$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H19" s="7">
+      <c r="H19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(15,30,0))*(Orari!$T$6:$T$15&gt;TIME(15,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(15,30,0))*(Orari!$V$6:$V$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I19" s="7">
+      <c r="I19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(16,30,0))*(Orari!$T$6:$T$15&gt;TIME(16,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(16,30,0))*(Orari!$V$6:$V$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J19" s="7">
+      <c r="J19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(17,30,0))*(Orari!$T$6:$T$15&gt;TIME(17,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(17,30,0))*(Orari!$V$6:$V$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K19" s="7">
+      <c r="K19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(18,30,0))*(Orari!$T$6:$T$15&gt;TIME(18,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(18,30,0))*(Orari!$V$6:$V$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L19" s="7">
+      <c r="L19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(19,30,0))*(Orari!$T$6:$T$15&gt;TIME(19,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(19,30,0))*(Orari!$V$6:$V$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M19" s="7">
+      <c r="M19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(20,30,0))*(Orari!$T$6:$T$15&gt;TIME(20,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(20,30,0))*(Orari!$V$6:$V$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2639,51 +2647,51 @@
           <t>sabato 17 ottobre 2026</t>
         </is>
       </c>
-      <c r="B20" s="7">
+      <c r="B20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(9,30,0))*(Orari!$X$6:$X$15&gt;TIME(9,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(9,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C20" s="7">
+      <c r="C20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(10,30,0))*(Orari!$X$6:$X$15&gt;TIME(10,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(10,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D20" s="7">
+      <c r="D20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(11,30,0))*(Orari!$X$6:$X$15&gt;TIME(11,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(11,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E20" s="7">
+      <c r="E20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(12,30,0))*(Orari!$X$6:$X$15&gt;TIME(12,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(12,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F20" s="7">
+      <c r="F20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(13,30,0))*(Orari!$X$6:$X$15&gt;TIME(13,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(13,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G20" s="7">
+      <c r="G20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(14,30,0))*(Orari!$X$6:$X$15&gt;TIME(14,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(14,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H20" s="7">
+      <c r="H20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(15,30,0))*(Orari!$X$6:$X$15&gt;TIME(15,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(15,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I20" s="7">
+      <c r="I20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(16,30,0))*(Orari!$X$6:$X$15&gt;TIME(16,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(16,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J20" s="7">
+      <c r="J20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(17,30,0))*(Orari!$X$6:$X$15&gt;TIME(17,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(17,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K20" s="7">
+      <c r="K20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(18,30,0))*(Orari!$X$6:$X$15&gt;TIME(18,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(18,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L20" s="7">
+      <c r="L20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(19,30,0))*(Orari!$X$6:$X$15&gt;TIME(19,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(19,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M20" s="7">
+      <c r="M20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(20,30,0))*(Orari!$X$6:$X$15&gt;TIME(20,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(20,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2694,51 +2702,51 @@
           <t>domenica 18 ottobre 2026</t>
         </is>
       </c>
-      <c r="B21" s="7">
+      <c r="B21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(9,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(9,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(9,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C21" s="7">
+      <c r="C21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(10,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(10,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(10,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D21" s="7">
+      <c r="D21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(11,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(11,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(11,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E21" s="7">
+      <c r="E21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(12,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(12,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(12,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F21" s="7">
+      <c r="F21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(13,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(13,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(13,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G21" s="7">
+      <c r="G21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(14,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(14,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(14,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H21" s="7">
+      <c r="H21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(15,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(15,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(15,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I21" s="7">
+      <c r="I21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(16,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(16,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(16,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J21" s="7">
+      <c r="J21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(17,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(17,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(17,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K21" s="7">
+      <c r="K21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(18,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(18,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(18,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L21" s="7">
+      <c r="L21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(19,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(19,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(19,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M21" s="7">
+      <c r="M21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(20,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(20,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(20,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2823,51 +2831,51 @@
           <t>lunedì 12 ottobre 2026</t>
         </is>
       </c>
-      <c r="B25" s="7">
+      <c r="B25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(9,30,0))*(Orari!$D$6:$D$15&gt;TIME(9,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(9,30,0))*(Orari!$F$6:$F$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C25" s="7">
+      <c r="C25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(10,30,0))*(Orari!$D$6:$D$15&gt;TIME(10,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(10,30,0))*(Orari!$F$6:$F$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D25" s="7">
+      <c r="D25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(11,30,0))*(Orari!$D$6:$D$15&gt;TIME(11,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(11,30,0))*(Orari!$F$6:$F$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E25" s="7">
+      <c r="E25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(12,30,0))*(Orari!$D$6:$D$15&gt;TIME(12,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(12,30,0))*(Orari!$F$6:$F$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F25" s="7">
+      <c r="F25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(13,30,0))*(Orari!$D$6:$D$15&gt;TIME(13,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(13,30,0))*(Orari!$F$6:$F$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G25" s="7">
+      <c r="G25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(14,30,0))*(Orari!$D$6:$D$15&gt;TIME(14,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(14,30,0))*(Orari!$F$6:$F$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H25" s="7">
+      <c r="H25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(15,30,0))*(Orari!$D$6:$D$15&gt;TIME(15,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(15,30,0))*(Orari!$F$6:$F$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I25" s="7">
+      <c r="I25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(16,30,0))*(Orari!$D$6:$D$15&gt;TIME(16,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(16,30,0))*(Orari!$F$6:$F$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J25" s="7">
+      <c r="J25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(17,30,0))*(Orari!$D$6:$D$15&gt;TIME(17,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(17,30,0))*(Orari!$F$6:$F$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K25" s="7">
+      <c r="K25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(18,30,0))*(Orari!$D$6:$D$15&gt;TIME(18,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(18,30,0))*(Orari!$F$6:$F$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L25" s="7">
+      <c r="L25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(19,30,0))*(Orari!$D$6:$D$15&gt;TIME(19,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(19,30,0))*(Orari!$F$6:$F$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M25" s="7">
+      <c r="M25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(20,30,0))*(Orari!$D$6:$D$15&gt;TIME(20,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(20,30,0))*(Orari!$F$6:$F$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2878,51 +2886,51 @@
           <t>martedì 13 ottobre 2026</t>
         </is>
       </c>
-      <c r="B26" s="7">
+      <c r="B26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(9,30,0))*(Orari!$H$6:$H$15&gt;TIME(9,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(9,30,0))*(Orari!$J$6:$J$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C26" s="7">
+      <c r="C26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(10,30,0))*(Orari!$H$6:$H$15&gt;TIME(10,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(10,30,0))*(Orari!$J$6:$J$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D26" s="7">
+      <c r="D26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(11,30,0))*(Orari!$H$6:$H$15&gt;TIME(11,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(11,30,0))*(Orari!$J$6:$J$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E26" s="7">
+      <c r="E26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(12,30,0))*(Orari!$H$6:$H$15&gt;TIME(12,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(12,30,0))*(Orari!$J$6:$J$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F26" s="7">
+      <c r="F26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(13,30,0))*(Orari!$H$6:$H$15&gt;TIME(13,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(13,30,0))*(Orari!$J$6:$J$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G26" s="7">
+      <c r="G26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(14,30,0))*(Orari!$H$6:$H$15&gt;TIME(14,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(14,30,0))*(Orari!$J$6:$J$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H26" s="7">
+      <c r="H26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(15,30,0))*(Orari!$H$6:$H$15&gt;TIME(15,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(15,30,0))*(Orari!$J$6:$J$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I26" s="7">
+      <c r="I26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(16,30,0))*(Orari!$H$6:$H$15&gt;TIME(16,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(16,30,0))*(Orari!$J$6:$J$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J26" s="7">
+      <c r="J26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(17,30,0))*(Orari!$H$6:$H$15&gt;TIME(17,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(17,30,0))*(Orari!$J$6:$J$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K26" s="7">
+      <c r="K26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(18,30,0))*(Orari!$H$6:$H$15&gt;TIME(18,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(18,30,0))*(Orari!$J$6:$J$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L26" s="7">
+      <c r="L26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(19,30,0))*(Orari!$H$6:$H$15&gt;TIME(19,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(19,30,0))*(Orari!$J$6:$J$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M26" s="7">
+      <c r="M26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(20,30,0))*(Orari!$H$6:$H$15&gt;TIME(20,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(20,30,0))*(Orari!$J$6:$J$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2933,51 +2941,51 @@
           <t>mercoledì 14 ottobre 2026</t>
         </is>
       </c>
-      <c r="B27" s="7">
+      <c r="B27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(9,30,0))*(Orari!$L$6:$L$15&gt;TIME(9,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(9,30,0))*(Orari!$N$6:$N$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C27" s="7">
+      <c r="C27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(10,30,0))*(Orari!$L$6:$L$15&gt;TIME(10,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(10,30,0))*(Orari!$N$6:$N$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D27" s="7">
+      <c r="D27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(11,30,0))*(Orari!$L$6:$L$15&gt;TIME(11,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(11,30,0))*(Orari!$N$6:$N$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E27" s="7">
+      <c r="E27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(12,30,0))*(Orari!$L$6:$L$15&gt;TIME(12,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(12,30,0))*(Orari!$N$6:$N$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F27" s="7">
+      <c r="F27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(13,30,0))*(Orari!$L$6:$L$15&gt;TIME(13,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(13,30,0))*(Orari!$N$6:$N$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G27" s="7">
+      <c r="G27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(14,30,0))*(Orari!$L$6:$L$15&gt;TIME(14,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(14,30,0))*(Orari!$N$6:$N$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H27" s="7">
+      <c r="H27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(15,30,0))*(Orari!$L$6:$L$15&gt;TIME(15,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(15,30,0))*(Orari!$N$6:$N$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I27" s="7">
+      <c r="I27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(16,30,0))*(Orari!$L$6:$L$15&gt;TIME(16,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(16,30,0))*(Orari!$N$6:$N$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J27" s="7">
+      <c r="J27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(17,30,0))*(Orari!$L$6:$L$15&gt;TIME(17,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(17,30,0))*(Orari!$N$6:$N$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K27" s="7">
+      <c r="K27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(18,30,0))*(Orari!$L$6:$L$15&gt;TIME(18,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(18,30,0))*(Orari!$N$6:$N$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L27" s="7">
+      <c r="L27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(19,30,0))*(Orari!$L$6:$L$15&gt;TIME(19,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(19,30,0))*(Orari!$N$6:$N$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M27" s="7">
+      <c r="M27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(20,30,0))*(Orari!$L$6:$L$15&gt;TIME(20,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(20,30,0))*(Orari!$N$6:$N$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2988,51 +2996,51 @@
           <t>giovedì 15 ottobre 2026</t>
         </is>
       </c>
-      <c r="B28" s="7">
+      <c r="B28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(9,30,0))*(Orari!$P$6:$P$15&gt;TIME(9,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(9,30,0))*(Orari!$R$6:$R$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C28" s="7">
+      <c r="C28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(10,30,0))*(Orari!$P$6:$P$15&gt;TIME(10,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(10,30,0))*(Orari!$R$6:$R$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D28" s="7">
+      <c r="D28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(11,30,0))*(Orari!$P$6:$P$15&gt;TIME(11,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(11,30,0))*(Orari!$R$6:$R$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E28" s="7">
+      <c r="E28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(12,30,0))*(Orari!$P$6:$P$15&gt;TIME(12,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(12,30,0))*(Orari!$R$6:$R$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F28" s="7">
+      <c r="F28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(13,30,0))*(Orari!$P$6:$P$15&gt;TIME(13,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(13,30,0))*(Orari!$R$6:$R$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G28" s="7">
+      <c r="G28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(14,30,0))*(Orari!$P$6:$P$15&gt;TIME(14,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(14,30,0))*(Orari!$R$6:$R$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H28" s="7">
+      <c r="H28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(15,30,0))*(Orari!$P$6:$P$15&gt;TIME(15,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(15,30,0))*(Orari!$R$6:$R$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I28" s="7">
+      <c r="I28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(16,30,0))*(Orari!$P$6:$P$15&gt;TIME(16,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(16,30,0))*(Orari!$R$6:$R$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J28" s="7">
+      <c r="J28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(17,30,0))*(Orari!$P$6:$P$15&gt;TIME(17,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(17,30,0))*(Orari!$R$6:$R$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K28" s="7">
+      <c r="K28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(18,30,0))*(Orari!$P$6:$P$15&gt;TIME(18,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(18,30,0))*(Orari!$R$6:$R$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L28" s="7">
+      <c r="L28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(19,30,0))*(Orari!$P$6:$P$15&gt;TIME(19,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(19,30,0))*(Orari!$R$6:$R$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M28" s="7">
+      <c r="M28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(20,30,0))*(Orari!$P$6:$P$15&gt;TIME(20,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(20,30,0))*(Orari!$R$6:$R$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -3043,51 +3051,51 @@
           <t>venerdì 16 ottobre 2026</t>
         </is>
       </c>
-      <c r="B29" s="7">
+      <c r="B29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(9,30,0))*(Orari!$T$6:$T$15&gt;TIME(9,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(9,30,0))*(Orari!$V$6:$V$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C29" s="7">
+      <c r="C29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(10,30,0))*(Orari!$T$6:$T$15&gt;TIME(10,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(10,30,0))*(Orari!$V$6:$V$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D29" s="7">
+      <c r="D29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(11,30,0))*(Orari!$T$6:$T$15&gt;TIME(11,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(11,30,0))*(Orari!$V$6:$V$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E29" s="7">
+      <c r="E29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(12,30,0))*(Orari!$T$6:$T$15&gt;TIME(12,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(12,30,0))*(Orari!$V$6:$V$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F29" s="7">
+      <c r="F29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(13,30,0))*(Orari!$T$6:$T$15&gt;TIME(13,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(13,30,0))*(Orari!$V$6:$V$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G29" s="7">
+      <c r="G29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(14,30,0))*(Orari!$T$6:$T$15&gt;TIME(14,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(14,30,0))*(Orari!$V$6:$V$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H29" s="7">
+      <c r="H29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(15,30,0))*(Orari!$T$6:$T$15&gt;TIME(15,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(15,30,0))*(Orari!$V$6:$V$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I29" s="7">
+      <c r="I29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(16,30,0))*(Orari!$T$6:$T$15&gt;TIME(16,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(16,30,0))*(Orari!$V$6:$V$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J29" s="7">
+      <c r="J29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(17,30,0))*(Orari!$T$6:$T$15&gt;TIME(17,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(17,30,0))*(Orari!$V$6:$V$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K29" s="7">
+      <c r="K29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(18,30,0))*(Orari!$T$6:$T$15&gt;TIME(18,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(18,30,0))*(Orari!$V$6:$V$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L29" s="7">
+      <c r="L29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(19,30,0))*(Orari!$T$6:$T$15&gt;TIME(19,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(19,30,0))*(Orari!$V$6:$V$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M29" s="7">
+      <c r="M29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(20,30,0))*(Orari!$T$6:$T$15&gt;TIME(20,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(20,30,0))*(Orari!$V$6:$V$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -3098,51 +3106,51 @@
           <t>sabato 17 ottobre 2026</t>
         </is>
       </c>
-      <c r="B30" s="7">
+      <c r="B30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(9,30,0))*(Orari!$X$6:$X$15&gt;TIME(9,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(9,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C30" s="7">
+      <c r="C30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(10,30,0))*(Orari!$X$6:$X$15&gt;TIME(10,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(10,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D30" s="7">
+      <c r="D30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(11,30,0))*(Orari!$X$6:$X$15&gt;TIME(11,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(11,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E30" s="7">
+      <c r="E30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(12,30,0))*(Orari!$X$6:$X$15&gt;TIME(12,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(12,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F30" s="7">
+      <c r="F30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(13,30,0))*(Orari!$X$6:$X$15&gt;TIME(13,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(13,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G30" s="7">
+      <c r="G30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(14,30,0))*(Orari!$X$6:$X$15&gt;TIME(14,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(14,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H30" s="7">
+      <c r="H30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(15,30,0))*(Orari!$X$6:$X$15&gt;TIME(15,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(15,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I30" s="7">
+      <c r="I30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(16,30,0))*(Orari!$X$6:$X$15&gt;TIME(16,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(16,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J30" s="7">
+      <c r="J30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(17,30,0))*(Orari!$X$6:$X$15&gt;TIME(17,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(17,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K30" s="7">
+      <c r="K30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(18,30,0))*(Orari!$X$6:$X$15&gt;TIME(18,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(18,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L30" s="7">
+      <c r="L30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(19,30,0))*(Orari!$X$6:$X$15&gt;TIME(19,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(19,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M30" s="7">
+      <c r="M30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(20,30,0))*(Orari!$X$6:$X$15&gt;TIME(20,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(20,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -3153,51 +3161,51 @@
           <t>domenica 18 ottobre 2026</t>
         </is>
       </c>
-      <c r="B31" s="7">
+      <c r="B31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(9,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(9,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(9,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C31" s="7">
+      <c r="C31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(10,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(10,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(10,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D31" s="7">
+      <c r="D31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(11,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(11,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(11,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E31" s="7">
+      <c r="E31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(12,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(12,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(12,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F31" s="7">
+      <c r="F31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(13,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(13,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(13,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G31" s="7">
+      <c r="G31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(14,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(14,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(14,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H31" s="7">
+      <c r="H31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(15,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(15,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(15,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I31" s="7">
+      <c r="I31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(16,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(16,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(16,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J31" s="7">
+      <c r="J31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(17,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(17,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(17,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K31" s="7">
+      <c r="K31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(18,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(18,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(18,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L31" s="7">
+      <c r="L31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(19,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(19,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(19,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M31" s="7">
+      <c r="M31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(20,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(20,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(20,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Orari: casse fissate dal foglio del negozio, Latini Alessandro al posto di Bruni Laura
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RgW8tUpL59m5j1P2CKTdxn
</commit_message>
<xml_diff>
--- a/orari/Orari_12-18_ottobre_2026.xlsx
+++ b/orari/Orari_12-18_ottobre_2026.xlsx
@@ -104,10 +104,10 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AF20"/>
+  <dimension ref="A1:AF21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -869,7 +869,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>BRUNI LAURA</t>
+          <t>LATINI ALESSANDRO</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -877,14 +877,14 @@
           <t>Addetto vendite</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="D6" s="5" t="n">
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
+      <c r="F6" s="6" t="n">
+        <v>0.875</v>
+      </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
@@ -893,41 +893,49 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
       <c r="J6" s="7" t="n"/>
-      <c r="K6" s="6" t="n"/>
-      <c r="L6" s="6" t="n"/>
-      <c r="M6" s="5" t="n">
+      <c r="K6" s="5" t="n"/>
+      <c r="L6" s="5" t="n"/>
+      <c r="M6" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="N6" s="5" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="O6" s="5" t="n">
+      <c r="N6" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="O6" s="6" t="n">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="P6" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="Q6" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="R6" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="S6" s="6" t="n">
         <v>0.4166666666666667</v>
       </c>
-      <c r="P6" s="5" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="Q6" s="6" t="n"/>
-      <c r="R6" s="6" t="n"/>
-      <c r="S6" s="6" t="n"/>
-      <c r="T6" s="6" t="n"/>
-      <c r="U6" s="5" t="n">
+      <c r="T6" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="U6" s="6" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="V6" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="W6" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="X6" s="6" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="Y6" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="V6" s="5" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="W6" s="5" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="X6" s="5" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="Y6" s="5" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="Z6" s="5" t="n">
-        <v>0.8333333333333334</v>
+      <c r="Z6" s="6" t="n">
+        <v>0.7916666666666666</v>
       </c>
       <c r="AA6" s="7" t="inlineStr">
         <is>
@@ -941,8 +949,8 @@
         <f>ROUND(24*(N(D6)-N(C6)+N(F6)-N(E6)+N(H6)-N(G6)+N(J6)-N(I6)+N(L6)-N(K6)+N(N6)-N(M6)+N(P6)-N(O6)+N(R6)-N(Q6)+N(T6)-N(S6)+N(V6)-N(U6)+N(X6)-N(W6)+N(Z6)-N(Y6)+N(AB6)-N(AA6)+N(AD6)-N(AC6)),2)</f>
         <v/>
       </c>
-      <c r="AF6" s="6" t="n">
-        <v>30</v>
+      <c r="AF6" s="5" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="7">
@@ -956,83 +964,83 @@
           <t>Vicedirettore</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G7" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="H7" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="I7" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="H7" s="7" t="n"/>
-      <c r="I7" s="7" t="n"/>
-      <c r="J7" s="7" t="n"/>
-      <c r="K7" s="5" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="L7" s="5" t="n">
+      <c r="L7" s="7" t="n"/>
+      <c r="M7" s="7" t="n"/>
+      <c r="N7" s="7" t="n"/>
+      <c r="O7" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="P7" s="6" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="Q7" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="S7" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="T7" s="7" t="n"/>
+      <c r="U7" s="7" t="n"/>
+      <c r="V7" s="7" t="n"/>
+      <c r="W7" s="6" t="n">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="X7" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="M7" s="5" t="n">
+      <c r="Y7" s="6" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="N7" s="5" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="O7" s="5" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="P7" s="5" t="n">
+      <c r="Z7" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="AA7" s="5" t="n"/>
+      <c r="AB7" s="5" t="n"/>
+      <c r="AC7" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="Q7" s="5" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="R7" s="5" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="S7" s="5" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="T7" s="5" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="U7" s="5" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="V7" s="5" t="n">
+      <c r="AD7" s="6" t="n">
         <v>0.875</v>
       </c>
-      <c r="W7" s="5" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="X7" s="5" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="Y7" s="5" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="Z7" s="5" t="n">
-        <v>0.7916666666666666</v>
-      </c>
-      <c r="AA7" s="7" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="AB7" s="7" t="n"/>
-      <c r="AC7" s="7" t="n"/>
-      <c r="AD7" s="7" t="n"/>
       <c r="AE7" s="8">
         <f>ROUND(24*(N(D7)-N(C7)+N(F7)-N(E7)+N(H7)-N(G7)+N(J7)-N(I7)+N(L7)-N(K7)+N(N7)-N(M7)+N(P7)-N(O7)+N(R7)-N(Q7)+N(T7)-N(S7)+N(V7)-N(U7)+N(X7)-N(W7)+N(Z7)-N(Y7)+N(AB7)-N(AA7)+N(AD7)-N(AC7)),2)</f>
         <v/>
       </c>
-      <c r="AF7" s="6" t="inlineStr">
+      <c r="AF7" s="5" t="inlineStr">
         <is>
           <t>44-45</t>
         </is>
@@ -1049,79 +1057,79 @@
           <t>Addetto vendite</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="5" t="n">
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="J8" s="6" t="n">
         <v>0.875</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="K8" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="L8" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="M8" s="6" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="N8" s="6" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="O8" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="P8" s="7" t="n"/>
+      <c r="Q8" s="7" t="n"/>
+      <c r="R8" s="7" t="n"/>
+      <c r="S8" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="T8" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="U8" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="V8" s="6" t="n">
         <v>0.7916666666666666</v>
       </c>
-      <c r="K8" s="7" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="L8" s="7" t="n"/>
-      <c r="M8" s="7" t="n"/>
-      <c r="N8" s="7" t="n"/>
-      <c r="O8" s="6" t="n"/>
-      <c r="P8" s="6" t="n"/>
-      <c r="Q8" s="5" t="n">
+      <c r="W8" s="6" t="n">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="X8" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="Y8" s="6" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="Z8" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="AA8" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="AB8" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="R8" s="5" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="S8" s="7" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="T8" s="7" t="n"/>
-      <c r="U8" s="7" t="n"/>
-      <c r="V8" s="7" t="n"/>
-      <c r="W8" s="5" t="n">
-        <v>0.4583333333333333</v>
-      </c>
-      <c r="X8" s="5" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="Y8" s="5" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="Z8" s="5" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="AA8" s="5" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="AB8" s="5" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="AC8" s="5" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="AD8" s="5" t="n">
-        <v>0.875</v>
-      </c>
+      <c r="AC8" s="5" t="n"/>
+      <c r="AD8" s="5" t="n"/>
       <c r="AE8" s="8">
         <f>ROUND(24*(N(D8)-N(C8)+N(F8)-N(E8)+N(H8)-N(G8)+N(J8)-N(I8)+N(L8)-N(K8)+N(N8)-N(M8)+N(P8)-N(O8)+N(R8)-N(Q8)+N(T8)-N(S8)+N(V8)-N(U8)+N(X8)-N(W8)+N(Z8)-N(Y8)+N(AB8)-N(AA8)+N(AD8)-N(AC8)),2)</f>
         <v/>
       </c>
-      <c r="AF8" s="6" t="n">
+      <c r="AF8" s="5" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1136,41 +1144,45 @@
           <t>Addetto vendite</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="5" t="n">
+      <c r="C9" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="D9" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="E9" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="7" t="n"/>
+      <c r="K9" s="5" t="n"/>
+      <c r="L9" s="5" t="n"/>
+      <c r="M9" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="N9" s="6" t="n">
         <v>0.875</v>
       </c>
-      <c r="G9" s="5" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="H9" s="5" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="I9" s="5" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="J9" s="5" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="K9" s="7" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="L9" s="7" t="n"/>
-      <c r="M9" s="7" t="n"/>
-      <c r="N9" s="7" t="n"/>
-      <c r="O9" s="6" t="n"/>
-      <c r="P9" s="6" t="n"/>
-      <c r="Q9" s="5" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="R9" s="5" t="n">
-        <v>0.875</v>
+      <c r="O9" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="P9" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q9" s="6" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="R9" s="6" t="n">
+        <v>0.7916666666666666</v>
       </c>
       <c r="S9" s="7" t="inlineStr">
         <is>
@@ -1180,35 +1192,31 @@
       <c r="T9" s="7" t="n"/>
       <c r="U9" s="7" t="n"/>
       <c r="V9" s="7" t="n"/>
-      <c r="W9" s="5" t="n">
+      <c r="W9" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="X9" s="5" t="n">
+      <c r="X9" s="6" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="Y9" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="Y9" s="5" t="n">
+      <c r="Z9" s="6" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="AA9" s="5" t="n"/>
+      <c r="AB9" s="5" t="n"/>
+      <c r="AC9" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="Z9" s="5" t="n">
-        <v>0.7916666666666666</v>
-      </c>
-      <c r="AA9" s="5" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="AB9" s="5" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="AC9" s="5" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="AD9" s="5" t="n">
-        <v>0.7916666666666666</v>
+      <c r="AD9" s="6" t="n">
+        <v>0.875</v>
       </c>
       <c r="AE9" s="8">
         <f>ROUND(24*(N(D9)-N(C9)+N(F9)-N(E9)+N(H9)-N(G9)+N(J9)-N(I9)+N(L9)-N(K9)+N(N9)-N(M9)+N(P9)-N(O9)+N(R9)-N(Q9)+N(T9)-N(S9)+N(V9)-N(U9)+N(X9)-N(W9)+N(Z9)-N(Y9)+N(AB9)-N(AA9)+N(AD9)-N(AC9)),2)</f>
         <v/>
       </c>
-      <c r="AF9" s="6" t="n">
+      <c r="AF9" s="5" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1231,26 +1239,26 @@
       <c r="D10" s="7" t="n"/>
       <c r="E10" s="7" t="n"/>
       <c r="F10" s="7" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="5" t="n">
+      <c r="G10" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="L10" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="J10" s="5" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="K10" s="5" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="L10" s="5" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="M10" s="5" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="N10" s="5" t="n">
-        <v>0.875</v>
-      </c>
+      <c r="M10" s="5" t="n"/>
+      <c r="N10" s="5" t="n"/>
       <c r="O10" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
@@ -1259,43 +1267,43 @@
       <c r="P10" s="7" t="n"/>
       <c r="Q10" s="7" t="n"/>
       <c r="R10" s="7" t="n"/>
-      <c r="S10" s="5" t="n">
+      <c r="S10" s="5" t="n"/>
+      <c r="T10" s="5" t="n"/>
+      <c r="U10" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="V10" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="W10" s="6" t="n">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="X10" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="Y10" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="Z10" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="AA10" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="T10" s="5" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="U10" s="5" t="n">
+      <c r="AB10" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="V10" s="5" t="n">
+      <c r="AC10" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="AD10" s="6" t="n">
         <v>0.7916666666666666</v>
-      </c>
-      <c r="W10" s="5" t="n">
-        <v>0.4583333333333333</v>
-      </c>
-      <c r="X10" s="5" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="Y10" s="5" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="Z10" s="5" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="AA10" s="6" t="n"/>
-      <c r="AB10" s="6" t="n"/>
-      <c r="AC10" s="5" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="AD10" s="5" t="n">
-        <v>0.875</v>
       </c>
       <c r="AE10" s="8">
         <f>ROUND(24*(N(D10)-N(C10)+N(F10)-N(E10)+N(H10)-N(G10)+N(J10)-N(I10)+N(L10)-N(K10)+N(N10)-N(M10)+N(P10)-N(O10)+N(R10)-N(Q10)+N(T10)-N(S10)+N(V10)-N(U10)+N(X10)-N(W10)+N(Z10)-N(Y10)+N(AB10)-N(AA10)+N(AD10)-N(AC10)),2)</f>
         <v/>
       </c>
-      <c r="AF10" s="6" t="n">
+      <c r="AF10" s="5" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1310,79 +1318,83 @@
           <t>Cassiera</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="5" t="n">
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="7" t="n"/>
+      <c r="J11" s="7" t="n"/>
+      <c r="K11" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="S11" s="6" t="n">
         <v>0.4583333333333333</v>
       </c>
-      <c r="H11" s="5" t="n">
+      <c r="T11" s="6" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="U11" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="I11" s="5" t="n">
+      <c r="V11" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="W11" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="X11" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="J11" s="5" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="K11" s="5" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="L11" s="5" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="M11" s="5" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="N11" s="5" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="O11" s="7" t="inlineStr">
+      <c r="Y11" s="5" t="n"/>
+      <c r="Z11" s="5" t="n"/>
+      <c r="AA11" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="P11" s="7" t="n"/>
-      <c r="Q11" s="7" t="n"/>
-      <c r="R11" s="7" t="n"/>
-      <c r="S11" s="5" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="T11" s="5" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="U11" s="6" t="n"/>
-      <c r="V11" s="6" t="n"/>
-      <c r="W11" s="5" t="n">
-        <v>0.4583333333333333</v>
-      </c>
-      <c r="X11" s="5" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="Y11" s="5" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="Z11" s="5" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="AA11" s="5" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="AB11" s="5" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="AC11" s="6" t="n"/>
-      <c r="AD11" s="6" t="n"/>
+      <c r="AB11" s="7" t="n"/>
+      <c r="AC11" s="7" t="n"/>
+      <c r="AD11" s="7" t="n"/>
       <c r="AE11" s="8">
         <f>ROUND(24*(N(D11)-N(C11)+N(F11)-N(E11)+N(H11)-N(G11)+N(J11)-N(I11)+N(L11)-N(K11)+N(N11)-N(M11)+N(P11)-N(O11)+N(R11)-N(Q11)+N(T11)-N(S11)+N(V11)-N(U11)+N(X11)-N(W11)+N(Z11)-N(Y11)+N(AB11)-N(AA11)+N(AD11)-N(AC11)),2)</f>
         <v/>
       </c>
-      <c r="AF11" s="6" t="n">
+      <c r="AF11" s="5" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1397,71 +1409,71 @@
           <t>Cassiera</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="6" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="I12" s="5" t="n"/>
+      <c r="J12" s="5" t="n"/>
+      <c r="K12" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="7" t="n"/>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="L12" s="7" t="n"/>
+      <c r="M12" s="7" t="n"/>
+      <c r="N12" s="7" t="n"/>
+      <c r="O12" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="H12" s="7" t="n"/>
-      <c r="I12" s="7" t="n"/>
-      <c r="J12" s="7" t="n"/>
-      <c r="K12" s="5" t="n">
+      <c r="P12" s="7" t="n"/>
+      <c r="Q12" s="7" t="n"/>
+      <c r="R12" s="7" t="n"/>
+      <c r="S12" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="L12" s="5" t="n">
+      <c r="T12" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="U12" s="5" t="n"/>
+      <c r="V12" s="5" t="n"/>
+      <c r="W12" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="X12" s="7" t="n"/>
+      <c r="Y12" s="7" t="n"/>
+      <c r="Z12" s="7" t="n"/>
+      <c r="AA12" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="AB12" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="AC12" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="M12" s="6" t="n"/>
-      <c r="N12" s="6" t="n"/>
-      <c r="O12" s="6" t="n"/>
-      <c r="P12" s="6" t="n"/>
-      <c r="Q12" s="5" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="R12" s="5" t="n">
+      <c r="AD12" s="6" t="n">
         <v>0.875</v>
       </c>
-      <c r="S12" s="6" t="n"/>
-      <c r="T12" s="6" t="n"/>
-      <c r="U12" s="5" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="V12" s="5" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="W12" s="5" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="X12" s="5" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="Y12" s="5" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="Z12" s="5" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="AA12" s="7" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="AB12" s="7" t="n"/>
-      <c r="AC12" s="7" t="n"/>
-      <c r="AD12" s="7" t="n"/>
       <c r="AE12" s="8">
         <f>ROUND(24*(N(D12)-N(C12)+N(F12)-N(E12)+N(H12)-N(G12)+N(J12)-N(I12)+N(L12)-N(K12)+N(N12)-N(M12)+N(P12)-N(O12)+N(R12)-N(Q12)+N(T12)-N(S12)+N(V12)-N(U12)+N(X12)-N(W12)+N(Z12)-N(Y12)+N(AB12)-N(AA12)+N(AD12)-N(AC12)),2)</f>
         <v/>
       </c>
-      <c r="AF12" s="6" t="n">
+      <c r="AF12" s="5" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1476,57 +1488,53 @@
           <t>Cassiera</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="5" t="n">
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="5" t="n"/>
+      <c r="H13" s="5" t="n"/>
+      <c r="I13" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="J13" s="6" t="n">
         <v>0.875</v>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="K13" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="H13" s="5" t="n">
+      <c r="L13" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="M13" s="5" t="n"/>
+      <c r="N13" s="5" t="n"/>
+      <c r="O13" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="P13" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="Q13" s="5" t="n"/>
+      <c r="R13" s="5" t="n"/>
+      <c r="S13" s="5" t="n"/>
+      <c r="T13" s="5" t="n"/>
+      <c r="U13" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="I13" s="6" t="n"/>
-      <c r="J13" s="6" t="n"/>
-      <c r="K13" s="7" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7" t="n"/>
-      <c r="N13" s="7" t="n"/>
-      <c r="O13" s="5" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="P13" s="5" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="Q13" s="6" t="n"/>
-      <c r="R13" s="6" t="n"/>
-      <c r="S13" s="7" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="T13" s="7" t="n"/>
-      <c r="U13" s="7" t="n"/>
-      <c r="V13" s="7" t="n"/>
-      <c r="W13" s="5" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="X13" s="5" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Y13" s="5" t="n">
-        <v>0.5416666666666666</v>
-      </c>
-      <c r="Z13" s="5" t="n">
-        <v>0.7083333333333334</v>
+      <c r="V13" s="6" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="W13" s="5" t="n"/>
+      <c r="X13" s="5" t="n"/>
+      <c r="Y13" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="Z13" s="6" t="n">
+        <v>0.875</v>
       </c>
       <c r="AA13" s="7" t="inlineStr">
         <is>
@@ -1540,7 +1548,7 @@
         <f>ROUND(24*(N(D13)-N(C13)+N(F13)-N(E13)+N(H13)-N(G13)+N(J13)-N(I13)+N(L13)-N(K13)+N(N13)-N(M13)+N(P13)-N(O13)+N(R13)-N(Q13)+N(T13)-N(S13)+N(V13)-N(U13)+N(X13)-N(W13)+N(Z13)-N(Y13)+N(AB13)-N(AA13)+N(AD13)-N(AC13)),2)</f>
         <v/>
       </c>
-      <c r="AF13" s="6" t="n">
+      <c r="AF13" s="5" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1555,22 +1563,22 @@
           <t>Cassiera</t>
         </is>
       </c>
-      <c r="C14" s="5" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="D14" s="5" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="H14" s="7" t="n"/>
-      <c r="I14" s="7" t="n"/>
-      <c r="J14" s="7" t="n"/>
+      <c r="C14" s="6" t="n">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="n"/>
+      <c r="H14" s="5" t="n"/>
+      <c r="I14" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>0.75</v>
+      </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
@@ -1579,14 +1587,14 @@
       <c r="L14" s="7" t="n"/>
       <c r="M14" s="7" t="n"/>
       <c r="N14" s="7" t="n"/>
-      <c r="O14" s="5" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="P14" s="5" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="Q14" s="6" t="n"/>
-      <c r="R14" s="6" t="n"/>
+      <c r="O14" s="5" t="n"/>
+      <c r="P14" s="5" t="n"/>
+      <c r="Q14" s="6" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="R14" s="6" t="n">
+        <v>0.875</v>
+      </c>
       <c r="S14" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
@@ -1595,31 +1603,31 @@
       <c r="T14" s="7" t="n"/>
       <c r="U14" s="7" t="n"/>
       <c r="V14" s="7" t="n"/>
-      <c r="W14" s="5" t="n">
+      <c r="W14" s="5" t="n"/>
+      <c r="X14" s="5" t="n"/>
+      <c r="Y14" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="Z14" s="6" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="AA14" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="X14" s="5" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Y14" s="5" t="n">
+      <c r="AB14" s="6" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="Z14" s="5" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="AA14" s="6" t="n"/>
-      <c r="AB14" s="6" t="n"/>
-      <c r="AC14" s="5" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="AD14" s="5" t="n">
-        <v>0.875</v>
+      <c r="AC14" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="AD14" s="6" t="n">
+        <v>0.7916666666666666</v>
       </c>
       <c r="AE14" s="8">
         <f>ROUND(24*(N(D14)-N(C14)+N(F14)-N(E14)+N(H14)-N(G14)+N(J14)-N(I14)+N(L14)-N(K14)+N(N14)-N(M14)+N(P14)-N(O14)+N(R14)-N(Q14)+N(T14)-N(S14)+N(V14)-N(U14)+N(X14)-N(W14)+N(Z14)-N(Y14)+N(AB14)-N(AA14)+N(AD14)-N(AC14)),2)</f>
         <v/>
       </c>
-      <c r="AF14" s="6" t="n">
+      <c r="AF14" s="5" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1634,64 +1642,64 @@
           <t>Magazziniere</t>
         </is>
       </c>
-      <c r="C15" s="5" t="n">
+      <c r="C15" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D15" s="6" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="E15" s="5" t="n">
+      <c r="E15" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="F15" s="5" t="n">
+      <c r="F15" s="6" t="n">
         <v>0.75</v>
       </c>
-      <c r="G15" s="5" t="n">
+      <c r="G15" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="H15" s="6" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="I15" s="5" t="n">
+      <c r="I15" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="J15" s="5" t="n">
+      <c r="J15" s="6" t="n">
         <v>0.75</v>
       </c>
-      <c r="K15" s="5" t="n">
+      <c r="K15" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="L15" s="5" t="n">
+      <c r="L15" s="6" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="M15" s="5" t="n">
+      <c r="M15" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="N15" s="5" t="n">
+      <c r="N15" s="6" t="n">
         <v>0.75</v>
       </c>
-      <c r="O15" s="5" t="n">
+      <c r="O15" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="P15" s="5" t="n">
+      <c r="P15" s="6" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="Q15" s="5" t="n">
+      <c r="Q15" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="R15" s="5" t="n">
+      <c r="R15" s="6" t="n">
         <v>0.75</v>
       </c>
-      <c r="S15" s="5" t="n">
+      <c r="S15" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="T15" s="5" t="n">
+      <c r="T15" s="6" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="U15" s="5" t="n">
+      <c r="U15" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="V15" s="5" t="n">
+      <c r="V15" s="6" t="n">
         <v>0.75</v>
       </c>
       <c r="W15" s="7" t="inlineStr">
@@ -1714,7 +1722,7 @@
         <f>ROUND(24*(N(D15)-N(C15)+N(F15)-N(E15)+N(H15)-N(G15)+N(J15)-N(I15)+N(L15)-N(K15)+N(N15)-N(M15)+N(P15)-N(O15)+N(R15)-N(Q15)+N(T15)-N(S15)+N(V15)-N(U15)+N(X15)-N(W15)+N(Z15)-N(Y15)+N(AB15)-N(AA15)+N(AD15)-N(AC15)),2)</f>
         <v/>
       </c>
-      <c r="AF15" s="6" t="n">
+      <c r="AF15" s="5" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1735,49 +1743,57 @@
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>Laura Bruni: turni continuati di 6 ore, mai in apertura o chiusura. Luigi Diana: lun-ven 9-13 / 14-18, sabato e domenica a casa.</t>
+          <t>Orari delle casse (Benedetta, Martina, Debora, Giorgia) presi dal foglio del negozio; Luigi Diana lun-ven 9-13 / 14-18.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
+          <t>Sabato giornata intera per tutto il reparto; il terzo addetto di reparto messo di preferenza al pomeriggio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
           <t>Il foglio 'Copertura' conta ora per ora quante persone ci sono (si aggiorna da solo se modifichi gli orari).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="48">
+  <mergeCells count="46">
     <mergeCell ref="W4:X4"/>
     <mergeCell ref="S9:V9"/>
     <mergeCell ref="Y4:Z4"/>
     <mergeCell ref="K14:N14"/>
+    <mergeCell ref="C8:F8"/>
+    <mergeCell ref="O12:R12"/>
+    <mergeCell ref="O8:R8"/>
     <mergeCell ref="AA3:AD3"/>
-    <mergeCell ref="O11:R11"/>
-    <mergeCell ref="AA12:AD12"/>
+    <mergeCell ref="K7:N7"/>
+    <mergeCell ref="AA11:AD11"/>
     <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C13:F13"/>
     <mergeCell ref="E4:F4"/>
-    <mergeCell ref="K13:N13"/>
+    <mergeCell ref="G9:J9"/>
     <mergeCell ref="C3:F3"/>
     <mergeCell ref="K3:N3"/>
-    <mergeCell ref="G14:J14"/>
     <mergeCell ref="O3:R3"/>
-    <mergeCell ref="G12:J12"/>
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="O10:R10"/>
+    <mergeCell ref="G11:J11"/>
     <mergeCell ref="O4:P4"/>
-    <mergeCell ref="K9:N9"/>
+    <mergeCell ref="W15:Z15"/>
     <mergeCell ref="AA4:AB4"/>
     <mergeCell ref="Q4:R4"/>
-    <mergeCell ref="W15:Z15"/>
     <mergeCell ref="AC4:AD4"/>
     <mergeCell ref="AF3:AF5"/>
     <mergeCell ref="AA13:AD13"/>
     <mergeCell ref="S3:V3"/>
-    <mergeCell ref="S8:V8"/>
     <mergeCell ref="AE3:AE5"/>
-    <mergeCell ref="G7:J7"/>
     <mergeCell ref="AA6:AD6"/>
+    <mergeCell ref="S7:V7"/>
     <mergeCell ref="C10:F10"/>
     <mergeCell ref="AA15:AD15"/>
     <mergeCell ref="S14:V14"/>
@@ -1786,13 +1802,10 @@
     <mergeCell ref="I4:J4"/>
     <mergeCell ref="W3:Z3"/>
     <mergeCell ref="G3:J3"/>
-    <mergeCell ref="S13:V13"/>
-    <mergeCell ref="C12:F12"/>
     <mergeCell ref="A3:A5"/>
-    <mergeCell ref="K8:N8"/>
-    <mergeCell ref="C11:F11"/>
+    <mergeCell ref="K12:N12"/>
     <mergeCell ref="K4:L4"/>
-    <mergeCell ref="AA7:AD7"/>
+    <mergeCell ref="W12:Z12"/>
     <mergeCell ref="M4:N4"/>
     <mergeCell ref="S4:T4"/>
     <mergeCell ref="U4:V4"/>
@@ -1913,51 +1926,51 @@
           <t>lunedì 12 ottobre 2026</t>
         </is>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(9,30,0))*(Orari!$D$6:$D$15&gt;TIME(9,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(9,30,0))*(Orari!$F$6:$F$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(10,30,0))*(Orari!$D$6:$D$15&gt;TIME(10,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(10,30,0))*(Orari!$F$6:$F$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(11,30,0))*(Orari!$D$6:$D$15&gt;TIME(11,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(11,30,0))*(Orari!$F$6:$F$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(12,30,0))*(Orari!$D$6:$D$15&gt;TIME(12,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(12,30,0))*(Orari!$F$6:$F$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(13,30,0))*(Orari!$D$6:$D$15&gt;TIME(13,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(13,30,0))*(Orari!$F$6:$F$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(14,30,0))*(Orari!$D$6:$D$15&gt;TIME(14,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(14,30,0))*(Orari!$F$6:$F$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H5" s="6">
+      <c r="H5" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(15,30,0))*(Orari!$D$6:$D$15&gt;TIME(15,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(15,30,0))*(Orari!$F$6:$F$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I5" s="6">
+      <c r="I5" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(16,30,0))*(Orari!$D$6:$D$15&gt;TIME(16,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(16,30,0))*(Orari!$F$6:$F$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J5" s="6">
+      <c r="J5" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(17,30,0))*(Orari!$D$6:$D$15&gt;TIME(17,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(17,30,0))*(Orari!$F$6:$F$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K5" s="6">
+      <c r="K5" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(18,30,0))*(Orari!$D$6:$D$15&gt;TIME(18,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(18,30,0))*(Orari!$F$6:$F$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L5" s="6">
+      <c r="L5" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(19,30,0))*(Orari!$D$6:$D$15&gt;TIME(19,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(19,30,0))*(Orari!$F$6:$F$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M5" s="6">
+      <c r="M5" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(20,30,0))*(Orari!$D$6:$D$15&gt;TIME(20,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(20,30,0))*(Orari!$F$6:$F$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -1968,51 +1981,51 @@
           <t>martedì 13 ottobre 2026</t>
         </is>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(9,30,0))*(Orari!$H$6:$H$15&gt;TIME(9,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(9,30,0))*(Orari!$J$6:$J$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(10,30,0))*(Orari!$H$6:$H$15&gt;TIME(10,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(10,30,0))*(Orari!$J$6:$J$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(11,30,0))*(Orari!$H$6:$H$15&gt;TIME(11,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(11,30,0))*(Orari!$J$6:$J$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(12,30,0))*(Orari!$H$6:$H$15&gt;TIME(12,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(12,30,0))*(Orari!$J$6:$J$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(13,30,0))*(Orari!$H$6:$H$15&gt;TIME(13,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(13,30,0))*(Orari!$J$6:$J$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G6" s="6">
+      <c r="G6" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(14,30,0))*(Orari!$H$6:$H$15&gt;TIME(14,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(14,30,0))*(Orari!$J$6:$J$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(15,30,0))*(Orari!$H$6:$H$15&gt;TIME(15,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(15,30,0))*(Orari!$J$6:$J$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I6" s="6">
+      <c r="I6" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(16,30,0))*(Orari!$H$6:$H$15&gt;TIME(16,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(16,30,0))*(Orari!$J$6:$J$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J6" s="6">
+      <c r="J6" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(17,30,0))*(Orari!$H$6:$H$15&gt;TIME(17,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(17,30,0))*(Orari!$J$6:$J$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K6" s="6">
+      <c r="K6" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(18,30,0))*(Orari!$H$6:$H$15&gt;TIME(18,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(18,30,0))*(Orari!$J$6:$J$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L6" s="6">
+      <c r="L6" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(19,30,0))*(Orari!$H$6:$H$15&gt;TIME(19,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(19,30,0))*(Orari!$J$6:$J$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M6" s="6">
+      <c r="M6" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(20,30,0))*(Orari!$H$6:$H$15&gt;TIME(20,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(20,30,0))*(Orari!$J$6:$J$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2023,51 +2036,51 @@
           <t>mercoledì 14 ottobre 2026</t>
         </is>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(9,30,0))*(Orari!$L$6:$L$15&gt;TIME(9,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(9,30,0))*(Orari!$N$6:$N$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(10,30,0))*(Orari!$L$6:$L$15&gt;TIME(10,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(10,30,0))*(Orari!$N$6:$N$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(11,30,0))*(Orari!$L$6:$L$15&gt;TIME(11,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(11,30,0))*(Orari!$N$6:$N$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(12,30,0))*(Orari!$L$6:$L$15&gt;TIME(12,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(12,30,0))*(Orari!$N$6:$N$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(13,30,0))*(Orari!$L$6:$L$15&gt;TIME(13,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(13,30,0))*(Orari!$N$6:$N$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(14,30,0))*(Orari!$L$6:$L$15&gt;TIME(14,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(14,30,0))*(Orari!$N$6:$N$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(15,30,0))*(Orari!$L$6:$L$15&gt;TIME(15,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(15,30,0))*(Orari!$N$6:$N$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I7" s="6">
+      <c r="I7" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(16,30,0))*(Orari!$L$6:$L$15&gt;TIME(16,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(16,30,0))*(Orari!$N$6:$N$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J7" s="6">
+      <c r="J7" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(17,30,0))*(Orari!$L$6:$L$15&gt;TIME(17,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(17,30,0))*(Orari!$N$6:$N$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K7" s="6">
+      <c r="K7" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(18,30,0))*(Orari!$L$6:$L$15&gt;TIME(18,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(18,30,0))*(Orari!$N$6:$N$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L7" s="6">
+      <c r="L7" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(19,30,0))*(Orari!$L$6:$L$15&gt;TIME(19,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(19,30,0))*(Orari!$N$6:$N$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M7" s="6">
+      <c r="M7" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(20,30,0))*(Orari!$L$6:$L$15&gt;TIME(20,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(20,30,0))*(Orari!$N$6:$N$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2078,51 +2091,51 @@
           <t>giovedì 15 ottobre 2026</t>
         </is>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(9,30,0))*(Orari!$P$6:$P$15&gt;TIME(9,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(9,30,0))*(Orari!$R$6:$R$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(10,30,0))*(Orari!$P$6:$P$15&gt;TIME(10,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(10,30,0))*(Orari!$R$6:$R$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(11,30,0))*(Orari!$P$6:$P$15&gt;TIME(11,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(11,30,0))*(Orari!$R$6:$R$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(12,30,0))*(Orari!$P$6:$P$15&gt;TIME(12,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(12,30,0))*(Orari!$R$6:$R$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(13,30,0))*(Orari!$P$6:$P$15&gt;TIME(13,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(13,30,0))*(Orari!$R$6:$R$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(14,30,0))*(Orari!$P$6:$P$15&gt;TIME(14,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(14,30,0))*(Orari!$R$6:$R$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(15,30,0))*(Orari!$P$6:$P$15&gt;TIME(15,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(15,30,0))*(Orari!$R$6:$R$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I8" s="6">
+      <c r="I8" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(16,30,0))*(Orari!$P$6:$P$15&gt;TIME(16,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(16,30,0))*(Orari!$R$6:$R$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J8" s="6">
+      <c r="J8" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(17,30,0))*(Orari!$P$6:$P$15&gt;TIME(17,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(17,30,0))*(Orari!$R$6:$R$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K8" s="6">
+      <c r="K8" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(18,30,0))*(Orari!$P$6:$P$15&gt;TIME(18,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(18,30,0))*(Orari!$R$6:$R$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L8" s="6">
+      <c r="L8" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(19,30,0))*(Orari!$P$6:$P$15&gt;TIME(19,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(19,30,0))*(Orari!$R$6:$R$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M8" s="6">
+      <c r="M8" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(20,30,0))*(Orari!$P$6:$P$15&gt;TIME(20,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(20,30,0))*(Orari!$R$6:$R$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2133,51 +2146,51 @@
           <t>venerdì 16 ottobre 2026</t>
         </is>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(9,30,0))*(Orari!$T$6:$T$15&gt;TIME(9,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(9,30,0))*(Orari!$V$6:$V$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(10,30,0))*(Orari!$T$6:$T$15&gt;TIME(10,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(10,30,0))*(Orari!$V$6:$V$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(11,30,0))*(Orari!$T$6:$T$15&gt;TIME(11,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(11,30,0))*(Orari!$V$6:$V$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(12,30,0))*(Orari!$T$6:$T$15&gt;TIME(12,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(12,30,0))*(Orari!$V$6:$V$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(13,30,0))*(Orari!$T$6:$T$15&gt;TIME(13,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(13,30,0))*(Orari!$V$6:$V$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G9" s="6">
+      <c r="G9" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(14,30,0))*(Orari!$T$6:$T$15&gt;TIME(14,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(14,30,0))*(Orari!$V$6:$V$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H9" s="6">
+      <c r="H9" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(15,30,0))*(Orari!$T$6:$T$15&gt;TIME(15,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(15,30,0))*(Orari!$V$6:$V$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I9" s="6">
+      <c r="I9" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(16,30,0))*(Orari!$T$6:$T$15&gt;TIME(16,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(16,30,0))*(Orari!$V$6:$V$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J9" s="6">
+      <c r="J9" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(17,30,0))*(Orari!$T$6:$T$15&gt;TIME(17,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(17,30,0))*(Orari!$V$6:$V$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K9" s="6">
+      <c r="K9" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(18,30,0))*(Orari!$T$6:$T$15&gt;TIME(18,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(18,30,0))*(Orari!$V$6:$V$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L9" s="6">
+      <c r="L9" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(19,30,0))*(Orari!$T$6:$T$15&gt;TIME(19,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(19,30,0))*(Orari!$V$6:$V$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M9" s="6">
+      <c r="M9" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(20,30,0))*(Orari!$T$6:$T$15&gt;TIME(20,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(20,30,0))*(Orari!$V$6:$V$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2188,51 +2201,51 @@
           <t>sabato 17 ottobre 2026</t>
         </is>
       </c>
-      <c r="B10" s="6">
+      <c r="B10" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(9,30,0))*(Orari!$X$6:$X$15&gt;TIME(9,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(9,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(10,30,0))*(Orari!$X$6:$X$15&gt;TIME(10,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(10,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(11,30,0))*(Orari!$X$6:$X$15&gt;TIME(11,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(11,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(12,30,0))*(Orari!$X$6:$X$15&gt;TIME(12,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(12,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(13,30,0))*(Orari!$X$6:$X$15&gt;TIME(13,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(13,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G10" s="6">
+      <c r="G10" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(14,30,0))*(Orari!$X$6:$X$15&gt;TIME(14,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(14,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H10" s="6">
+      <c r="H10" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(15,30,0))*(Orari!$X$6:$X$15&gt;TIME(15,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(15,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I10" s="6">
+      <c r="I10" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(16,30,0))*(Orari!$X$6:$X$15&gt;TIME(16,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(16,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J10" s="6">
+      <c r="J10" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(17,30,0))*(Orari!$X$6:$X$15&gt;TIME(17,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(17,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K10" s="6">
+      <c r="K10" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(18,30,0))*(Orari!$X$6:$X$15&gt;TIME(18,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(18,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L10" s="6">
+      <c r="L10" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(19,30,0))*(Orari!$X$6:$X$15&gt;TIME(19,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(19,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M10" s="6">
+      <c r="M10" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(20,30,0))*(Orari!$X$6:$X$15&gt;TIME(20,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(20,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2243,51 +2256,51 @@
           <t>domenica 18 ottobre 2026</t>
         </is>
       </c>
-      <c r="B11" s="6">
+      <c r="B11" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(9,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(9,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(9,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(10,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(10,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(10,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(11,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(11,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(11,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(12,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(12,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(12,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(13,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(13,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(13,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G11" s="6">
+      <c r="G11" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(14,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(14,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(14,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H11" s="6">
+      <c r="H11" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(15,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(15,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(15,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I11" s="6">
+      <c r="I11" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(16,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(16,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(16,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J11" s="6">
+      <c r="J11" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(17,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(17,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(17,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K11" s="6">
+      <c r="K11" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(18,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(18,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(18,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L11" s="6">
+      <c r="L11" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(19,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(19,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(19,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M11" s="6">
+      <c r="M11" s="5">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(20,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(20,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(20,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2372,51 +2385,51 @@
           <t>lunedì 12 ottobre 2026</t>
         </is>
       </c>
-      <c r="B15" s="6">
+      <c r="B15" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(9,30,0))*(Orari!$D$6:$D$15&gt;TIME(9,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(9,30,0))*(Orari!$F$6:$F$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C15" s="6">
+      <c r="C15" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(10,30,0))*(Orari!$D$6:$D$15&gt;TIME(10,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(10,30,0))*(Orari!$F$6:$F$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(11,30,0))*(Orari!$D$6:$D$15&gt;TIME(11,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(11,30,0))*(Orari!$F$6:$F$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(12,30,0))*(Orari!$D$6:$D$15&gt;TIME(12,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(12,30,0))*(Orari!$F$6:$F$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F15" s="6">
+      <c r="F15" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(13,30,0))*(Orari!$D$6:$D$15&gt;TIME(13,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(13,30,0))*(Orari!$F$6:$F$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G15" s="6">
+      <c r="G15" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(14,30,0))*(Orari!$D$6:$D$15&gt;TIME(14,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(14,30,0))*(Orari!$F$6:$F$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H15" s="6">
+      <c r="H15" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(15,30,0))*(Orari!$D$6:$D$15&gt;TIME(15,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(15,30,0))*(Orari!$F$6:$F$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I15" s="6">
+      <c r="I15" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(16,30,0))*(Orari!$D$6:$D$15&gt;TIME(16,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(16,30,0))*(Orari!$F$6:$F$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J15" s="6">
+      <c r="J15" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(17,30,0))*(Orari!$D$6:$D$15&gt;TIME(17,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(17,30,0))*(Orari!$F$6:$F$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K15" s="6">
+      <c r="K15" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(18,30,0))*(Orari!$D$6:$D$15&gt;TIME(18,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(18,30,0))*(Orari!$F$6:$F$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L15" s="6">
+      <c r="L15" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(19,30,0))*(Orari!$D$6:$D$15&gt;TIME(19,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(19,30,0))*(Orari!$F$6:$F$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M15" s="6">
+      <c r="M15" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(20,30,0))*(Orari!$D$6:$D$15&gt;TIME(20,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(20,30,0))*(Orari!$F$6:$F$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2427,51 +2440,51 @@
           <t>martedì 13 ottobre 2026</t>
         </is>
       </c>
-      <c r="B16" s="6">
+      <c r="B16" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(9,30,0))*(Orari!$H$6:$H$15&gt;TIME(9,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(9,30,0))*(Orari!$J$6:$J$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C16" s="6">
+      <c r="C16" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(10,30,0))*(Orari!$H$6:$H$15&gt;TIME(10,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(10,30,0))*(Orari!$J$6:$J$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(11,30,0))*(Orari!$H$6:$H$15&gt;TIME(11,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(11,30,0))*(Orari!$J$6:$J$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E16" s="6">
+      <c r="E16" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(12,30,0))*(Orari!$H$6:$H$15&gt;TIME(12,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(12,30,0))*(Orari!$J$6:$J$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F16" s="6">
+      <c r="F16" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(13,30,0))*(Orari!$H$6:$H$15&gt;TIME(13,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(13,30,0))*(Orari!$J$6:$J$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G16" s="6">
+      <c r="G16" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(14,30,0))*(Orari!$H$6:$H$15&gt;TIME(14,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(14,30,0))*(Orari!$J$6:$J$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H16" s="6">
+      <c r="H16" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(15,30,0))*(Orari!$H$6:$H$15&gt;TIME(15,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(15,30,0))*(Orari!$J$6:$J$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I16" s="6">
+      <c r="I16" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(16,30,0))*(Orari!$H$6:$H$15&gt;TIME(16,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(16,30,0))*(Orari!$J$6:$J$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J16" s="6">
+      <c r="J16" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(17,30,0))*(Orari!$H$6:$H$15&gt;TIME(17,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(17,30,0))*(Orari!$J$6:$J$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K16" s="6">
+      <c r="K16" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(18,30,0))*(Orari!$H$6:$H$15&gt;TIME(18,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(18,30,0))*(Orari!$J$6:$J$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L16" s="6">
+      <c r="L16" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(19,30,0))*(Orari!$H$6:$H$15&gt;TIME(19,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(19,30,0))*(Orari!$J$6:$J$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M16" s="6">
+      <c r="M16" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(20,30,0))*(Orari!$H$6:$H$15&gt;TIME(20,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(20,30,0))*(Orari!$J$6:$J$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2482,51 +2495,51 @@
           <t>mercoledì 14 ottobre 2026</t>
         </is>
       </c>
-      <c r="B17" s="6">
+      <c r="B17" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(9,30,0))*(Orari!$L$6:$L$15&gt;TIME(9,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(9,30,0))*(Orari!$N$6:$N$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C17" s="6">
+      <c r="C17" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(10,30,0))*(Orari!$L$6:$L$15&gt;TIME(10,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(10,30,0))*(Orari!$N$6:$N$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(11,30,0))*(Orari!$L$6:$L$15&gt;TIME(11,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(11,30,0))*(Orari!$N$6:$N$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(12,30,0))*(Orari!$L$6:$L$15&gt;TIME(12,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(12,30,0))*(Orari!$N$6:$N$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F17" s="6">
+      <c r="F17" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(13,30,0))*(Orari!$L$6:$L$15&gt;TIME(13,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(13,30,0))*(Orari!$N$6:$N$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G17" s="6">
+      <c r="G17" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(14,30,0))*(Orari!$L$6:$L$15&gt;TIME(14,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(14,30,0))*(Orari!$N$6:$N$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H17" s="6">
+      <c r="H17" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(15,30,0))*(Orari!$L$6:$L$15&gt;TIME(15,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(15,30,0))*(Orari!$N$6:$N$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I17" s="6">
+      <c r="I17" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(16,30,0))*(Orari!$L$6:$L$15&gt;TIME(16,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(16,30,0))*(Orari!$N$6:$N$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J17" s="6">
+      <c r="J17" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(17,30,0))*(Orari!$L$6:$L$15&gt;TIME(17,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(17,30,0))*(Orari!$N$6:$N$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K17" s="6">
+      <c r="K17" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(18,30,0))*(Orari!$L$6:$L$15&gt;TIME(18,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(18,30,0))*(Orari!$N$6:$N$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L17" s="6">
+      <c r="L17" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(19,30,0))*(Orari!$L$6:$L$15&gt;TIME(19,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(19,30,0))*(Orari!$N$6:$N$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M17" s="6">
+      <c r="M17" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(20,30,0))*(Orari!$L$6:$L$15&gt;TIME(20,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(20,30,0))*(Orari!$N$6:$N$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2537,51 +2550,51 @@
           <t>giovedì 15 ottobre 2026</t>
         </is>
       </c>
-      <c r="B18" s="6">
+      <c r="B18" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(9,30,0))*(Orari!$P$6:$P$15&gt;TIME(9,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(9,30,0))*(Orari!$R$6:$R$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C18" s="6">
+      <c r="C18" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(10,30,0))*(Orari!$P$6:$P$15&gt;TIME(10,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(10,30,0))*(Orari!$R$6:$R$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(11,30,0))*(Orari!$P$6:$P$15&gt;TIME(11,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(11,30,0))*(Orari!$R$6:$R$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(12,30,0))*(Orari!$P$6:$P$15&gt;TIME(12,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(12,30,0))*(Orari!$R$6:$R$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F18" s="6">
+      <c r="F18" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(13,30,0))*(Orari!$P$6:$P$15&gt;TIME(13,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(13,30,0))*(Orari!$R$6:$R$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G18" s="6">
+      <c r="G18" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(14,30,0))*(Orari!$P$6:$P$15&gt;TIME(14,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(14,30,0))*(Orari!$R$6:$R$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H18" s="6">
+      <c r="H18" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(15,30,0))*(Orari!$P$6:$P$15&gt;TIME(15,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(15,30,0))*(Orari!$R$6:$R$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I18" s="6">
+      <c r="I18" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(16,30,0))*(Orari!$P$6:$P$15&gt;TIME(16,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(16,30,0))*(Orari!$R$6:$R$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J18" s="6">
+      <c r="J18" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(17,30,0))*(Orari!$P$6:$P$15&gt;TIME(17,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(17,30,0))*(Orari!$R$6:$R$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K18" s="6">
+      <c r="K18" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(18,30,0))*(Orari!$P$6:$P$15&gt;TIME(18,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(18,30,0))*(Orari!$R$6:$R$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L18" s="6">
+      <c r="L18" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(19,30,0))*(Orari!$P$6:$P$15&gt;TIME(19,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(19,30,0))*(Orari!$R$6:$R$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M18" s="6">
+      <c r="M18" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(20,30,0))*(Orari!$P$6:$P$15&gt;TIME(20,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(20,30,0))*(Orari!$R$6:$R$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2592,51 +2605,51 @@
           <t>venerdì 16 ottobre 2026</t>
         </is>
       </c>
-      <c r="B19" s="6">
+      <c r="B19" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(9,30,0))*(Orari!$T$6:$T$15&gt;TIME(9,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(9,30,0))*(Orari!$V$6:$V$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C19" s="6">
+      <c r="C19" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(10,30,0))*(Orari!$T$6:$T$15&gt;TIME(10,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(10,30,0))*(Orari!$V$6:$V$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(11,30,0))*(Orari!$T$6:$T$15&gt;TIME(11,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(11,30,0))*(Orari!$V$6:$V$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E19" s="6">
+      <c r="E19" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(12,30,0))*(Orari!$T$6:$T$15&gt;TIME(12,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(12,30,0))*(Orari!$V$6:$V$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F19" s="6">
+      <c r="F19" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(13,30,0))*(Orari!$T$6:$T$15&gt;TIME(13,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(13,30,0))*(Orari!$V$6:$V$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G19" s="6">
+      <c r="G19" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(14,30,0))*(Orari!$T$6:$T$15&gt;TIME(14,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(14,30,0))*(Orari!$V$6:$V$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H19" s="6">
+      <c r="H19" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(15,30,0))*(Orari!$T$6:$T$15&gt;TIME(15,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(15,30,0))*(Orari!$V$6:$V$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I19" s="6">
+      <c r="I19" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(16,30,0))*(Orari!$T$6:$T$15&gt;TIME(16,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(16,30,0))*(Orari!$V$6:$V$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J19" s="6">
+      <c r="J19" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(17,30,0))*(Orari!$T$6:$T$15&gt;TIME(17,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(17,30,0))*(Orari!$V$6:$V$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K19" s="6">
+      <c r="K19" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(18,30,0))*(Orari!$T$6:$T$15&gt;TIME(18,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(18,30,0))*(Orari!$V$6:$V$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L19" s="6">
+      <c r="L19" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(19,30,0))*(Orari!$T$6:$T$15&gt;TIME(19,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(19,30,0))*(Orari!$V$6:$V$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M19" s="6">
+      <c r="M19" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(20,30,0))*(Orari!$T$6:$T$15&gt;TIME(20,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(20,30,0))*(Orari!$V$6:$V$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2647,51 +2660,51 @@
           <t>sabato 17 ottobre 2026</t>
         </is>
       </c>
-      <c r="B20" s="6">
+      <c r="B20" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(9,30,0))*(Orari!$X$6:$X$15&gt;TIME(9,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(9,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C20" s="6">
+      <c r="C20" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(10,30,0))*(Orari!$X$6:$X$15&gt;TIME(10,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(10,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D20" s="6">
+      <c r="D20" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(11,30,0))*(Orari!$X$6:$X$15&gt;TIME(11,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(11,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E20" s="6">
+      <c r="E20" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(12,30,0))*(Orari!$X$6:$X$15&gt;TIME(12,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(12,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F20" s="6">
+      <c r="F20" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(13,30,0))*(Orari!$X$6:$X$15&gt;TIME(13,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(13,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G20" s="6">
+      <c r="G20" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(14,30,0))*(Orari!$X$6:$X$15&gt;TIME(14,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(14,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H20" s="6">
+      <c r="H20" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(15,30,0))*(Orari!$X$6:$X$15&gt;TIME(15,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(15,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I20" s="6">
+      <c r="I20" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(16,30,0))*(Orari!$X$6:$X$15&gt;TIME(16,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(16,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J20" s="6">
+      <c r="J20" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(17,30,0))*(Orari!$X$6:$X$15&gt;TIME(17,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(17,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K20" s="6">
+      <c r="K20" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(18,30,0))*(Orari!$X$6:$X$15&gt;TIME(18,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(18,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L20" s="6">
+      <c r="L20" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(19,30,0))*(Orari!$X$6:$X$15&gt;TIME(19,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(19,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M20" s="6">
+      <c r="M20" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(20,30,0))*(Orari!$X$6:$X$15&gt;TIME(20,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(20,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2702,51 +2715,51 @@
           <t>domenica 18 ottobre 2026</t>
         </is>
       </c>
-      <c r="B21" s="6">
+      <c r="B21" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(9,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(9,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(9,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(10,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(10,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(10,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(11,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(11,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(11,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E21" s="6">
+      <c r="E21" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(12,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(12,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(12,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F21" s="6">
+      <c r="F21" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(13,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(13,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(13,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G21" s="6">
+      <c r="G21" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(14,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(14,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(14,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H21" s="6">
+      <c r="H21" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(15,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(15,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(15,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I21" s="6">
+      <c r="I21" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(16,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(16,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(16,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J21" s="6">
+      <c r="J21" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(17,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(17,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(17,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K21" s="6">
+      <c r="K21" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(18,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(18,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(18,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L21" s="6">
+      <c r="L21" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(19,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(19,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(19,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M21" s="6">
+      <c r="M21" s="5">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(20,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(20,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(20,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2831,51 +2844,51 @@
           <t>lunedì 12 ottobre 2026</t>
         </is>
       </c>
-      <c r="B25" s="6">
+      <c r="B25" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(9,30,0))*(Orari!$D$6:$D$15&gt;TIME(9,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(9,30,0))*(Orari!$F$6:$F$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C25" s="6">
+      <c r="C25" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(10,30,0))*(Orari!$D$6:$D$15&gt;TIME(10,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(10,30,0))*(Orari!$F$6:$F$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D25" s="6">
+      <c r="D25" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(11,30,0))*(Orari!$D$6:$D$15&gt;TIME(11,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(11,30,0))*(Orari!$F$6:$F$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E25" s="6">
+      <c r="E25" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(12,30,0))*(Orari!$D$6:$D$15&gt;TIME(12,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(12,30,0))*(Orari!$F$6:$F$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F25" s="6">
+      <c r="F25" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(13,30,0))*(Orari!$D$6:$D$15&gt;TIME(13,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(13,30,0))*(Orari!$F$6:$F$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G25" s="6">
+      <c r="G25" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(14,30,0))*(Orari!$D$6:$D$15&gt;TIME(14,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(14,30,0))*(Orari!$F$6:$F$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H25" s="6">
+      <c r="H25" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(15,30,0))*(Orari!$D$6:$D$15&gt;TIME(15,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(15,30,0))*(Orari!$F$6:$F$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I25" s="6">
+      <c r="I25" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(16,30,0))*(Orari!$D$6:$D$15&gt;TIME(16,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(16,30,0))*(Orari!$F$6:$F$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J25" s="6">
+      <c r="J25" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(17,30,0))*(Orari!$D$6:$D$15&gt;TIME(17,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(17,30,0))*(Orari!$F$6:$F$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K25" s="6">
+      <c r="K25" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(18,30,0))*(Orari!$D$6:$D$15&gt;TIME(18,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(18,30,0))*(Orari!$F$6:$F$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L25" s="6">
+      <c r="L25" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(19,30,0))*(Orari!$D$6:$D$15&gt;TIME(19,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(19,30,0))*(Orari!$F$6:$F$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M25" s="6">
+      <c r="M25" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(20,30,0))*(Orari!$D$6:$D$15&gt;TIME(20,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(20,30,0))*(Orari!$F$6:$F$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2886,51 +2899,51 @@
           <t>martedì 13 ottobre 2026</t>
         </is>
       </c>
-      <c r="B26" s="6">
+      <c r="B26" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(9,30,0))*(Orari!$H$6:$H$15&gt;TIME(9,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(9,30,0))*(Orari!$J$6:$J$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C26" s="6">
+      <c r="C26" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(10,30,0))*(Orari!$H$6:$H$15&gt;TIME(10,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(10,30,0))*(Orari!$J$6:$J$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D26" s="6">
+      <c r="D26" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(11,30,0))*(Orari!$H$6:$H$15&gt;TIME(11,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(11,30,0))*(Orari!$J$6:$J$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E26" s="6">
+      <c r="E26" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(12,30,0))*(Orari!$H$6:$H$15&gt;TIME(12,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(12,30,0))*(Orari!$J$6:$J$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F26" s="6">
+      <c r="F26" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(13,30,0))*(Orari!$H$6:$H$15&gt;TIME(13,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(13,30,0))*(Orari!$J$6:$J$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G26" s="6">
+      <c r="G26" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(14,30,0))*(Orari!$H$6:$H$15&gt;TIME(14,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(14,30,0))*(Orari!$J$6:$J$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H26" s="6">
+      <c r="H26" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(15,30,0))*(Orari!$H$6:$H$15&gt;TIME(15,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(15,30,0))*(Orari!$J$6:$J$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I26" s="6">
+      <c r="I26" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(16,30,0))*(Orari!$H$6:$H$15&gt;TIME(16,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(16,30,0))*(Orari!$J$6:$J$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J26" s="6">
+      <c r="J26" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(17,30,0))*(Orari!$H$6:$H$15&gt;TIME(17,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(17,30,0))*(Orari!$J$6:$J$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K26" s="6">
+      <c r="K26" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(18,30,0))*(Orari!$H$6:$H$15&gt;TIME(18,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(18,30,0))*(Orari!$J$6:$J$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L26" s="6">
+      <c r="L26" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(19,30,0))*(Orari!$H$6:$H$15&gt;TIME(19,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(19,30,0))*(Orari!$J$6:$J$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M26" s="6">
+      <c r="M26" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(20,30,0))*(Orari!$H$6:$H$15&gt;TIME(20,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(20,30,0))*(Orari!$J$6:$J$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2941,51 +2954,51 @@
           <t>mercoledì 14 ottobre 2026</t>
         </is>
       </c>
-      <c r="B27" s="6">
+      <c r="B27" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(9,30,0))*(Orari!$L$6:$L$15&gt;TIME(9,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(9,30,0))*(Orari!$N$6:$N$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C27" s="6">
+      <c r="C27" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(10,30,0))*(Orari!$L$6:$L$15&gt;TIME(10,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(10,30,0))*(Orari!$N$6:$N$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D27" s="6">
+      <c r="D27" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(11,30,0))*(Orari!$L$6:$L$15&gt;TIME(11,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(11,30,0))*(Orari!$N$6:$N$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E27" s="6">
+      <c r="E27" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(12,30,0))*(Orari!$L$6:$L$15&gt;TIME(12,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(12,30,0))*(Orari!$N$6:$N$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F27" s="6">
+      <c r="F27" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(13,30,0))*(Orari!$L$6:$L$15&gt;TIME(13,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(13,30,0))*(Orari!$N$6:$N$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G27" s="6">
+      <c r="G27" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(14,30,0))*(Orari!$L$6:$L$15&gt;TIME(14,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(14,30,0))*(Orari!$N$6:$N$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H27" s="6">
+      <c r="H27" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(15,30,0))*(Orari!$L$6:$L$15&gt;TIME(15,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(15,30,0))*(Orari!$N$6:$N$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I27" s="6">
+      <c r="I27" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(16,30,0))*(Orari!$L$6:$L$15&gt;TIME(16,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(16,30,0))*(Orari!$N$6:$N$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J27" s="6">
+      <c r="J27" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(17,30,0))*(Orari!$L$6:$L$15&gt;TIME(17,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(17,30,0))*(Orari!$N$6:$N$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K27" s="6">
+      <c r="K27" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(18,30,0))*(Orari!$L$6:$L$15&gt;TIME(18,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(18,30,0))*(Orari!$N$6:$N$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L27" s="6">
+      <c r="L27" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(19,30,0))*(Orari!$L$6:$L$15&gt;TIME(19,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(19,30,0))*(Orari!$N$6:$N$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M27" s="6">
+      <c r="M27" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(20,30,0))*(Orari!$L$6:$L$15&gt;TIME(20,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(20,30,0))*(Orari!$N$6:$N$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2996,51 +3009,51 @@
           <t>giovedì 15 ottobre 2026</t>
         </is>
       </c>
-      <c r="B28" s="6">
+      <c r="B28" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(9,30,0))*(Orari!$P$6:$P$15&gt;TIME(9,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(9,30,0))*(Orari!$R$6:$R$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C28" s="6">
+      <c r="C28" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(10,30,0))*(Orari!$P$6:$P$15&gt;TIME(10,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(10,30,0))*(Orari!$R$6:$R$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D28" s="6">
+      <c r="D28" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(11,30,0))*(Orari!$P$6:$P$15&gt;TIME(11,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(11,30,0))*(Orari!$R$6:$R$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E28" s="6">
+      <c r="E28" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(12,30,0))*(Orari!$P$6:$P$15&gt;TIME(12,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(12,30,0))*(Orari!$R$6:$R$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F28" s="6">
+      <c r="F28" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(13,30,0))*(Orari!$P$6:$P$15&gt;TIME(13,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(13,30,0))*(Orari!$R$6:$R$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G28" s="6">
+      <c r="G28" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(14,30,0))*(Orari!$P$6:$P$15&gt;TIME(14,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(14,30,0))*(Orari!$R$6:$R$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H28" s="6">
+      <c r="H28" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(15,30,0))*(Orari!$P$6:$P$15&gt;TIME(15,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(15,30,0))*(Orari!$R$6:$R$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I28" s="6">
+      <c r="I28" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(16,30,0))*(Orari!$P$6:$P$15&gt;TIME(16,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(16,30,0))*(Orari!$R$6:$R$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J28" s="6">
+      <c r="J28" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(17,30,0))*(Orari!$P$6:$P$15&gt;TIME(17,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(17,30,0))*(Orari!$R$6:$R$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K28" s="6">
+      <c r="K28" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(18,30,0))*(Orari!$P$6:$P$15&gt;TIME(18,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(18,30,0))*(Orari!$R$6:$R$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L28" s="6">
+      <c r="L28" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(19,30,0))*(Orari!$P$6:$P$15&gt;TIME(19,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(19,30,0))*(Orari!$R$6:$R$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M28" s="6">
+      <c r="M28" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(20,30,0))*(Orari!$P$6:$P$15&gt;TIME(20,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(20,30,0))*(Orari!$R$6:$R$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -3051,51 +3064,51 @@
           <t>venerdì 16 ottobre 2026</t>
         </is>
       </c>
-      <c r="B29" s="6">
+      <c r="B29" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(9,30,0))*(Orari!$T$6:$T$15&gt;TIME(9,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(9,30,0))*(Orari!$V$6:$V$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C29" s="6">
+      <c r="C29" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(10,30,0))*(Orari!$T$6:$T$15&gt;TIME(10,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(10,30,0))*(Orari!$V$6:$V$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D29" s="6">
+      <c r="D29" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(11,30,0))*(Orari!$T$6:$T$15&gt;TIME(11,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(11,30,0))*(Orari!$V$6:$V$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E29" s="6">
+      <c r="E29" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(12,30,0))*(Orari!$T$6:$T$15&gt;TIME(12,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(12,30,0))*(Orari!$V$6:$V$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F29" s="6">
+      <c r="F29" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(13,30,0))*(Orari!$T$6:$T$15&gt;TIME(13,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(13,30,0))*(Orari!$V$6:$V$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G29" s="6">
+      <c r="G29" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(14,30,0))*(Orari!$T$6:$T$15&gt;TIME(14,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(14,30,0))*(Orari!$V$6:$V$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H29" s="6">
+      <c r="H29" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(15,30,0))*(Orari!$T$6:$T$15&gt;TIME(15,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(15,30,0))*(Orari!$V$6:$V$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I29" s="6">
+      <c r="I29" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(16,30,0))*(Orari!$T$6:$T$15&gt;TIME(16,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(16,30,0))*(Orari!$V$6:$V$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J29" s="6">
+      <c r="J29" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(17,30,0))*(Orari!$T$6:$T$15&gt;TIME(17,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(17,30,0))*(Orari!$V$6:$V$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K29" s="6">
+      <c r="K29" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(18,30,0))*(Orari!$T$6:$T$15&gt;TIME(18,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(18,30,0))*(Orari!$V$6:$V$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L29" s="6">
+      <c r="L29" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(19,30,0))*(Orari!$T$6:$T$15&gt;TIME(19,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(19,30,0))*(Orari!$V$6:$V$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M29" s="6">
+      <c r="M29" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(20,30,0))*(Orari!$T$6:$T$15&gt;TIME(20,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(20,30,0))*(Orari!$V$6:$V$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -3106,51 +3119,51 @@
           <t>sabato 17 ottobre 2026</t>
         </is>
       </c>
-      <c r="B30" s="6">
+      <c r="B30" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(9,30,0))*(Orari!$X$6:$X$15&gt;TIME(9,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(9,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C30" s="6">
+      <c r="C30" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(10,30,0))*(Orari!$X$6:$X$15&gt;TIME(10,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(10,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D30" s="6">
+      <c r="D30" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(11,30,0))*(Orari!$X$6:$X$15&gt;TIME(11,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(11,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E30" s="6">
+      <c r="E30" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(12,30,0))*(Orari!$X$6:$X$15&gt;TIME(12,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(12,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F30" s="6">
+      <c r="F30" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(13,30,0))*(Orari!$X$6:$X$15&gt;TIME(13,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(13,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G30" s="6">
+      <c r="G30" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(14,30,0))*(Orari!$X$6:$X$15&gt;TIME(14,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(14,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H30" s="6">
+      <c r="H30" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(15,30,0))*(Orari!$X$6:$X$15&gt;TIME(15,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(15,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I30" s="6">
+      <c r="I30" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(16,30,0))*(Orari!$X$6:$X$15&gt;TIME(16,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(16,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J30" s="6">
+      <c r="J30" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(17,30,0))*(Orari!$X$6:$X$15&gt;TIME(17,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(17,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K30" s="6">
+      <c r="K30" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(18,30,0))*(Orari!$X$6:$X$15&gt;TIME(18,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(18,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L30" s="6">
+      <c r="L30" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(19,30,0))*(Orari!$X$6:$X$15&gt;TIME(19,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(19,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M30" s="6">
+      <c r="M30" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(20,30,0))*(Orari!$X$6:$X$15&gt;TIME(20,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(20,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -3161,51 +3174,51 @@
           <t>domenica 18 ottobre 2026</t>
         </is>
       </c>
-      <c r="B31" s="6">
+      <c r="B31" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(9,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(9,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(9,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C31" s="6">
+      <c r="C31" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(10,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(10,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(10,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D31" s="6">
+      <c r="D31" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(11,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(11,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(11,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E31" s="6">
+      <c r="E31" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(12,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(12,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(12,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F31" s="6">
+      <c r="F31" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(13,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(13,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(13,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G31" s="6">
+      <c r="G31" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(14,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(14,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(14,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H31" s="6">
+      <c r="H31" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(15,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(15,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(15,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I31" s="6">
+      <c r="I31" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(16,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(16,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(16,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J31" s="6">
+      <c r="J31" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(17,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(17,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(17,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K31" s="6">
+      <c r="K31" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(18,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(18,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(18,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L31" s="6">
+      <c r="L31" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(19,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(19,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(19,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M31" s="6">
+      <c r="M31" s="5">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(20,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(20,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(20,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Orari: Bruni Laura (30h) al posto di Latini Alessandro
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RgW8tUpL59m5j1P2CKTdxn
</commit_message>
<xml_diff>
--- a/orari/Orari_12-18_ottobre_2026.xlsx
+++ b/orari/Orari_12-18_ottobre_2026.xlsx
@@ -104,13 +104,13 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -869,7 +869,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>LATINI ALESSANDRO</t>
+          <t>BRUNI LAURA</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -877,56 +877,48 @@
           <t>Addetto vendite</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
       <c r="D6" s="5" t="n"/>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="H6" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="F6" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
       <c r="J6" s="7" t="n"/>
-      <c r="K6" s="5" t="n"/>
-      <c r="L6" s="5" t="n"/>
+      <c r="K6" s="7" t="n"/>
+      <c r="L6" s="7" t="n"/>
       <c r="M6" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="N6" s="6" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="P6" s="5" t="n"/>
+      <c r="Q6" s="5" t="n"/>
+      <c r="R6" s="5" t="n"/>
+      <c r="S6" s="7" t="n"/>
+      <c r="T6" s="7" t="n"/>
+      <c r="U6" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="N6" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="O6" s="6" t="n">
-        <v>0.4583333333333333</v>
-      </c>
-      <c r="P6" s="6" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="Q6" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="R6" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="S6" s="6" t="n">
+      <c r="V6" s="6" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="W6" s="6" t="n">
         <v>0.4166666666666667</v>
-      </c>
-      <c r="T6" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="U6" s="6" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="V6" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="W6" s="6" t="n">
-        <v>0.375</v>
       </c>
       <c r="X6" s="6" t="n">
         <v>0.5416666666666666</v>
@@ -935,22 +927,22 @@
         <v>0.5833333333333334</v>
       </c>
       <c r="Z6" s="6" t="n">
-        <v>0.7916666666666666</v>
-      </c>
-      <c r="AA6" s="7" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="AB6" s="7" t="n"/>
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="AA6" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="AB6" s="6" t="n">
+        <v>0.625</v>
+      </c>
       <c r="AC6" s="7" t="n"/>
       <c r="AD6" s="7" t="n"/>
       <c r="AE6" s="8">
         <f>ROUND(24*(N(D6)-N(C6)+N(F6)-N(E6)+N(H6)-N(G6)+N(J6)-N(I6)+N(L6)-N(K6)+N(N6)-N(M6)+N(P6)-N(O6)+N(R6)-N(Q6)+N(T6)-N(S6)+N(V6)-N(U6)+N(X6)-N(W6)+N(Z6)-N(Y6)+N(AB6)-N(AA6)+N(AD6)-N(AC6)),2)</f>
         <v/>
       </c>
-      <c r="AF6" s="5" t="n">
-        <v>40</v>
+      <c r="AF6" s="7" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="7">
@@ -982,40 +974,36 @@
       <c r="H7" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="I7" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="J7" s="6" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="K7" s="7" t="inlineStr">
+      <c r="I7" s="7" t="n"/>
+      <c r="J7" s="7" t="n"/>
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="L7" s="7" t="n"/>
-      <c r="M7" s="7" t="n"/>
-      <c r="N7" s="7" t="n"/>
+      <c r="L7" s="5" t="n"/>
+      <c r="M7" s="5" t="n"/>
+      <c r="N7" s="5" t="n"/>
       <c r="O7" s="6" t="n">
         <v>0.4166666666666667</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>0.5416666666666666</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.7083333333333334</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>0.875</v>
       </c>
-      <c r="S7" s="7" t="inlineStr">
+      <c r="S7" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="T7" s="7" t="n"/>
-      <c r="U7" s="7" t="n"/>
-      <c r="V7" s="7" t="n"/>
+      <c r="T7" s="5" t="n"/>
+      <c r="U7" s="5" t="n"/>
+      <c r="V7" s="5" t="n"/>
       <c r="W7" s="6" t="n">
         <v>0.4583333333333333</v>
       </c>
@@ -1028,19 +1016,23 @@
       <c r="Z7" s="6" t="n">
         <v>0.875</v>
       </c>
-      <c r="AA7" s="5" t="n"/>
-      <c r="AB7" s="5" t="n"/>
+      <c r="AA7" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="AB7" s="6" t="n">
+        <v>0.625</v>
+      </c>
       <c r="AC7" s="6" t="n">
-        <v>0.625</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="AD7" s="6" t="n">
-        <v>0.875</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="AE7" s="8">
         <f>ROUND(24*(N(D7)-N(C7)+N(F7)-N(E7)+N(H7)-N(G7)+N(J7)-N(I7)+N(L7)-N(K7)+N(N7)-N(M7)+N(P7)-N(O7)+N(R7)-N(Q7)+N(T7)-N(S7)+N(V7)-N(U7)+N(X7)-N(W7)+N(Z7)-N(Y7)+N(AB7)-N(AA7)+N(AD7)-N(AC7)),2)</f>
         <v/>
       </c>
-      <c r="AF7" s="5" t="inlineStr">
+      <c r="AF7" s="7" t="inlineStr">
         <is>
           <t>44-45</t>
         </is>
@@ -1057,16 +1049,16 @@
           <t>Addetto vendite</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="7" t="n"/>
       <c r="I8" s="6" t="n">
         <v>0.625</v>
       </c>
@@ -1077,22 +1069,22 @@
         <v>0.375</v>
       </c>
       <c r="L8" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="M8" s="6" t="n">
         <v>0.625</v>
-      </c>
-      <c r="M8" s="6" t="n">
-        <v>0.6666666666666666</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="O8" s="7" t="inlineStr">
+      <c r="O8" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="P8" s="7" t="n"/>
-      <c r="Q8" s="7" t="n"/>
-      <c r="R8" s="7" t="n"/>
+      <c r="P8" s="5" t="n"/>
+      <c r="Q8" s="5" t="n"/>
+      <c r="R8" s="5" t="n"/>
       <c r="S8" s="6" t="n">
         <v>0.375</v>
       </c>
@@ -1106,30 +1098,30 @@
         <v>0.7916666666666666</v>
       </c>
       <c r="W8" s="6" t="n">
-        <v>0.4583333333333333</v>
+        <v>0.375</v>
       </c>
       <c r="X8" s="6" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5416666666666666</v>
       </c>
       <c r="Y8" s="6" t="n">
-        <v>0.7083333333333334</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="Z8" s="6" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="AA8" s="7" t="n"/>
+      <c r="AB8" s="7" t="n"/>
+      <c r="AC8" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="AD8" s="6" t="n">
         <v>0.875</v>
       </c>
-      <c r="AA8" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="AB8" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="AC8" s="5" t="n"/>
-      <c r="AD8" s="5" t="n"/>
       <c r="AE8" s="8">
         <f>ROUND(24*(N(D8)-N(C8)+N(F8)-N(E8)+N(H8)-N(G8)+N(J8)-N(I8)+N(L8)-N(K8)+N(N8)-N(M8)+N(P8)-N(O8)+N(R8)-N(Q8)+N(T8)-N(S8)+N(V8)-N(U8)+N(X8)-N(W8)+N(Z8)-N(Y8)+N(AB8)-N(AA8)+N(AD8)-N(AC8)),2)</f>
         <v/>
       </c>
-      <c r="AF8" s="5" t="n">
+      <c r="AF8" s="7" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1154,58 +1146,58 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="H9" s="7" t="n"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
-      <c r="K9" s="5" t="n"/>
-      <c r="L9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="5" t="n"/>
+      <c r="J9" s="5" t="n"/>
+      <c r="K9" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
       <c r="M9" s="6" t="n">
-        <v>0.625</v>
+        <v>0.7083333333333334</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>0.875</v>
       </c>
-      <c r="O9" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="P9" s="6" t="n">
-        <v>0.5</v>
-      </c>
+      <c r="O9" s="7" t="n"/>
+      <c r="P9" s="7" t="n"/>
       <c r="Q9" s="6" t="n">
-        <v>0.5416666666666666</v>
+        <v>0.625</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>0.7916666666666666</v>
-      </c>
-      <c r="S9" s="7" t="inlineStr">
+        <v>0.875</v>
+      </c>
+      <c r="S9" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="T9" s="7" t="n"/>
-      <c r="U9" s="7" t="n"/>
-      <c r="V9" s="7" t="n"/>
+      <c r="T9" s="5" t="n"/>
+      <c r="U9" s="5" t="n"/>
+      <c r="V9" s="5" t="n"/>
       <c r="W9" s="6" t="n">
         <v>0.375</v>
       </c>
       <c r="X9" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Y9" s="6" t="n">
         <v>0.5416666666666666</v>
-      </c>
-      <c r="Y9" s="6" t="n">
-        <v>0.5833333333333334</v>
       </c>
       <c r="Z9" s="6" t="n">
         <v>0.7916666666666666</v>
       </c>
-      <c r="AA9" s="5" t="n"/>
-      <c r="AB9" s="5" t="n"/>
+      <c r="AA9" s="7" t="n"/>
+      <c r="AB9" s="7" t="n"/>
       <c r="AC9" s="6" t="n">
         <v>0.625</v>
       </c>
@@ -1216,7 +1208,7 @@
         <f>ROUND(24*(N(D9)-N(C9)+N(F9)-N(E9)+N(H9)-N(G9)+N(J9)-N(I9)+N(L9)-N(K9)+N(N9)-N(M9)+N(P9)-N(O9)+N(R9)-N(Q9)+N(T9)-N(S9)+N(V9)-N(U9)+N(X9)-N(W9)+N(Z9)-N(Y9)+N(AB9)-N(AA9)+N(AD9)-N(AC9)),2)</f>
         <v/>
       </c>
-      <c r="AF9" s="5" t="n">
+      <c r="AF9" s="7" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1231,46 +1223,50 @@
           <t>Addetto vendite</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
+      <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
-      <c r="G10" s="6" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="H10" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
+      <c r="E10" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
       <c r="I10" s="6" t="n">
-        <v>0.7083333333333334</v>
+        <v>0.625</v>
       </c>
       <c r="J10" s="6" t="n">
         <v>0.875</v>
       </c>
-      <c r="K10" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="L10" s="6" t="n">
-        <v>0.625</v>
-      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="n"/>
       <c r="M10" s="5" t="n"/>
       <c r="N10" s="5" t="n"/>
-      <c r="O10" s="7" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="P10" s="7" t="n"/>
-      <c r="Q10" s="7" t="n"/>
-      <c r="R10" s="7" t="n"/>
-      <c r="S10" s="5" t="n"/>
-      <c r="T10" s="5" t="n"/>
+      <c r="O10" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="P10" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="Q10" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="R10" s="6" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="S10" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="T10" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
       <c r="U10" s="6" t="n">
-        <v>0.625</v>
+        <v>0.7083333333333334</v>
       </c>
       <c r="V10" s="6" t="n">
         <v>0.875</v>
@@ -1279,31 +1275,27 @@
         <v>0.4583333333333333</v>
       </c>
       <c r="X10" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="Y10" s="6" t="n">
         <v>0.625</v>
-      </c>
-      <c r="Y10" s="6" t="n">
-        <v>0.6666666666666666</v>
       </c>
       <c r="Z10" s="6" t="n">
         <v>0.875</v>
       </c>
-      <c r="AA10" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="AB10" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="AC10" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="AD10" s="6" t="n">
-        <v>0.7916666666666666</v>
-      </c>
+      <c r="AA10" s="5" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="AB10" s="5" t="n"/>
+      <c r="AC10" s="5" t="n"/>
+      <c r="AD10" s="5" t="n"/>
       <c r="AE10" s="8">
         <f>ROUND(24*(N(D10)-N(C10)+N(F10)-N(E10)+N(H10)-N(G10)+N(J10)-N(I10)+N(L10)-N(K10)+N(N10)-N(M10)+N(P10)-N(O10)+N(R10)-N(Q10)+N(T10)-N(S10)+N(V10)-N(U10)+N(X10)-N(W10)+N(Z10)-N(Y10)+N(AB10)-N(AA10)+N(AD10)-N(AC10)),2)</f>
         <v/>
       </c>
-      <c r="AF10" s="5" t="n">
+      <c r="AF10" s="7" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1330,14 +1322,14 @@
       <c r="F11" s="6" t="n">
         <v>0.7083333333333334</v>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="H11" s="7" t="n"/>
-      <c r="I11" s="7" t="n"/>
-      <c r="J11" s="7" t="n"/>
+      <c r="H11" s="5" t="n"/>
+      <c r="I11" s="5" t="n"/>
+      <c r="J11" s="5" t="n"/>
       <c r="K11" s="6" t="n">
         <v>0.4166666666666667</v>
       </c>
@@ -1380,21 +1372,21 @@
       <c r="X11" s="6" t="n">
         <v>0.625</v>
       </c>
-      <c r="Y11" s="5" t="n"/>
-      <c r="Z11" s="5" t="n"/>
-      <c r="AA11" s="7" t="inlineStr">
+      <c r="Y11" s="7" t="n"/>
+      <c r="Z11" s="7" t="n"/>
+      <c r="AA11" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="AB11" s="7" t="n"/>
-      <c r="AC11" s="7" t="n"/>
-      <c r="AD11" s="7" t="n"/>
+      <c r="AB11" s="5" t="n"/>
+      <c r="AC11" s="5" t="n"/>
+      <c r="AD11" s="5" t="n"/>
       <c r="AE11" s="8">
         <f>ROUND(24*(N(D11)-N(C11)+N(F11)-N(E11)+N(H11)-N(G11)+N(J11)-N(I11)+N(L11)-N(K11)+N(N11)-N(M11)+N(P11)-N(O11)+N(R11)-N(Q11)+N(T11)-N(S11)+N(V11)-N(U11)+N(X11)-N(W11)+N(Z11)-N(Y11)+N(AB11)-N(AA11)+N(AD11)-N(AC11)),2)</f>
         <v/>
       </c>
-      <c r="AF11" s="5" t="n">
+      <c r="AF11" s="7" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1409,8 +1401,8 @@
           <t>Cassiera</t>
         </is>
       </c>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="7" t="n"/>
       <c r="E12" s="6" t="n">
         <v>0.7083333333333334</v>
       </c>
@@ -1423,40 +1415,40 @@
       <c r="H12" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="I12" s="5" t="n"/>
-      <c r="J12" s="5" t="n"/>
-      <c r="K12" s="7" t="inlineStr">
+      <c r="I12" s="7" t="n"/>
+      <c r="J12" s="7" t="n"/>
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="L12" s="7" t="n"/>
-      <c r="M12" s="7" t="n"/>
-      <c r="N12" s="7" t="n"/>
-      <c r="O12" s="7" t="inlineStr">
+      <c r="L12" s="5" t="n"/>
+      <c r="M12" s="5" t="n"/>
+      <c r="N12" s="5" t="n"/>
+      <c r="O12" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="P12" s="7" t="n"/>
-      <c r="Q12" s="7" t="n"/>
-      <c r="R12" s="7" t="n"/>
+      <c r="P12" s="5" t="n"/>
+      <c r="Q12" s="5" t="n"/>
+      <c r="R12" s="5" t="n"/>
       <c r="S12" s="6" t="n">
         <v>0.375</v>
       </c>
       <c r="T12" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="U12" s="5" t="n"/>
-      <c r="V12" s="5" t="n"/>
-      <c r="W12" s="7" t="inlineStr">
+      <c r="U12" s="7" t="n"/>
+      <c r="V12" s="7" t="n"/>
+      <c r="W12" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="X12" s="7" t="n"/>
-      <c r="Y12" s="7" t="n"/>
-      <c r="Z12" s="7" t="n"/>
+      <c r="X12" s="5" t="n"/>
+      <c r="Y12" s="5" t="n"/>
+      <c r="Z12" s="5" t="n"/>
       <c r="AA12" s="6" t="n">
         <v>0.4166666666666667</v>
       </c>
@@ -1473,7 +1465,7 @@
         <f>ROUND(24*(N(D12)-N(C12)+N(F12)-N(E12)+N(H12)-N(G12)+N(J12)-N(I12)+N(L12)-N(K12)+N(N12)-N(M12)+N(P12)-N(O12)+N(R12)-N(Q12)+N(T12)-N(S12)+N(V12)-N(U12)+N(X12)-N(W12)+N(Z12)-N(Y12)+N(AB12)-N(AA12)+N(AD12)-N(AC12)),2)</f>
         <v/>
       </c>
-      <c r="AF12" s="5" t="n">
+      <c r="AF12" s="7" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1488,16 +1480,16 @@
           <t>Cassiera</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="7" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
       <c r="I13" s="6" t="n">
         <v>0.625</v>
       </c>
@@ -1510,45 +1502,45 @@
       <c r="L13" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="M13" s="5" t="n"/>
-      <c r="N13" s="5" t="n"/>
+      <c r="M13" s="7" t="n"/>
+      <c r="N13" s="7" t="n"/>
       <c r="O13" s="6" t="n">
         <v>0.4166666666666667</v>
       </c>
       <c r="P13" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="Q13" s="5" t="n"/>
-      <c r="R13" s="5" t="n"/>
-      <c r="S13" s="5" t="n"/>
-      <c r="T13" s="5" t="n"/>
+      <c r="Q13" s="7" t="n"/>
+      <c r="R13" s="7" t="n"/>
+      <c r="S13" s="7" t="n"/>
+      <c r="T13" s="7" t="n"/>
       <c r="U13" s="6" t="n">
         <v>0.625</v>
       </c>
       <c r="V13" s="6" t="n">
         <v>0.7916666666666666</v>
       </c>
-      <c r="W13" s="5" t="n"/>
-      <c r="X13" s="5" t="n"/>
+      <c r="W13" s="7" t="n"/>
+      <c r="X13" s="7" t="n"/>
       <c r="Y13" s="6" t="n">
         <v>0.6666666666666666</v>
       </c>
       <c r="Z13" s="6" t="n">
         <v>0.875</v>
       </c>
-      <c r="AA13" s="7" t="inlineStr">
+      <c r="AA13" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="AB13" s="7" t="n"/>
-      <c r="AC13" s="7" t="n"/>
-      <c r="AD13" s="7" t="n"/>
+      <c r="AB13" s="5" t="n"/>
+      <c r="AC13" s="5" t="n"/>
+      <c r="AD13" s="5" t="n"/>
       <c r="AE13" s="8">
         <f>ROUND(24*(N(D13)-N(C13)+N(F13)-N(E13)+N(H13)-N(G13)+N(J13)-N(I13)+N(L13)-N(K13)+N(N13)-N(M13)+N(P13)-N(O13)+N(R13)-N(Q13)+N(T13)-N(S13)+N(V13)-N(U13)+N(X13)-N(W13)+N(Z13)-N(Y13)+N(AB13)-N(AA13)+N(AD13)-N(AC13)),2)</f>
         <v/>
       </c>
-      <c r="AF13" s="5" t="n">
+      <c r="AF13" s="7" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1569,42 +1561,42 @@
       <c r="D14" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="7" t="n"/>
       <c r="I14" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
       <c r="J14" s="6" t="n">
         <v>0.75</v>
       </c>
-      <c r="K14" s="7" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="L14" s="7" t="n"/>
-      <c r="M14" s="7" t="n"/>
-      <c r="N14" s="7" t="n"/>
-      <c r="O14" s="5" t="n"/>
-      <c r="P14" s="5" t="n"/>
+      <c r="L14" s="5" t="n"/>
+      <c r="M14" s="5" t="n"/>
+      <c r="N14" s="5" t="n"/>
+      <c r="O14" s="7" t="n"/>
+      <c r="P14" s="7" t="n"/>
       <c r="Q14" s="6" t="n">
         <v>0.7083333333333334</v>
       </c>
       <c r="R14" s="6" t="n">
         <v>0.875</v>
       </c>
-      <c r="S14" s="7" t="inlineStr">
+      <c r="S14" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="T14" s="7" t="n"/>
-      <c r="U14" s="7" t="n"/>
-      <c r="V14" s="7" t="n"/>
-      <c r="W14" s="5" t="n"/>
-      <c r="X14" s="5" t="n"/>
+      <c r="T14" s="5" t="n"/>
+      <c r="U14" s="5" t="n"/>
+      <c r="V14" s="5" t="n"/>
+      <c r="W14" s="7" t="n"/>
+      <c r="X14" s="7" t="n"/>
       <c r="Y14" s="6" t="n">
         <v>0.625</v>
       </c>
@@ -1627,7 +1619,7 @@
         <f>ROUND(24*(N(D14)-N(C14)+N(F14)-N(E14)+N(H14)-N(G14)+N(J14)-N(I14)+N(L14)-N(K14)+N(N14)-N(M14)+N(P14)-N(O14)+N(R14)-N(Q14)+N(T14)-N(S14)+N(V14)-N(U14)+N(X14)-N(W14)+N(Z14)-N(Y14)+N(AB14)-N(AA14)+N(AD14)-N(AC14)),2)</f>
         <v/>
       </c>
-      <c r="AF14" s="5" t="n">
+      <c r="AF14" s="7" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1702,27 +1694,27 @@
       <c r="V15" s="6" t="n">
         <v>0.75</v>
       </c>
-      <c r="W15" s="7" t="inlineStr">
+      <c r="W15" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="X15" s="7" t="n"/>
-      <c r="Y15" s="7" t="n"/>
-      <c r="Z15" s="7" t="n"/>
-      <c r="AA15" s="7" t="inlineStr">
+      <c r="X15" s="5" t="n"/>
+      <c r="Y15" s="5" t="n"/>
+      <c r="Z15" s="5" t="n"/>
+      <c r="AA15" s="5" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="AB15" s="7" t="n"/>
-      <c r="AC15" s="7" t="n"/>
-      <c r="AD15" s="7" t="n"/>
+      <c r="AB15" s="5" t="n"/>
+      <c r="AC15" s="5" t="n"/>
+      <c r="AD15" s="5" t="n"/>
       <c r="AE15" s="8">
         <f>ROUND(24*(N(D15)-N(C15)+N(F15)-N(E15)+N(H15)-N(G15)+N(J15)-N(I15)+N(L15)-N(K15)+N(N15)-N(M15)+N(P15)-N(O15)+N(R15)-N(Q15)+N(T15)-N(S15)+N(V15)-N(U15)+N(X15)-N(W15)+N(Z15)-N(Y15)+N(AB15)-N(AA15)+N(AD15)-N(AC15)),2)</f>
         <v/>
       </c>
-      <c r="AF15" s="5" t="n">
+      <c r="AF15" s="7" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1772,6 +1764,7 @@
     <mergeCell ref="O8:R8"/>
     <mergeCell ref="AA3:AD3"/>
     <mergeCell ref="K7:N7"/>
+    <mergeCell ref="K10:N10"/>
     <mergeCell ref="AA11:AD11"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C13:F13"/>
@@ -1780,25 +1773,24 @@
     <mergeCell ref="C3:F3"/>
     <mergeCell ref="K3:N3"/>
     <mergeCell ref="O3:R3"/>
+    <mergeCell ref="C6:F6"/>
     <mergeCell ref="B3:B5"/>
-    <mergeCell ref="O10:R10"/>
     <mergeCell ref="G11:J11"/>
+    <mergeCell ref="O6:R6"/>
     <mergeCell ref="O4:P4"/>
-    <mergeCell ref="W15:Z15"/>
+    <mergeCell ref="AA10:AD10"/>
     <mergeCell ref="AA4:AB4"/>
     <mergeCell ref="Q4:R4"/>
+    <mergeCell ref="W15:Z15"/>
     <mergeCell ref="AC4:AD4"/>
     <mergeCell ref="AF3:AF5"/>
     <mergeCell ref="AA13:AD13"/>
     <mergeCell ref="S3:V3"/>
     <mergeCell ref="AE3:AE5"/>
-    <mergeCell ref="AA6:AD6"/>
     <mergeCell ref="S7:V7"/>
-    <mergeCell ref="C10:F10"/>
     <mergeCell ref="AA15:AD15"/>
     <mergeCell ref="S14:V14"/>
     <mergeCell ref="G4:H4"/>
-    <mergeCell ref="G6:J6"/>
     <mergeCell ref="I4:J4"/>
     <mergeCell ref="W3:Z3"/>
     <mergeCell ref="G3:J3"/>
@@ -1926,51 +1918,51 @@
           <t>lunedì 12 ottobre 2026</t>
         </is>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(9,30,0))*(Orari!$D$6:$D$15&gt;TIME(9,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(9,30,0))*(Orari!$F$6:$F$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(10,30,0))*(Orari!$D$6:$D$15&gt;TIME(10,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(10,30,0))*(Orari!$F$6:$F$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(11,30,0))*(Orari!$D$6:$D$15&gt;TIME(11,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(11,30,0))*(Orari!$F$6:$F$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(12,30,0))*(Orari!$D$6:$D$15&gt;TIME(12,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(12,30,0))*(Orari!$F$6:$F$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(13,30,0))*(Orari!$D$6:$D$15&gt;TIME(13,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(13,30,0))*(Orari!$F$6:$F$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(14,30,0))*(Orari!$D$6:$D$15&gt;TIME(14,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(14,30,0))*(Orari!$F$6:$F$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(15,30,0))*(Orari!$D$6:$D$15&gt;TIME(15,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(15,30,0))*(Orari!$F$6:$F$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I5" s="5">
+      <c r="I5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(16,30,0))*(Orari!$D$6:$D$15&gt;TIME(16,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(16,30,0))*(Orari!$F$6:$F$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J5" s="5">
+      <c r="J5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(17,30,0))*(Orari!$D$6:$D$15&gt;TIME(17,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(17,30,0))*(Orari!$F$6:$F$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K5" s="5">
+      <c r="K5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(18,30,0))*(Orari!$D$6:$D$15&gt;TIME(18,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(18,30,0))*(Orari!$F$6:$F$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L5" s="5">
+      <c r="L5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(19,30,0))*(Orari!$D$6:$D$15&gt;TIME(19,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(19,30,0))*(Orari!$F$6:$F$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M5" s="5">
+      <c r="M5" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(20,30,0))*(Orari!$D$6:$D$15&gt;TIME(20,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(20,30,0))*(Orari!$F$6:$F$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -1981,51 +1973,51 @@
           <t>martedì 13 ottobre 2026</t>
         </is>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(9,30,0))*(Orari!$H$6:$H$15&gt;TIME(9,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(9,30,0))*(Orari!$J$6:$J$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(10,30,0))*(Orari!$H$6:$H$15&gt;TIME(10,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(10,30,0))*(Orari!$J$6:$J$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(11,30,0))*(Orari!$H$6:$H$15&gt;TIME(11,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(11,30,0))*(Orari!$J$6:$J$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(12,30,0))*(Orari!$H$6:$H$15&gt;TIME(12,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(12,30,0))*(Orari!$J$6:$J$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(13,30,0))*(Orari!$H$6:$H$15&gt;TIME(13,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(13,30,0))*(Orari!$J$6:$J$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(14,30,0))*(Orari!$H$6:$H$15&gt;TIME(14,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(14,30,0))*(Orari!$J$6:$J$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(15,30,0))*(Orari!$H$6:$H$15&gt;TIME(15,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(15,30,0))*(Orari!$J$6:$J$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I6" s="5">
+      <c r="I6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(16,30,0))*(Orari!$H$6:$H$15&gt;TIME(16,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(16,30,0))*(Orari!$J$6:$J$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J6" s="5">
+      <c r="J6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(17,30,0))*(Orari!$H$6:$H$15&gt;TIME(17,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(17,30,0))*(Orari!$J$6:$J$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K6" s="5">
+      <c r="K6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(18,30,0))*(Orari!$H$6:$H$15&gt;TIME(18,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(18,30,0))*(Orari!$J$6:$J$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L6" s="5">
+      <c r="L6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(19,30,0))*(Orari!$H$6:$H$15&gt;TIME(19,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(19,30,0))*(Orari!$J$6:$J$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M6" s="5">
+      <c r="M6" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(20,30,0))*(Orari!$H$6:$H$15&gt;TIME(20,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(20,30,0))*(Orari!$J$6:$J$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2036,51 +2028,51 @@
           <t>mercoledì 14 ottobre 2026</t>
         </is>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(9,30,0))*(Orari!$L$6:$L$15&gt;TIME(9,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(9,30,0))*(Orari!$N$6:$N$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(10,30,0))*(Orari!$L$6:$L$15&gt;TIME(10,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(10,30,0))*(Orari!$N$6:$N$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(11,30,0))*(Orari!$L$6:$L$15&gt;TIME(11,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(11,30,0))*(Orari!$N$6:$N$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(12,30,0))*(Orari!$L$6:$L$15&gt;TIME(12,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(12,30,0))*(Orari!$N$6:$N$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(13,30,0))*(Orari!$L$6:$L$15&gt;TIME(13,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(13,30,0))*(Orari!$N$6:$N$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(14,30,0))*(Orari!$L$6:$L$15&gt;TIME(14,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(14,30,0))*(Orari!$N$6:$N$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(15,30,0))*(Orari!$L$6:$L$15&gt;TIME(15,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(15,30,0))*(Orari!$N$6:$N$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I7" s="5">
+      <c r="I7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(16,30,0))*(Orari!$L$6:$L$15&gt;TIME(16,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(16,30,0))*(Orari!$N$6:$N$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(17,30,0))*(Orari!$L$6:$L$15&gt;TIME(17,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(17,30,0))*(Orari!$N$6:$N$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(18,30,0))*(Orari!$L$6:$L$15&gt;TIME(18,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(18,30,0))*(Orari!$N$6:$N$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L7" s="5">
+      <c r="L7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(19,30,0))*(Orari!$L$6:$L$15&gt;TIME(19,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(19,30,0))*(Orari!$N$6:$N$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M7" s="5">
+      <c r="M7" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(20,30,0))*(Orari!$L$6:$L$15&gt;TIME(20,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(20,30,0))*(Orari!$N$6:$N$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2091,51 +2083,51 @@
           <t>giovedì 15 ottobre 2026</t>
         </is>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(9,30,0))*(Orari!$P$6:$P$15&gt;TIME(9,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(9,30,0))*(Orari!$R$6:$R$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(10,30,0))*(Orari!$P$6:$P$15&gt;TIME(10,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(10,30,0))*(Orari!$R$6:$R$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(11,30,0))*(Orari!$P$6:$P$15&gt;TIME(11,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(11,30,0))*(Orari!$R$6:$R$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(12,30,0))*(Orari!$P$6:$P$15&gt;TIME(12,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(12,30,0))*(Orari!$R$6:$R$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(13,30,0))*(Orari!$P$6:$P$15&gt;TIME(13,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(13,30,0))*(Orari!$R$6:$R$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(14,30,0))*(Orari!$P$6:$P$15&gt;TIME(14,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(14,30,0))*(Orari!$R$6:$R$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(15,30,0))*(Orari!$P$6:$P$15&gt;TIME(15,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(15,30,0))*(Orari!$R$6:$R$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I8" s="5">
+      <c r="I8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(16,30,0))*(Orari!$P$6:$P$15&gt;TIME(16,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(16,30,0))*(Orari!$R$6:$R$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(17,30,0))*(Orari!$P$6:$P$15&gt;TIME(17,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(17,30,0))*(Orari!$R$6:$R$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(18,30,0))*(Orari!$P$6:$P$15&gt;TIME(18,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(18,30,0))*(Orari!$R$6:$R$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L8" s="5">
+      <c r="L8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(19,30,0))*(Orari!$P$6:$P$15&gt;TIME(19,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(19,30,0))*(Orari!$R$6:$R$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M8" s="5">
+      <c r="M8" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(20,30,0))*(Orari!$P$6:$P$15&gt;TIME(20,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(20,30,0))*(Orari!$R$6:$R$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2146,51 +2138,51 @@
           <t>venerdì 16 ottobre 2026</t>
         </is>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(9,30,0))*(Orari!$T$6:$T$15&gt;TIME(9,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(9,30,0))*(Orari!$V$6:$V$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(10,30,0))*(Orari!$T$6:$T$15&gt;TIME(10,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(10,30,0))*(Orari!$V$6:$V$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(11,30,0))*(Orari!$T$6:$T$15&gt;TIME(11,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(11,30,0))*(Orari!$V$6:$V$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(12,30,0))*(Orari!$T$6:$T$15&gt;TIME(12,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(12,30,0))*(Orari!$V$6:$V$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(13,30,0))*(Orari!$T$6:$T$15&gt;TIME(13,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(13,30,0))*(Orari!$V$6:$V$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(14,30,0))*(Orari!$T$6:$T$15&gt;TIME(14,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(14,30,0))*(Orari!$V$6:$V$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(15,30,0))*(Orari!$T$6:$T$15&gt;TIME(15,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(15,30,0))*(Orari!$V$6:$V$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I9" s="5">
+      <c r="I9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(16,30,0))*(Orari!$T$6:$T$15&gt;TIME(16,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(16,30,0))*(Orari!$V$6:$V$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(17,30,0))*(Orari!$T$6:$T$15&gt;TIME(17,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(17,30,0))*(Orari!$V$6:$V$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(18,30,0))*(Orari!$T$6:$T$15&gt;TIME(18,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(18,30,0))*(Orari!$V$6:$V$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L9" s="5">
+      <c r="L9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(19,30,0))*(Orari!$T$6:$T$15&gt;TIME(19,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(19,30,0))*(Orari!$V$6:$V$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M9" s="5">
+      <c r="M9" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(20,30,0))*(Orari!$T$6:$T$15&gt;TIME(20,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(20,30,0))*(Orari!$V$6:$V$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2201,51 +2193,51 @@
           <t>sabato 17 ottobre 2026</t>
         </is>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(9,30,0))*(Orari!$X$6:$X$15&gt;TIME(9,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(9,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(10,30,0))*(Orari!$X$6:$X$15&gt;TIME(10,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(10,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(11,30,0))*(Orari!$X$6:$X$15&gt;TIME(11,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(11,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(12,30,0))*(Orari!$X$6:$X$15&gt;TIME(12,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(12,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(13,30,0))*(Orari!$X$6:$X$15&gt;TIME(13,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(13,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(14,30,0))*(Orari!$X$6:$X$15&gt;TIME(14,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(14,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(15,30,0))*(Orari!$X$6:$X$15&gt;TIME(15,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(15,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I10" s="5">
+      <c r="I10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(16,30,0))*(Orari!$X$6:$X$15&gt;TIME(16,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(16,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(17,30,0))*(Orari!$X$6:$X$15&gt;TIME(17,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(17,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K10" s="5">
+      <c r="K10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(18,30,0))*(Orari!$X$6:$X$15&gt;TIME(18,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(18,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L10" s="5">
+      <c r="L10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(19,30,0))*(Orari!$X$6:$X$15&gt;TIME(19,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(19,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M10" s="5">
+      <c r="M10" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(20,30,0))*(Orari!$X$6:$X$15&gt;TIME(20,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(20,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2256,51 +2248,51 @@
           <t>domenica 18 ottobre 2026</t>
         </is>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(9,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(9,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(9,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(10,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(10,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(10,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(11,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(11,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(11,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(12,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(12,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(12,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F11" s="5">
+      <c r="F11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(13,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(13,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(13,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(14,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(14,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(14,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(15,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(15,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(15,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I11" s="5">
+      <c r="I11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(16,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(16,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(16,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(17,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(17,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(17,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K11" s="5">
+      <c r="K11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(18,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(18,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(18,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L11" s="5">
+      <c r="L11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(19,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(19,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(19,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M11" s="5">
+      <c r="M11" s="7">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(20,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(20,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(20,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2385,51 +2377,51 @@
           <t>lunedì 12 ottobre 2026</t>
         </is>
       </c>
-      <c r="B15" s="5">
+      <c r="B15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(9,30,0))*(Orari!$D$6:$D$15&gt;TIME(9,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(9,30,0))*(Orari!$F$6:$F$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(10,30,0))*(Orari!$D$6:$D$15&gt;TIME(10,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(10,30,0))*(Orari!$F$6:$F$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(11,30,0))*(Orari!$D$6:$D$15&gt;TIME(11,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(11,30,0))*(Orari!$F$6:$F$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(12,30,0))*(Orari!$D$6:$D$15&gt;TIME(12,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(12,30,0))*(Orari!$F$6:$F$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(13,30,0))*(Orari!$D$6:$D$15&gt;TIME(13,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(13,30,0))*(Orari!$F$6:$F$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(14,30,0))*(Orari!$D$6:$D$15&gt;TIME(14,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(14,30,0))*(Orari!$F$6:$F$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(15,30,0))*(Orari!$D$6:$D$15&gt;TIME(15,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(15,30,0))*(Orari!$F$6:$F$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I15" s="5">
+      <c r="I15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(16,30,0))*(Orari!$D$6:$D$15&gt;TIME(16,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(16,30,0))*(Orari!$F$6:$F$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J15" s="5">
+      <c r="J15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(17,30,0))*(Orari!$D$6:$D$15&gt;TIME(17,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(17,30,0))*(Orari!$F$6:$F$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K15" s="5">
+      <c r="K15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(18,30,0))*(Orari!$D$6:$D$15&gt;TIME(18,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(18,30,0))*(Orari!$F$6:$F$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L15" s="5">
+      <c r="L15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(19,30,0))*(Orari!$D$6:$D$15&gt;TIME(19,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(19,30,0))*(Orari!$F$6:$F$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M15" s="5">
+      <c r="M15" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(20,30,0))*(Orari!$D$6:$D$15&gt;TIME(20,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(20,30,0))*(Orari!$F$6:$F$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2440,51 +2432,51 @@
           <t>martedì 13 ottobre 2026</t>
         </is>
       </c>
-      <c r="B16" s="5">
+      <c r="B16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(9,30,0))*(Orari!$H$6:$H$15&gt;TIME(9,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(9,30,0))*(Orari!$J$6:$J$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C16" s="5">
+      <c r="C16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(10,30,0))*(Orari!$H$6:$H$15&gt;TIME(10,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(10,30,0))*(Orari!$J$6:$J$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D16" s="5">
+      <c r="D16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(11,30,0))*(Orari!$H$6:$H$15&gt;TIME(11,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(11,30,0))*(Orari!$J$6:$J$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(12,30,0))*(Orari!$H$6:$H$15&gt;TIME(12,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(12,30,0))*(Orari!$J$6:$J$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F16" s="5">
+      <c r="F16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(13,30,0))*(Orari!$H$6:$H$15&gt;TIME(13,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(13,30,0))*(Orari!$J$6:$J$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G16" s="5">
+      <c r="G16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(14,30,0))*(Orari!$H$6:$H$15&gt;TIME(14,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(14,30,0))*(Orari!$J$6:$J$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H16" s="5">
+      <c r="H16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(15,30,0))*(Orari!$H$6:$H$15&gt;TIME(15,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(15,30,0))*(Orari!$J$6:$J$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I16" s="5">
+      <c r="I16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(16,30,0))*(Orari!$H$6:$H$15&gt;TIME(16,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(16,30,0))*(Orari!$J$6:$J$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J16" s="5">
+      <c r="J16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(17,30,0))*(Orari!$H$6:$H$15&gt;TIME(17,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(17,30,0))*(Orari!$J$6:$J$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K16" s="5">
+      <c r="K16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(18,30,0))*(Orari!$H$6:$H$15&gt;TIME(18,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(18,30,0))*(Orari!$J$6:$J$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L16" s="5">
+      <c r="L16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(19,30,0))*(Orari!$H$6:$H$15&gt;TIME(19,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(19,30,0))*(Orari!$J$6:$J$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M16" s="5">
+      <c r="M16" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(20,30,0))*(Orari!$H$6:$H$15&gt;TIME(20,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(20,30,0))*(Orari!$J$6:$J$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2495,51 +2487,51 @@
           <t>mercoledì 14 ottobre 2026</t>
         </is>
       </c>
-      <c r="B17" s="5">
+      <c r="B17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(9,30,0))*(Orari!$L$6:$L$15&gt;TIME(9,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(9,30,0))*(Orari!$N$6:$N$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C17" s="5">
+      <c r="C17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(10,30,0))*(Orari!$L$6:$L$15&gt;TIME(10,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(10,30,0))*(Orari!$N$6:$N$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D17" s="5">
+      <c r="D17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(11,30,0))*(Orari!$L$6:$L$15&gt;TIME(11,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(11,30,0))*(Orari!$N$6:$N$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E17" s="5">
+      <c r="E17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(12,30,0))*(Orari!$L$6:$L$15&gt;TIME(12,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(12,30,0))*(Orari!$N$6:$N$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F17" s="5">
+      <c r="F17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(13,30,0))*(Orari!$L$6:$L$15&gt;TIME(13,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(13,30,0))*(Orari!$N$6:$N$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G17" s="5">
+      <c r="G17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(14,30,0))*(Orari!$L$6:$L$15&gt;TIME(14,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(14,30,0))*(Orari!$N$6:$N$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H17" s="5">
+      <c r="H17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(15,30,0))*(Orari!$L$6:$L$15&gt;TIME(15,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(15,30,0))*(Orari!$N$6:$N$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I17" s="5">
+      <c r="I17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(16,30,0))*(Orari!$L$6:$L$15&gt;TIME(16,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(16,30,0))*(Orari!$N$6:$N$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J17" s="5">
+      <c r="J17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(17,30,0))*(Orari!$L$6:$L$15&gt;TIME(17,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(17,30,0))*(Orari!$N$6:$N$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K17" s="5">
+      <c r="K17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(18,30,0))*(Orari!$L$6:$L$15&gt;TIME(18,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(18,30,0))*(Orari!$N$6:$N$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L17" s="5">
+      <c r="L17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(19,30,0))*(Orari!$L$6:$L$15&gt;TIME(19,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(19,30,0))*(Orari!$N$6:$N$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M17" s="5">
+      <c r="M17" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(20,30,0))*(Orari!$L$6:$L$15&gt;TIME(20,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(20,30,0))*(Orari!$N$6:$N$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2550,51 +2542,51 @@
           <t>giovedì 15 ottobre 2026</t>
         </is>
       </c>
-      <c r="B18" s="5">
+      <c r="B18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(9,30,0))*(Orari!$P$6:$P$15&gt;TIME(9,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(9,30,0))*(Orari!$R$6:$R$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C18" s="5">
+      <c r="C18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(10,30,0))*(Orari!$P$6:$P$15&gt;TIME(10,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(10,30,0))*(Orari!$R$6:$R$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D18" s="5">
+      <c r="D18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(11,30,0))*(Orari!$P$6:$P$15&gt;TIME(11,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(11,30,0))*(Orari!$R$6:$R$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E18" s="5">
+      <c r="E18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(12,30,0))*(Orari!$P$6:$P$15&gt;TIME(12,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(12,30,0))*(Orari!$R$6:$R$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F18" s="5">
+      <c r="F18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(13,30,0))*(Orari!$P$6:$P$15&gt;TIME(13,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(13,30,0))*(Orari!$R$6:$R$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G18" s="5">
+      <c r="G18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(14,30,0))*(Orari!$P$6:$P$15&gt;TIME(14,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(14,30,0))*(Orari!$R$6:$R$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H18" s="5">
+      <c r="H18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(15,30,0))*(Orari!$P$6:$P$15&gt;TIME(15,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(15,30,0))*(Orari!$R$6:$R$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I18" s="5">
+      <c r="I18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(16,30,0))*(Orari!$P$6:$P$15&gt;TIME(16,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(16,30,0))*(Orari!$R$6:$R$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J18" s="5">
+      <c r="J18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(17,30,0))*(Orari!$P$6:$P$15&gt;TIME(17,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(17,30,0))*(Orari!$R$6:$R$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K18" s="5">
+      <c r="K18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(18,30,0))*(Orari!$P$6:$P$15&gt;TIME(18,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(18,30,0))*(Orari!$R$6:$R$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L18" s="5">
+      <c r="L18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(19,30,0))*(Orari!$P$6:$P$15&gt;TIME(19,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(19,30,0))*(Orari!$R$6:$R$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M18" s="5">
+      <c r="M18" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(20,30,0))*(Orari!$P$6:$P$15&gt;TIME(20,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(20,30,0))*(Orari!$R$6:$R$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2605,51 +2597,51 @@
           <t>venerdì 16 ottobre 2026</t>
         </is>
       </c>
-      <c r="B19" s="5">
+      <c r="B19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(9,30,0))*(Orari!$T$6:$T$15&gt;TIME(9,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(9,30,0))*(Orari!$V$6:$V$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C19" s="5">
+      <c r="C19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(10,30,0))*(Orari!$T$6:$T$15&gt;TIME(10,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(10,30,0))*(Orari!$V$6:$V$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D19" s="5">
+      <c r="D19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(11,30,0))*(Orari!$T$6:$T$15&gt;TIME(11,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(11,30,0))*(Orari!$V$6:$V$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E19" s="5">
+      <c r="E19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(12,30,0))*(Orari!$T$6:$T$15&gt;TIME(12,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(12,30,0))*(Orari!$V$6:$V$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F19" s="5">
+      <c r="F19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(13,30,0))*(Orari!$T$6:$T$15&gt;TIME(13,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(13,30,0))*(Orari!$V$6:$V$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G19" s="5">
+      <c r="G19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(14,30,0))*(Orari!$T$6:$T$15&gt;TIME(14,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(14,30,0))*(Orari!$V$6:$V$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H19" s="5">
+      <c r="H19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(15,30,0))*(Orari!$T$6:$T$15&gt;TIME(15,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(15,30,0))*(Orari!$V$6:$V$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I19" s="5">
+      <c r="I19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(16,30,0))*(Orari!$T$6:$T$15&gt;TIME(16,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(16,30,0))*(Orari!$V$6:$V$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J19" s="5">
+      <c r="J19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(17,30,0))*(Orari!$T$6:$T$15&gt;TIME(17,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(17,30,0))*(Orari!$V$6:$V$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K19" s="5">
+      <c r="K19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(18,30,0))*(Orari!$T$6:$T$15&gt;TIME(18,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(18,30,0))*(Orari!$V$6:$V$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L19" s="5">
+      <c r="L19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(19,30,0))*(Orari!$T$6:$T$15&gt;TIME(19,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(19,30,0))*(Orari!$V$6:$V$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M19" s="5">
+      <c r="M19" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(20,30,0))*(Orari!$T$6:$T$15&gt;TIME(20,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(20,30,0))*(Orari!$V$6:$V$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2660,51 +2652,51 @@
           <t>sabato 17 ottobre 2026</t>
         </is>
       </c>
-      <c r="B20" s="5">
+      <c r="B20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(9,30,0))*(Orari!$X$6:$X$15&gt;TIME(9,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(9,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C20" s="5">
+      <c r="C20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(10,30,0))*(Orari!$X$6:$X$15&gt;TIME(10,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(10,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D20" s="5">
+      <c r="D20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(11,30,0))*(Orari!$X$6:$X$15&gt;TIME(11,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(11,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E20" s="5">
+      <c r="E20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(12,30,0))*(Orari!$X$6:$X$15&gt;TIME(12,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(12,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F20" s="5">
+      <c r="F20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(13,30,0))*(Orari!$X$6:$X$15&gt;TIME(13,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(13,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G20" s="5">
+      <c r="G20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(14,30,0))*(Orari!$X$6:$X$15&gt;TIME(14,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(14,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H20" s="5">
+      <c r="H20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(15,30,0))*(Orari!$X$6:$X$15&gt;TIME(15,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(15,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I20" s="5">
+      <c r="I20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(16,30,0))*(Orari!$X$6:$X$15&gt;TIME(16,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(16,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J20" s="5">
+      <c r="J20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(17,30,0))*(Orari!$X$6:$X$15&gt;TIME(17,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(17,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K20" s="5">
+      <c r="K20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(18,30,0))*(Orari!$X$6:$X$15&gt;TIME(18,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(18,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L20" s="5">
+      <c r="L20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(19,30,0))*(Orari!$X$6:$X$15&gt;TIME(19,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(19,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M20" s="5">
+      <c r="M20" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(20,30,0))*(Orari!$X$6:$X$15&gt;TIME(20,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(20,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2715,51 +2707,51 @@
           <t>domenica 18 ottobre 2026</t>
         </is>
       </c>
-      <c r="B21" s="5">
+      <c r="B21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(9,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(9,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(9,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C21" s="5">
+      <c r="C21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(10,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(10,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(10,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D21" s="5">
+      <c r="D21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(11,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(11,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(11,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E21" s="5">
+      <c r="E21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(12,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(12,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(12,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F21" s="5">
+      <c r="F21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(13,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(13,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(13,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G21" s="5">
+      <c r="G21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(14,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(14,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(14,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H21" s="5">
+      <c r="H21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(15,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(15,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(15,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I21" s="5">
+      <c r="I21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(16,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(16,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(16,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J21" s="5">
+      <c r="J21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(17,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(17,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(17,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K21" s="5">
+      <c r="K21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(18,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(18,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(18,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L21" s="5">
+      <c r="L21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(19,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(19,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(19,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M21" s="5">
+      <c r="M21" s="7">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(20,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(20,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(20,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2844,51 +2836,51 @@
           <t>lunedì 12 ottobre 2026</t>
         </is>
       </c>
-      <c r="B25" s="5">
+      <c r="B25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(9,30,0))*(Orari!$D$6:$D$15&gt;TIME(9,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(9,30,0))*(Orari!$F$6:$F$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C25" s="5">
+      <c r="C25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(10,30,0))*(Orari!$D$6:$D$15&gt;TIME(10,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(10,30,0))*(Orari!$F$6:$F$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D25" s="5">
+      <c r="D25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(11,30,0))*(Orari!$D$6:$D$15&gt;TIME(11,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(11,30,0))*(Orari!$F$6:$F$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E25" s="5">
+      <c r="E25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(12,30,0))*(Orari!$D$6:$D$15&gt;TIME(12,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(12,30,0))*(Orari!$F$6:$F$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F25" s="5">
+      <c r="F25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(13,30,0))*(Orari!$D$6:$D$15&gt;TIME(13,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(13,30,0))*(Orari!$F$6:$F$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G25" s="5">
+      <c r="G25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(14,30,0))*(Orari!$D$6:$D$15&gt;TIME(14,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(14,30,0))*(Orari!$F$6:$F$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H25" s="5">
+      <c r="H25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(15,30,0))*(Orari!$D$6:$D$15&gt;TIME(15,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(15,30,0))*(Orari!$F$6:$F$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I25" s="5">
+      <c r="I25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(16,30,0))*(Orari!$D$6:$D$15&gt;TIME(16,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(16,30,0))*(Orari!$F$6:$F$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J25" s="5">
+      <c r="J25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(17,30,0))*(Orari!$D$6:$D$15&gt;TIME(17,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(17,30,0))*(Orari!$F$6:$F$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K25" s="5">
+      <c r="K25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(18,30,0))*(Orari!$D$6:$D$15&gt;TIME(18,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(18,30,0))*(Orari!$F$6:$F$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L25" s="5">
+      <c r="L25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(19,30,0))*(Orari!$D$6:$D$15&gt;TIME(19,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(19,30,0))*(Orari!$F$6:$F$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M25" s="5">
+      <c r="M25" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(20,30,0))*(Orari!$D$6:$D$15&gt;TIME(20,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(20,30,0))*(Orari!$F$6:$F$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2899,51 +2891,51 @@
           <t>martedì 13 ottobre 2026</t>
         </is>
       </c>
-      <c r="B26" s="5">
+      <c r="B26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(9,30,0))*(Orari!$H$6:$H$15&gt;TIME(9,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(9,30,0))*(Orari!$J$6:$J$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C26" s="5">
+      <c r="C26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(10,30,0))*(Orari!$H$6:$H$15&gt;TIME(10,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(10,30,0))*(Orari!$J$6:$J$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D26" s="5">
+      <c r="D26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(11,30,0))*(Orari!$H$6:$H$15&gt;TIME(11,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(11,30,0))*(Orari!$J$6:$J$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E26" s="5">
+      <c r="E26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(12,30,0))*(Orari!$H$6:$H$15&gt;TIME(12,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(12,30,0))*(Orari!$J$6:$J$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F26" s="5">
+      <c r="F26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(13,30,0))*(Orari!$H$6:$H$15&gt;TIME(13,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(13,30,0))*(Orari!$J$6:$J$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G26" s="5">
+      <c r="G26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(14,30,0))*(Orari!$H$6:$H$15&gt;TIME(14,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(14,30,0))*(Orari!$J$6:$J$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H26" s="5">
+      <c r="H26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(15,30,0))*(Orari!$H$6:$H$15&gt;TIME(15,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(15,30,0))*(Orari!$J$6:$J$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I26" s="5">
+      <c r="I26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(16,30,0))*(Orari!$H$6:$H$15&gt;TIME(16,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(16,30,0))*(Orari!$J$6:$J$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J26" s="5">
+      <c r="J26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(17,30,0))*(Orari!$H$6:$H$15&gt;TIME(17,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(17,30,0))*(Orari!$J$6:$J$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K26" s="5">
+      <c r="K26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(18,30,0))*(Orari!$H$6:$H$15&gt;TIME(18,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(18,30,0))*(Orari!$J$6:$J$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L26" s="5">
+      <c r="L26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(19,30,0))*(Orari!$H$6:$H$15&gt;TIME(19,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(19,30,0))*(Orari!$J$6:$J$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M26" s="5">
+      <c r="M26" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(20,30,0))*(Orari!$H$6:$H$15&gt;TIME(20,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(20,30,0))*(Orari!$J$6:$J$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2954,51 +2946,51 @@
           <t>mercoledì 14 ottobre 2026</t>
         </is>
       </c>
-      <c r="B27" s="5">
+      <c r="B27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(9,30,0))*(Orari!$L$6:$L$15&gt;TIME(9,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(9,30,0))*(Orari!$N$6:$N$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C27" s="5">
+      <c r="C27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(10,30,0))*(Orari!$L$6:$L$15&gt;TIME(10,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(10,30,0))*(Orari!$N$6:$N$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D27" s="5">
+      <c r="D27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(11,30,0))*(Orari!$L$6:$L$15&gt;TIME(11,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(11,30,0))*(Orari!$N$6:$N$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E27" s="5">
+      <c r="E27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(12,30,0))*(Orari!$L$6:$L$15&gt;TIME(12,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(12,30,0))*(Orari!$N$6:$N$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F27" s="5">
+      <c r="F27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(13,30,0))*(Orari!$L$6:$L$15&gt;TIME(13,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(13,30,0))*(Orari!$N$6:$N$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G27" s="5">
+      <c r="G27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(14,30,0))*(Orari!$L$6:$L$15&gt;TIME(14,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(14,30,0))*(Orari!$N$6:$N$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H27" s="5">
+      <c r="H27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(15,30,0))*(Orari!$L$6:$L$15&gt;TIME(15,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(15,30,0))*(Orari!$N$6:$N$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I27" s="5">
+      <c r="I27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(16,30,0))*(Orari!$L$6:$L$15&gt;TIME(16,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(16,30,0))*(Orari!$N$6:$N$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J27" s="5">
+      <c r="J27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(17,30,0))*(Orari!$L$6:$L$15&gt;TIME(17,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(17,30,0))*(Orari!$N$6:$N$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K27" s="5">
+      <c r="K27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(18,30,0))*(Orari!$L$6:$L$15&gt;TIME(18,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(18,30,0))*(Orari!$N$6:$N$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L27" s="5">
+      <c r="L27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(19,30,0))*(Orari!$L$6:$L$15&gt;TIME(19,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(19,30,0))*(Orari!$N$6:$N$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M27" s="5">
+      <c r="M27" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(20,30,0))*(Orari!$L$6:$L$15&gt;TIME(20,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(20,30,0))*(Orari!$N$6:$N$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -3009,51 +3001,51 @@
           <t>giovedì 15 ottobre 2026</t>
         </is>
       </c>
-      <c r="B28" s="5">
+      <c r="B28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(9,30,0))*(Orari!$P$6:$P$15&gt;TIME(9,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(9,30,0))*(Orari!$R$6:$R$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C28" s="5">
+      <c r="C28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(10,30,0))*(Orari!$P$6:$P$15&gt;TIME(10,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(10,30,0))*(Orari!$R$6:$R$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D28" s="5">
+      <c r="D28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(11,30,0))*(Orari!$P$6:$P$15&gt;TIME(11,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(11,30,0))*(Orari!$R$6:$R$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E28" s="5">
+      <c r="E28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(12,30,0))*(Orari!$P$6:$P$15&gt;TIME(12,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(12,30,0))*(Orari!$R$6:$R$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F28" s="5">
+      <c r="F28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(13,30,0))*(Orari!$P$6:$P$15&gt;TIME(13,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(13,30,0))*(Orari!$R$6:$R$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G28" s="5">
+      <c r="G28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(14,30,0))*(Orari!$P$6:$P$15&gt;TIME(14,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(14,30,0))*(Orari!$R$6:$R$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H28" s="5">
+      <c r="H28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(15,30,0))*(Orari!$P$6:$P$15&gt;TIME(15,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(15,30,0))*(Orari!$R$6:$R$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I28" s="5">
+      <c r="I28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(16,30,0))*(Orari!$P$6:$P$15&gt;TIME(16,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(16,30,0))*(Orari!$R$6:$R$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J28" s="5">
+      <c r="J28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(17,30,0))*(Orari!$P$6:$P$15&gt;TIME(17,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(17,30,0))*(Orari!$R$6:$R$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K28" s="5">
+      <c r="K28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(18,30,0))*(Orari!$P$6:$P$15&gt;TIME(18,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(18,30,0))*(Orari!$R$6:$R$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L28" s="5">
+      <c r="L28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(19,30,0))*(Orari!$P$6:$P$15&gt;TIME(19,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(19,30,0))*(Orari!$R$6:$R$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M28" s="5">
+      <c r="M28" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(20,30,0))*(Orari!$P$6:$P$15&gt;TIME(20,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(20,30,0))*(Orari!$R$6:$R$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -3064,51 +3056,51 @@
           <t>venerdì 16 ottobre 2026</t>
         </is>
       </c>
-      <c r="B29" s="5">
+      <c r="B29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(9,30,0))*(Orari!$T$6:$T$15&gt;TIME(9,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(9,30,0))*(Orari!$V$6:$V$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C29" s="5">
+      <c r="C29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(10,30,0))*(Orari!$T$6:$T$15&gt;TIME(10,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(10,30,0))*(Orari!$V$6:$V$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D29" s="5">
+      <c r="D29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(11,30,0))*(Orari!$T$6:$T$15&gt;TIME(11,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(11,30,0))*(Orari!$V$6:$V$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E29" s="5">
+      <c r="E29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(12,30,0))*(Orari!$T$6:$T$15&gt;TIME(12,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(12,30,0))*(Orari!$V$6:$V$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F29" s="5">
+      <c r="F29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(13,30,0))*(Orari!$T$6:$T$15&gt;TIME(13,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(13,30,0))*(Orari!$V$6:$V$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G29" s="5">
+      <c r="G29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(14,30,0))*(Orari!$T$6:$T$15&gt;TIME(14,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(14,30,0))*(Orari!$V$6:$V$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H29" s="5">
+      <c r="H29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(15,30,0))*(Orari!$T$6:$T$15&gt;TIME(15,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(15,30,0))*(Orari!$V$6:$V$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I29" s="5">
+      <c r="I29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(16,30,0))*(Orari!$T$6:$T$15&gt;TIME(16,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(16,30,0))*(Orari!$V$6:$V$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J29" s="5">
+      <c r="J29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(17,30,0))*(Orari!$T$6:$T$15&gt;TIME(17,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(17,30,0))*(Orari!$V$6:$V$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K29" s="5">
+      <c r="K29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(18,30,0))*(Orari!$T$6:$T$15&gt;TIME(18,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(18,30,0))*(Orari!$V$6:$V$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L29" s="5">
+      <c r="L29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(19,30,0))*(Orari!$T$6:$T$15&gt;TIME(19,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(19,30,0))*(Orari!$V$6:$V$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M29" s="5">
+      <c r="M29" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(20,30,0))*(Orari!$T$6:$T$15&gt;TIME(20,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(20,30,0))*(Orari!$V$6:$V$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -3119,51 +3111,51 @@
           <t>sabato 17 ottobre 2026</t>
         </is>
       </c>
-      <c r="B30" s="5">
+      <c r="B30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(9,30,0))*(Orari!$X$6:$X$15&gt;TIME(9,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(9,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C30" s="5">
+      <c r="C30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(10,30,0))*(Orari!$X$6:$X$15&gt;TIME(10,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(10,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D30" s="5">
+      <c r="D30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(11,30,0))*(Orari!$X$6:$X$15&gt;TIME(11,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(11,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E30" s="5">
+      <c r="E30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(12,30,0))*(Orari!$X$6:$X$15&gt;TIME(12,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(12,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F30" s="5">
+      <c r="F30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(13,30,0))*(Orari!$X$6:$X$15&gt;TIME(13,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(13,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G30" s="5">
+      <c r="G30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(14,30,0))*(Orari!$X$6:$X$15&gt;TIME(14,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(14,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H30" s="5">
+      <c r="H30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(15,30,0))*(Orari!$X$6:$X$15&gt;TIME(15,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(15,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I30" s="5">
+      <c r="I30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(16,30,0))*(Orari!$X$6:$X$15&gt;TIME(16,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(16,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J30" s="5">
+      <c r="J30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(17,30,0))*(Orari!$X$6:$X$15&gt;TIME(17,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(17,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K30" s="5">
+      <c r="K30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(18,30,0))*(Orari!$X$6:$X$15&gt;TIME(18,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(18,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L30" s="5">
+      <c r="L30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(19,30,0))*(Orari!$X$6:$X$15&gt;TIME(19,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(19,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M30" s="5">
+      <c r="M30" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(20,30,0))*(Orari!$X$6:$X$15&gt;TIME(20,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(20,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -3174,51 +3166,51 @@
           <t>domenica 18 ottobre 2026</t>
         </is>
       </c>
-      <c r="B31" s="5">
+      <c r="B31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(9,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(9,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(9,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C31" s="5">
+      <c r="C31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(10,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(10,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(10,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D31" s="5">
+      <c r="D31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(11,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(11,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(11,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E31" s="5">
+      <c r="E31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(12,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(12,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(12,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F31" s="5">
+      <c r="F31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(13,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(13,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(13,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G31" s="5">
+      <c r="G31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(14,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(14,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(14,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H31" s="5">
+      <c r="H31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(15,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(15,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(15,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I31" s="5">
+      <c r="I31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(16,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(16,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(16,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J31" s="5">
+      <c r="J31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(17,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(17,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(17,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K31" s="5">
+      <c r="K31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(18,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(18,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(18,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L31" s="5">
+      <c r="L31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(19,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(19,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(19,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M31" s="5">
+      <c r="M31" s="7">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(20,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(20,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(20,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Orari: niente mezze giornate la domenica
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RgW8tUpL59m5j1P2CKTdxn
</commit_message>
<xml_diff>
--- a/orari/Orari_12-18_ottobre_2026.xlsx
+++ b/orari/Orari_12-18_ottobre_2026.xlsx
@@ -104,13 +104,13 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -877,71 +877,71 @@
           <t>Addetto vendite</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="5" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="6" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="H6" s="6" t="n">
-        <v>0.625</v>
-      </c>
+      <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
       <c r="J6" s="7" t="n"/>
-      <c r="K6" s="7" t="n"/>
-      <c r="L6" s="7" t="n"/>
-      <c r="M6" s="6" t="n">
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="6" t="n"/>
+      <c r="M6" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="N6" s="6" t="n">
+      <c r="N6" s="5" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="O6" s="5" t="inlineStr">
+      <c r="O6" s="6" t="n"/>
+      <c r="P6" s="6" t="n"/>
+      <c r="Q6" s="5" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="R6" s="5" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="S6" s="5" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="T6" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="U6" s="6" t="n"/>
+      <c r="V6" s="6" t="n"/>
+      <c r="W6" s="5" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="X6" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="Y6" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="Z6" s="5" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="AA6" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="P6" s="5" t="n"/>
-      <c r="Q6" s="5" t="n"/>
-      <c r="R6" s="5" t="n"/>
-      <c r="S6" s="7" t="n"/>
-      <c r="T6" s="7" t="n"/>
-      <c r="U6" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="V6" s="6" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="W6" s="6" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="X6" s="6" t="n">
-        <v>0.5416666666666666</v>
-      </c>
-      <c r="Y6" s="6" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="Z6" s="6" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="AA6" s="6" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="AB6" s="6" t="n">
-        <v>0.625</v>
-      </c>
+      <c r="AB6" s="7" t="n"/>
       <c r="AC6" s="7" t="n"/>
       <c r="AD6" s="7" t="n"/>
       <c r="AE6" s="8">
         <f>ROUND(24*(N(D6)-N(C6)+N(F6)-N(E6)+N(H6)-N(G6)+N(J6)-N(I6)+N(L6)-N(K6)+N(N6)-N(M6)+N(P6)-N(O6)+N(R6)-N(Q6)+N(T6)-N(S6)+N(V6)-N(U6)+N(X6)-N(W6)+N(Z6)-N(Y6)+N(AB6)-N(AA6)+N(AD6)-N(AC6)),2)</f>
         <v/>
       </c>
-      <c r="AF6" s="7" t="n">
+      <c r="AF6" s="6" t="n">
         <v>30</v>
       </c>
     </row>
@@ -956,83 +956,83 @@
           <t>Vicedirettore</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="5" t="n">
         <v>0.4166666666666667</v>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="H7" s="5" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="E7" s="6" t="n">
+      <c r="I7" s="5" t="n">
         <v>0.7083333333333334</v>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="J7" s="5" t="n">
         <v>0.875</v>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="n"/>
+      <c r="M7" s="7" t="n"/>
+      <c r="N7" s="7" t="n"/>
+      <c r="O7" s="5" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="P7" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="Q7" s="5" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="R7" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="S7" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="T7" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="I7" s="7" t="n"/>
-      <c r="J7" s="7" t="n"/>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="L7" s="5" t="n"/>
-      <c r="M7" s="5" t="n"/>
-      <c r="N7" s="5" t="n"/>
-      <c r="O7" s="6" t="n">
+      <c r="U7" s="6" t="n"/>
+      <c r="V7" s="6" t="n"/>
+      <c r="W7" s="5" t="n">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="X7" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="Y7" s="5" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="Z7" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="AA7" s="5" t="n">
         <v>0.4166666666666667</v>
       </c>
-      <c r="P7" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="Q7" s="6" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="R7" s="6" t="n">
+      <c r="AB7" s="5" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="AC7" s="5" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="AD7" s="5" t="n">
         <v>0.875</v>
-      </c>
-      <c r="S7" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="T7" s="5" t="n"/>
-      <c r="U7" s="5" t="n"/>
-      <c r="V7" s="5" t="n"/>
-      <c r="W7" s="6" t="n">
-        <v>0.4583333333333333</v>
-      </c>
-      <c r="X7" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="Y7" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="Z7" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="AA7" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="AB7" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="AC7" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="AD7" s="6" t="n">
-        <v>0.8333333333333334</v>
       </c>
       <c r="AE7" s="8">
         <f>ROUND(24*(N(D7)-N(C7)+N(F7)-N(E7)+N(H7)-N(G7)+N(J7)-N(I7)+N(L7)-N(K7)+N(N7)-N(M7)+N(P7)-N(O7)+N(R7)-N(Q7)+N(T7)-N(S7)+N(V7)-N(U7)+N(X7)-N(W7)+N(Z7)-N(Y7)+N(AB7)-N(AA7)+N(AD7)-N(AC7)),2)</f>
         <v/>
       </c>
-      <c r="AF7" s="7" t="inlineStr">
+      <c r="AF7" s="6" t="inlineStr">
         <is>
           <t>44-45</t>
         </is>
@@ -1049,79 +1049,79 @@
           <t>Addetto vendite</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="L8" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="M8" s="6" t="n"/>
+      <c r="N8" s="6" t="n"/>
+      <c r="O8" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="7" t="n"/>
-      <c r="H8" s="7" t="n"/>
-      <c r="I8" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="J8" s="6" t="n">
+      <c r="P8" s="7" t="n"/>
+      <c r="Q8" s="7" t="n"/>
+      <c r="R8" s="7" t="n"/>
+      <c r="S8" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="T8" s="7" t="n"/>
+      <c r="U8" s="7" t="n"/>
+      <c r="V8" s="7" t="n"/>
+      <c r="W8" s="5" t="n">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="X8" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="Y8" s="5" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="Z8" s="5" t="n">
         <v>0.875</v>
       </c>
-      <c r="K8" s="6" t="n">
+      <c r="AA8" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="L8" s="6" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="M8" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="N8" s="6" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="O8" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="P8" s="5" t="n"/>
-      <c r="Q8" s="5" t="n"/>
-      <c r="R8" s="5" t="n"/>
-      <c r="S8" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="T8" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="U8" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="V8" s="6" t="n">
+      <c r="AB8" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AC8" s="5" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="AD8" s="5" t="n">
         <v>0.7916666666666666</v>
-      </c>
-      <c r="W8" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="X8" s="6" t="n">
-        <v>0.5416666666666666</v>
-      </c>
-      <c r="Y8" s="6" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="Z8" s="6" t="n">
-        <v>0.7916666666666666</v>
-      </c>
-      <c r="AA8" s="7" t="n"/>
-      <c r="AB8" s="7" t="n"/>
-      <c r="AC8" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="AD8" s="6" t="n">
-        <v>0.875</v>
       </c>
       <c r="AE8" s="8">
         <f>ROUND(24*(N(D8)-N(C8)+N(F8)-N(E8)+N(H8)-N(G8)+N(J8)-N(I8)+N(L8)-N(K8)+N(N8)-N(M8)+N(P8)-N(O8)+N(R8)-N(Q8)+N(T8)-N(S8)+N(V8)-N(U8)+N(X8)-N(W8)+N(Z8)-N(Y8)+N(AB8)-N(AA8)+N(AD8)-N(AC8)),2)</f>
         <v/>
       </c>
-      <c r="AF8" s="7" t="n">
+      <c r="AF8" s="6" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1136,79 +1136,79 @@
           <t>Addetto vendite</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="7" t="n"/>
+      <c r="K9" s="5" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="M9" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="N9" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="O9" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="P9" s="7" t="n"/>
+      <c r="Q9" s="7" t="n"/>
+      <c r="R9" s="7" t="n"/>
+      <c r="S9" s="6" t="n"/>
+      <c r="T9" s="6" t="n"/>
+      <c r="U9" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="V9" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="W9" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="X9" s="5" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="Y9" s="5" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="Z9" s="5" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="AA9" s="5" t="n">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="AB9" s="5" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="AC9" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="E9" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>0.7916666666666666</v>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="6" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="L9" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="M9" s="6" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="N9" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="O9" s="7" t="n"/>
-      <c r="P9" s="7" t="n"/>
-      <c r="Q9" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="R9" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="S9" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="T9" s="5" t="n"/>
-      <c r="U9" s="5" t="n"/>
-      <c r="V9" s="5" t="n"/>
-      <c r="W9" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="X9" s="6" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Y9" s="6" t="n">
-        <v>0.5416666666666666</v>
-      </c>
-      <c r="Z9" s="6" t="n">
-        <v>0.7916666666666666</v>
-      </c>
-      <c r="AA9" s="7" t="n"/>
-      <c r="AB9" s="7" t="n"/>
-      <c r="AC9" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="AD9" s="6" t="n">
+      <c r="AD9" s="5" t="n">
         <v>0.875</v>
       </c>
       <c r="AE9" s="8">
         <f>ROUND(24*(N(D9)-N(C9)+N(F9)-N(E9)+N(H9)-N(G9)+N(J9)-N(I9)+N(L9)-N(K9)+N(N9)-N(M9)+N(P9)-N(O9)+N(R9)-N(Q9)+N(T9)-N(S9)+N(V9)-N(U9)+N(X9)-N(W9)+N(Z9)-N(Y9)+N(AB9)-N(AA9)+N(AD9)-N(AC9)),2)</f>
         <v/>
       </c>
-      <c r="AF9" s="7" t="n">
+      <c r="AF9" s="6" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1223,79 +1223,79 @@
           <t>Addetto vendite</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="6" t="n">
+      <c r="C10" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="D10" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="F10" s="6" t="n">
+      <c r="E10" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="J10" s="5" t="n">
         <v>0.875</v>
       </c>
-      <c r="G10" s="7" t="n"/>
-      <c r="H10" s="7" t="n"/>
-      <c r="I10" s="6" t="n">
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="L10" s="7" t="n"/>
+      <c r="M10" s="7" t="n"/>
+      <c r="N10" s="7" t="n"/>
+      <c r="O10" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="P10" s="5" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="Q10" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="J10" s="6" t="n">
+      <c r="R10" s="5" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="S10" s="6" t="n"/>
+      <c r="T10" s="6" t="n"/>
+      <c r="U10" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="V10" s="5" t="n">
         <v>0.875</v>
       </c>
-      <c r="K10" s="5" t="inlineStr">
+      <c r="W10" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="X10" s="5" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="Y10" s="5" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="Z10" s="5" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="AA10" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="L10" s="5" t="n"/>
-      <c r="M10" s="5" t="n"/>
-      <c r="N10" s="5" t="n"/>
-      <c r="O10" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="P10" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="Q10" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="R10" s="6" t="n">
-        <v>0.7916666666666666</v>
-      </c>
-      <c r="S10" s="6" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="T10" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="U10" s="6" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="V10" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="W10" s="6" t="n">
-        <v>0.4583333333333333</v>
-      </c>
-      <c r="X10" s="6" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="Y10" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="Z10" s="6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="AA10" s="5" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="AB10" s="5" t="n"/>
-      <c r="AC10" s="5" t="n"/>
-      <c r="AD10" s="5" t="n"/>
+      <c r="AB10" s="7" t="n"/>
+      <c r="AC10" s="7" t="n"/>
+      <c r="AD10" s="7" t="n"/>
       <c r="AE10" s="8">
         <f>ROUND(24*(N(D10)-N(C10)+N(F10)-N(E10)+N(H10)-N(G10)+N(J10)-N(I10)+N(L10)-N(K10)+N(N10)-N(M10)+N(P10)-N(O10)+N(R10)-N(Q10)+N(T10)-N(S10)+N(V10)-N(U10)+N(X10)-N(W10)+N(Z10)-N(Y10)+N(AB10)-N(AA10)+N(AD10)-N(AC10)),2)</f>
         <v/>
       </c>
-      <c r="AF10" s="7" t="n">
+      <c r="AF10" s="6" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1310,83 +1310,83 @@
           <t>Cassiera</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C11" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="D11" s="6" t="n">
+      <c r="D11" s="5" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="E11" s="6" t="n">
+      <c r="E11" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="5" t="n">
         <v>0.7083333333333334</v>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="5" t="n"/>
-      <c r="K11" s="6" t="n">
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="7" t="n"/>
+      <c r="J11" s="7" t="n"/>
+      <c r="K11" s="5" t="n">
         <v>0.4166666666666667</v>
       </c>
-      <c r="L11" s="6" t="n">
+      <c r="L11" s="5" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="M11" s="6" t="n">
+      <c r="M11" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="N11" s="6" t="n">
+      <c r="N11" s="5" t="n">
         <v>0.875</v>
       </c>
-      <c r="O11" s="6" t="n">
+      <c r="O11" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="P11" s="6" t="n">
+      <c r="P11" s="5" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="Q11" s="6" t="n">
+      <c r="Q11" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="R11" s="6" t="n">
+      <c r="R11" s="5" t="n">
         <v>0.75</v>
       </c>
-      <c r="S11" s="6" t="n">
+      <c r="S11" s="5" t="n">
         <v>0.4583333333333333</v>
       </c>
-      <c r="T11" s="6" t="n">
+      <c r="T11" s="5" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="U11" s="6" t="n">
+      <c r="U11" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="V11" s="6" t="n">
+      <c r="V11" s="5" t="n">
         <v>0.875</v>
       </c>
-      <c r="W11" s="6" t="n">
+      <c r="W11" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="X11" s="6" t="n">
+      <c r="X11" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="Y11" s="7" t="n"/>
-      <c r="Z11" s="7" t="n"/>
-      <c r="AA11" s="5" t="inlineStr">
+      <c r="Y11" s="6" t="n"/>
+      <c r="Z11" s="6" t="n"/>
+      <c r="AA11" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="AB11" s="5" t="n"/>
-      <c r="AC11" s="5" t="n"/>
-      <c r="AD11" s="5" t="n"/>
+      <c r="AB11" s="7" t="n"/>
+      <c r="AC11" s="7" t="n"/>
+      <c r="AD11" s="7" t="n"/>
       <c r="AE11" s="8">
         <f>ROUND(24*(N(D11)-N(C11)+N(F11)-N(E11)+N(H11)-N(G11)+N(J11)-N(I11)+N(L11)-N(K11)+N(N11)-N(M11)+N(P11)-N(O11)+N(R11)-N(Q11)+N(T11)-N(S11)+N(V11)-N(U11)+N(X11)-N(W11)+N(Z11)-N(Y11)+N(AB11)-N(AA11)+N(AD11)-N(AC11)),2)</f>
         <v/>
       </c>
-      <c r="AF11" s="7" t="n">
+      <c r="AF11" s="6" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1401,71 +1401,71 @@
           <t>Cassiera</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="6" t="n">
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="5" t="n">
         <v>0.7083333333333334</v>
       </c>
-      <c r="F12" s="6" t="n">
+      <c r="F12" s="5" t="n">
         <v>0.875</v>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="G12" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="H12" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="I12" s="7" t="n"/>
-      <c r="J12" s="7" t="n"/>
-      <c r="K12" s="5" t="inlineStr">
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="n"/>
+      <c r="K12" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="L12" s="5" t="n"/>
-      <c r="M12" s="5" t="n"/>
-      <c r="N12" s="5" t="n"/>
-      <c r="O12" s="5" t="inlineStr">
+      <c r="L12" s="7" t="n"/>
+      <c r="M12" s="7" t="n"/>
+      <c r="N12" s="7" t="n"/>
+      <c r="O12" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="P12" s="5" t="n"/>
-      <c r="Q12" s="5" t="n"/>
-      <c r="R12" s="5" t="n"/>
-      <c r="S12" s="6" t="n">
+      <c r="P12" s="7" t="n"/>
+      <c r="Q12" s="7" t="n"/>
+      <c r="R12" s="7" t="n"/>
+      <c r="S12" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="T12" s="6" t="n">
+      <c r="T12" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="U12" s="7" t="n"/>
-      <c r="V12" s="7" t="n"/>
-      <c r="W12" s="5" t="inlineStr">
+      <c r="U12" s="6" t="n"/>
+      <c r="V12" s="6" t="n"/>
+      <c r="W12" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="X12" s="5" t="n"/>
-      <c r="Y12" s="5" t="n"/>
-      <c r="Z12" s="5" t="n"/>
-      <c r="AA12" s="6" t="n">
+      <c r="X12" s="7" t="n"/>
+      <c r="Y12" s="7" t="n"/>
+      <c r="Z12" s="7" t="n"/>
+      <c r="AA12" s="5" t="n">
         <v>0.4166666666666667</v>
       </c>
-      <c r="AB12" s="6" t="n">
+      <c r="AB12" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="AC12" s="6" t="n">
+      <c r="AC12" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="AD12" s="6" t="n">
+      <c r="AD12" s="5" t="n">
         <v>0.875</v>
       </c>
       <c r="AE12" s="8">
         <f>ROUND(24*(N(D12)-N(C12)+N(F12)-N(E12)+N(H12)-N(G12)+N(J12)-N(I12)+N(L12)-N(K12)+N(N12)-N(M12)+N(P12)-N(O12)+N(R12)-N(Q12)+N(T12)-N(S12)+N(V12)-N(U12)+N(X12)-N(W12)+N(Z12)-N(Y12)+N(AB12)-N(AA12)+N(AD12)-N(AC12)),2)</f>
         <v/>
       </c>
-      <c r="AF12" s="7" t="n">
+      <c r="AF12" s="6" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1480,67 +1480,67 @@
           <t>Cassiera</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="7" t="n"/>
-      <c r="H13" s="7" t="n"/>
-      <c r="I13" s="6" t="n">
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="J13" s="6" t="n">
+      <c r="J13" s="5" t="n">
         <v>0.875</v>
       </c>
-      <c r="K13" s="6" t="n">
+      <c r="K13" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="L13" s="6" t="n">
+      <c r="L13" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="M13" s="7" t="n"/>
-      <c r="N13" s="7" t="n"/>
-      <c r="O13" s="6" t="n">
+      <c r="M13" s="6" t="n"/>
+      <c r="N13" s="6" t="n"/>
+      <c r="O13" s="5" t="n">
         <v>0.4166666666666667</v>
       </c>
-      <c r="P13" s="6" t="n">
+      <c r="P13" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="Q13" s="7" t="n"/>
-      <c r="R13" s="7" t="n"/>
-      <c r="S13" s="7" t="n"/>
-      <c r="T13" s="7" t="n"/>
-      <c r="U13" s="6" t="n">
+      <c r="Q13" s="6" t="n"/>
+      <c r="R13" s="6" t="n"/>
+      <c r="S13" s="6" t="n"/>
+      <c r="T13" s="6" t="n"/>
+      <c r="U13" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="V13" s="6" t="n">
+      <c r="V13" s="5" t="n">
         <v>0.7916666666666666</v>
       </c>
-      <c r="W13" s="7" t="n"/>
-      <c r="X13" s="7" t="n"/>
-      <c r="Y13" s="6" t="n">
+      <c r="W13" s="6" t="n"/>
+      <c r="X13" s="6" t="n"/>
+      <c r="Y13" s="5" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="Z13" s="6" t="n">
+      <c r="Z13" s="5" t="n">
         <v>0.875</v>
       </c>
-      <c r="AA13" s="5" t="inlineStr">
+      <c r="AA13" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="AB13" s="5" t="n"/>
-      <c r="AC13" s="5" t="n"/>
-      <c r="AD13" s="5" t="n"/>
+      <c r="AB13" s="7" t="n"/>
+      <c r="AC13" s="7" t="n"/>
+      <c r="AD13" s="7" t="n"/>
       <c r="AE13" s="8">
         <f>ROUND(24*(N(D13)-N(C13)+N(F13)-N(E13)+N(H13)-N(G13)+N(J13)-N(I13)+N(L13)-N(K13)+N(N13)-N(M13)+N(P13)-N(O13)+N(R13)-N(Q13)+N(T13)-N(S13)+N(V13)-N(U13)+N(X13)-N(W13)+N(Z13)-N(Y13)+N(AB13)-N(AA13)+N(AD13)-N(AC13)),2)</f>
         <v/>
       </c>
-      <c r="AF13" s="7" t="n">
+      <c r="AF13" s="6" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1555,71 +1555,71 @@
           <t>Cassiera</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C14" s="5" t="n">
         <v>0.4583333333333333</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D14" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="7" t="n"/>
-      <c r="G14" s="7" t="n"/>
-      <c r="H14" s="7" t="n"/>
-      <c r="I14" s="6" t="n">
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="J14" s="6" t="n">
+      <c r="J14" s="5" t="n">
         <v>0.75</v>
       </c>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="K14" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="L14" s="5" t="n"/>
-      <c r="M14" s="5" t="n"/>
-      <c r="N14" s="5" t="n"/>
-      <c r="O14" s="7" t="n"/>
-      <c r="P14" s="7" t="n"/>
-      <c r="Q14" s="6" t="n">
+      <c r="L14" s="7" t="n"/>
+      <c r="M14" s="7" t="n"/>
+      <c r="N14" s="7" t="n"/>
+      <c r="O14" s="6" t="n"/>
+      <c r="P14" s="6" t="n"/>
+      <c r="Q14" s="5" t="n">
         <v>0.7083333333333334</v>
       </c>
-      <c r="R14" s="6" t="n">
+      <c r="R14" s="5" t="n">
         <v>0.875</v>
       </c>
-      <c r="S14" s="5" t="inlineStr">
+      <c r="S14" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="T14" s="5" t="n"/>
-      <c r="U14" s="5" t="n"/>
-      <c r="V14" s="5" t="n"/>
-      <c r="W14" s="7" t="n"/>
-      <c r="X14" s="7" t="n"/>
-      <c r="Y14" s="6" t="n">
+      <c r="T14" s="7" t="n"/>
+      <c r="U14" s="7" t="n"/>
+      <c r="V14" s="7" t="n"/>
+      <c r="W14" s="6" t="n"/>
+      <c r="X14" s="6" t="n"/>
+      <c r="Y14" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="Z14" s="6" t="n">
+      <c r="Z14" s="5" t="n">
         <v>0.7916666666666666</v>
       </c>
-      <c r="AA14" s="6" t="n">
+      <c r="AA14" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="AB14" s="6" t="n">
+      <c r="AB14" s="5" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="AC14" s="6" t="n">
+      <c r="AC14" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="AD14" s="6" t="n">
+      <c r="AD14" s="5" t="n">
         <v>0.7916666666666666</v>
       </c>
       <c r="AE14" s="8">
         <f>ROUND(24*(N(D14)-N(C14)+N(F14)-N(E14)+N(H14)-N(G14)+N(J14)-N(I14)+N(L14)-N(K14)+N(N14)-N(M14)+N(P14)-N(O14)+N(R14)-N(Q14)+N(T14)-N(S14)+N(V14)-N(U14)+N(X14)-N(W14)+N(Z14)-N(Y14)+N(AB14)-N(AA14)+N(AD14)-N(AC14)),2)</f>
         <v/>
       </c>
-      <c r="AF14" s="7" t="n">
+      <c r="AF14" s="6" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1634,87 +1634,87 @@
           <t>Magazziniere</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="C15" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="D15" s="6" t="n">
+      <c r="D15" s="5" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="E15" s="6" t="n">
+      <c r="E15" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="F15" s="6" t="n">
+      <c r="F15" s="5" t="n">
         <v>0.75</v>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="G15" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="H15" s="6" t="n">
+      <c r="H15" s="5" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="I15" s="6" t="n">
+      <c r="I15" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="J15" s="6" t="n">
+      <c r="J15" s="5" t="n">
         <v>0.75</v>
       </c>
-      <c r="K15" s="6" t="n">
+      <c r="K15" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="L15" s="6" t="n">
+      <c r="L15" s="5" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="M15" s="6" t="n">
+      <c r="M15" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="N15" s="6" t="n">
+      <c r="N15" s="5" t="n">
         <v>0.75</v>
       </c>
-      <c r="O15" s="6" t="n">
+      <c r="O15" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="P15" s="6" t="n">
+      <c r="P15" s="5" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="Q15" s="6" t="n">
+      <c r="Q15" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="R15" s="6" t="n">
+      <c r="R15" s="5" t="n">
         <v>0.75</v>
       </c>
-      <c r="S15" s="6" t="n">
+      <c r="S15" s="5" t="n">
         <v>0.375</v>
       </c>
-      <c r="T15" s="6" t="n">
+      <c r="T15" s="5" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="U15" s="6" t="n">
+      <c r="U15" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="V15" s="6" t="n">
+      <c r="V15" s="5" t="n">
         <v>0.75</v>
       </c>
-      <c r="W15" s="5" t="inlineStr">
+      <c r="W15" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="X15" s="5" t="n"/>
-      <c r="Y15" s="5" t="n"/>
-      <c r="Z15" s="5" t="n"/>
-      <c r="AA15" s="5" t="inlineStr">
+      <c r="X15" s="7" t="n"/>
+      <c r="Y15" s="7" t="n"/>
+      <c r="Z15" s="7" t="n"/>
+      <c r="AA15" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="AB15" s="5" t="n"/>
-      <c r="AC15" s="5" t="n"/>
-      <c r="AD15" s="5" t="n"/>
+      <c r="AB15" s="7" t="n"/>
+      <c r="AC15" s="7" t="n"/>
+      <c r="AD15" s="7" t="n"/>
       <c r="AE15" s="8">
         <f>ROUND(24*(N(D15)-N(C15)+N(F15)-N(E15)+N(H15)-N(G15)+N(J15)-N(I15)+N(L15)-N(K15)+N(N15)-N(M15)+N(P15)-N(O15)+N(R15)-N(Q15)+N(T15)-N(S15)+N(V15)-N(U15)+N(X15)-N(W15)+N(Z15)-N(Y15)+N(AB15)-N(AA15)+N(AD15)-N(AC15)),2)</f>
         <v/>
       </c>
-      <c r="AF15" s="7" t="n">
+      <c r="AF15" s="6" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Sabato giornata intera per tutto il reparto; il terzo addetto di reparto messo di preferenza al pomeriggio.</t>
+          <t>Sabato giornata intera per tutto il reparto, domenica niente mezze giornate; il terzo addetto di reparto messo di preferenza al pomeriggio.</t>
         </is>
       </c>
     </row>
@@ -1756,13 +1756,12 @@
   </sheetData>
   <mergeCells count="46">
     <mergeCell ref="W4:X4"/>
-    <mergeCell ref="S9:V9"/>
     <mergeCell ref="Y4:Z4"/>
     <mergeCell ref="K14:N14"/>
-    <mergeCell ref="C8:F8"/>
     <mergeCell ref="O12:R12"/>
     <mergeCell ref="O8:R8"/>
     <mergeCell ref="AA3:AD3"/>
+    <mergeCell ref="C7:F7"/>
     <mergeCell ref="K7:N7"/>
     <mergeCell ref="K10:N10"/>
     <mergeCell ref="AA11:AD11"/>
@@ -1773,24 +1772,25 @@
     <mergeCell ref="C3:F3"/>
     <mergeCell ref="K3:N3"/>
     <mergeCell ref="O3:R3"/>
-    <mergeCell ref="C6:F6"/>
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="G11:J11"/>
-    <mergeCell ref="O6:R6"/>
+    <mergeCell ref="AA10:AD10"/>
     <mergeCell ref="O4:P4"/>
-    <mergeCell ref="AA10:AD10"/>
+    <mergeCell ref="W15:Z15"/>
     <mergeCell ref="AA4:AB4"/>
     <mergeCell ref="Q4:R4"/>
-    <mergeCell ref="W15:Z15"/>
     <mergeCell ref="AC4:AD4"/>
     <mergeCell ref="AF3:AF5"/>
+    <mergeCell ref="O9:R9"/>
     <mergeCell ref="AA13:AD13"/>
     <mergeCell ref="S3:V3"/>
+    <mergeCell ref="S8:V8"/>
     <mergeCell ref="AE3:AE5"/>
-    <mergeCell ref="S7:V7"/>
+    <mergeCell ref="AA6:AD6"/>
     <mergeCell ref="AA15:AD15"/>
     <mergeCell ref="S14:V14"/>
     <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G6:J6"/>
     <mergeCell ref="I4:J4"/>
     <mergeCell ref="W3:Z3"/>
     <mergeCell ref="G3:J3"/>
@@ -1918,51 +1918,51 @@
           <t>lunedì 12 ottobre 2026</t>
         </is>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(9,30,0))*(Orari!$D$6:$D$15&gt;TIME(9,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(9,30,0))*(Orari!$F$6:$F$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(10,30,0))*(Orari!$D$6:$D$15&gt;TIME(10,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(10,30,0))*(Orari!$F$6:$F$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(11,30,0))*(Orari!$D$6:$D$15&gt;TIME(11,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(11,30,0))*(Orari!$F$6:$F$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(12,30,0))*(Orari!$D$6:$D$15&gt;TIME(12,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(12,30,0))*(Orari!$F$6:$F$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(13,30,0))*(Orari!$D$6:$D$15&gt;TIME(13,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(13,30,0))*(Orari!$F$6:$F$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(14,30,0))*(Orari!$D$6:$D$15&gt;TIME(14,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(14,30,0))*(Orari!$F$6:$F$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(15,30,0))*(Orari!$D$6:$D$15&gt;TIME(15,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(15,30,0))*(Orari!$F$6:$F$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(16,30,0))*(Orari!$D$6:$D$15&gt;TIME(16,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(16,30,0))*(Orari!$F$6:$F$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J5" s="7">
+      <c r="J5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(17,30,0))*(Orari!$D$6:$D$15&gt;TIME(17,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(17,30,0))*(Orari!$F$6:$F$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K5" s="7">
+      <c r="K5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(18,30,0))*(Orari!$D$6:$D$15&gt;TIME(18,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(18,30,0))*(Orari!$F$6:$F$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L5" s="7">
+      <c r="L5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(19,30,0))*(Orari!$D$6:$D$15&gt;TIME(19,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(19,30,0))*(Orari!$F$6:$F$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M5" s="7">
+      <c r="M5" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$C$6:$C$15&lt;=TIME(20,30,0))*(Orari!$D$6:$D$15&gt;TIME(20,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(20,30,0))*(Orari!$F$6:$F$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -1973,51 +1973,51 @@
           <t>martedì 13 ottobre 2026</t>
         </is>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(9,30,0))*(Orari!$H$6:$H$15&gt;TIME(9,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(9,30,0))*(Orari!$J$6:$J$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(10,30,0))*(Orari!$H$6:$H$15&gt;TIME(10,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(10,30,0))*(Orari!$J$6:$J$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(11,30,0))*(Orari!$H$6:$H$15&gt;TIME(11,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(11,30,0))*(Orari!$J$6:$J$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(12,30,0))*(Orari!$H$6:$H$15&gt;TIME(12,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(12,30,0))*(Orari!$J$6:$J$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(13,30,0))*(Orari!$H$6:$H$15&gt;TIME(13,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(13,30,0))*(Orari!$J$6:$J$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(14,30,0))*(Orari!$H$6:$H$15&gt;TIME(14,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(14,30,0))*(Orari!$J$6:$J$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(15,30,0))*(Orari!$H$6:$H$15&gt;TIME(15,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(15,30,0))*(Orari!$J$6:$J$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(16,30,0))*(Orari!$H$6:$H$15&gt;TIME(16,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(16,30,0))*(Orari!$J$6:$J$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J6" s="7">
+      <c r="J6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(17,30,0))*(Orari!$H$6:$H$15&gt;TIME(17,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(17,30,0))*(Orari!$J$6:$J$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K6" s="7">
+      <c r="K6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(18,30,0))*(Orari!$H$6:$H$15&gt;TIME(18,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(18,30,0))*(Orari!$J$6:$J$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L6" s="7">
+      <c r="L6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(19,30,0))*(Orari!$H$6:$H$15&gt;TIME(19,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(19,30,0))*(Orari!$J$6:$J$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M6" s="7">
+      <c r="M6" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$G$6:$G$15&lt;=TIME(20,30,0))*(Orari!$H$6:$H$15&gt;TIME(20,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(20,30,0))*(Orari!$J$6:$J$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2028,51 +2028,51 @@
           <t>mercoledì 14 ottobre 2026</t>
         </is>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(9,30,0))*(Orari!$L$6:$L$15&gt;TIME(9,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(9,30,0))*(Orari!$N$6:$N$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(10,30,0))*(Orari!$L$6:$L$15&gt;TIME(10,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(10,30,0))*(Orari!$N$6:$N$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(11,30,0))*(Orari!$L$6:$L$15&gt;TIME(11,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(11,30,0))*(Orari!$N$6:$N$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(12,30,0))*(Orari!$L$6:$L$15&gt;TIME(12,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(12,30,0))*(Orari!$N$6:$N$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(13,30,0))*(Orari!$L$6:$L$15&gt;TIME(13,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(13,30,0))*(Orari!$N$6:$N$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(14,30,0))*(Orari!$L$6:$L$15&gt;TIME(14,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(14,30,0))*(Orari!$N$6:$N$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H7" s="7">
+      <c r="H7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(15,30,0))*(Orari!$L$6:$L$15&gt;TIME(15,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(15,30,0))*(Orari!$N$6:$N$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I7" s="7">
+      <c r="I7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(16,30,0))*(Orari!$L$6:$L$15&gt;TIME(16,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(16,30,0))*(Orari!$N$6:$N$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J7" s="7">
+      <c r="J7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(17,30,0))*(Orari!$L$6:$L$15&gt;TIME(17,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(17,30,0))*(Orari!$N$6:$N$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K7" s="7">
+      <c r="K7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(18,30,0))*(Orari!$L$6:$L$15&gt;TIME(18,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(18,30,0))*(Orari!$N$6:$N$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L7" s="7">
+      <c r="L7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(19,30,0))*(Orari!$L$6:$L$15&gt;TIME(19,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(19,30,0))*(Orari!$N$6:$N$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M7" s="7">
+      <c r="M7" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$K$6:$K$15&lt;=TIME(20,30,0))*(Orari!$L$6:$L$15&gt;TIME(20,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(20,30,0))*(Orari!$N$6:$N$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2083,51 +2083,51 @@
           <t>giovedì 15 ottobre 2026</t>
         </is>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(9,30,0))*(Orari!$P$6:$P$15&gt;TIME(9,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(9,30,0))*(Orari!$R$6:$R$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(10,30,0))*(Orari!$P$6:$P$15&gt;TIME(10,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(10,30,0))*(Orari!$R$6:$R$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(11,30,0))*(Orari!$P$6:$P$15&gt;TIME(11,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(11,30,0))*(Orari!$R$6:$R$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(12,30,0))*(Orari!$P$6:$P$15&gt;TIME(12,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(12,30,0))*(Orari!$R$6:$R$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(13,30,0))*(Orari!$P$6:$P$15&gt;TIME(13,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(13,30,0))*(Orari!$R$6:$R$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(14,30,0))*(Orari!$P$6:$P$15&gt;TIME(14,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(14,30,0))*(Orari!$R$6:$R$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(15,30,0))*(Orari!$P$6:$P$15&gt;TIME(15,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(15,30,0))*(Orari!$R$6:$R$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(16,30,0))*(Orari!$P$6:$P$15&gt;TIME(16,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(16,30,0))*(Orari!$R$6:$R$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J8" s="7">
+      <c r="J8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(17,30,0))*(Orari!$P$6:$P$15&gt;TIME(17,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(17,30,0))*(Orari!$R$6:$R$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K8" s="7">
+      <c r="K8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(18,30,0))*(Orari!$P$6:$P$15&gt;TIME(18,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(18,30,0))*(Orari!$R$6:$R$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L8" s="7">
+      <c r="L8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(19,30,0))*(Orari!$P$6:$P$15&gt;TIME(19,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(19,30,0))*(Orari!$R$6:$R$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M8" s="7">
+      <c r="M8" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$O$6:$O$15&lt;=TIME(20,30,0))*(Orari!$P$6:$P$15&gt;TIME(20,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(20,30,0))*(Orari!$R$6:$R$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2138,51 +2138,51 @@
           <t>venerdì 16 ottobre 2026</t>
         </is>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(9,30,0))*(Orari!$T$6:$T$15&gt;TIME(9,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(9,30,0))*(Orari!$V$6:$V$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(10,30,0))*(Orari!$T$6:$T$15&gt;TIME(10,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(10,30,0))*(Orari!$V$6:$V$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(11,30,0))*(Orari!$T$6:$T$15&gt;TIME(11,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(11,30,0))*(Orari!$V$6:$V$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(12,30,0))*(Orari!$T$6:$T$15&gt;TIME(12,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(12,30,0))*(Orari!$V$6:$V$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(13,30,0))*(Orari!$T$6:$T$15&gt;TIME(13,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(13,30,0))*(Orari!$V$6:$V$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(14,30,0))*(Orari!$T$6:$T$15&gt;TIME(14,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(14,30,0))*(Orari!$V$6:$V$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H9" s="7">
+      <c r="H9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(15,30,0))*(Orari!$T$6:$T$15&gt;TIME(15,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(15,30,0))*(Orari!$V$6:$V$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(16,30,0))*(Orari!$T$6:$T$15&gt;TIME(16,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(16,30,0))*(Orari!$V$6:$V$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J9" s="7">
+      <c r="J9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(17,30,0))*(Orari!$T$6:$T$15&gt;TIME(17,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(17,30,0))*(Orari!$V$6:$V$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K9" s="7">
+      <c r="K9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(18,30,0))*(Orari!$T$6:$T$15&gt;TIME(18,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(18,30,0))*(Orari!$V$6:$V$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L9" s="7">
+      <c r="L9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(19,30,0))*(Orari!$T$6:$T$15&gt;TIME(19,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(19,30,0))*(Orari!$V$6:$V$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M9" s="7">
+      <c r="M9" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$S$6:$S$15&lt;=TIME(20,30,0))*(Orari!$T$6:$T$15&gt;TIME(20,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(20,30,0))*(Orari!$V$6:$V$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2193,51 +2193,51 @@
           <t>sabato 17 ottobre 2026</t>
         </is>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(9,30,0))*(Orari!$X$6:$X$15&gt;TIME(9,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(9,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(10,30,0))*(Orari!$X$6:$X$15&gt;TIME(10,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(10,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(11,30,0))*(Orari!$X$6:$X$15&gt;TIME(11,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(11,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(12,30,0))*(Orari!$X$6:$X$15&gt;TIME(12,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(12,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F10" s="7">
+      <c r="F10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(13,30,0))*(Orari!$X$6:$X$15&gt;TIME(13,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(13,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G10" s="7">
+      <c r="G10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(14,30,0))*(Orari!$X$6:$X$15&gt;TIME(14,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(14,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H10" s="7">
+      <c r="H10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(15,30,0))*(Orari!$X$6:$X$15&gt;TIME(15,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(15,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I10" s="7">
+      <c r="I10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(16,30,0))*(Orari!$X$6:$X$15&gt;TIME(16,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(16,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J10" s="7">
+      <c r="J10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(17,30,0))*(Orari!$X$6:$X$15&gt;TIME(17,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(17,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K10" s="7">
+      <c r="K10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(18,30,0))*(Orari!$X$6:$X$15&gt;TIME(18,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(18,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L10" s="7">
+      <c r="L10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(19,30,0))*(Orari!$X$6:$X$15&gt;TIME(19,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(19,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M10" s="7">
+      <c r="M10" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$W$6:$W$15&lt;=TIME(20,30,0))*(Orari!$X$6:$X$15&gt;TIME(20,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(20,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2248,51 +2248,51 @@
           <t>domenica 18 ottobre 2026</t>
         </is>
       </c>
-      <c r="B11" s="7">
+      <c r="B11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(9,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(9,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(9,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(10,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(10,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(10,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(11,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(11,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(11,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(12,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(12,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(12,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F11" s="7">
+      <c r="F11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(13,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(13,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(13,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G11" s="7">
+      <c r="G11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(14,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(14,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(14,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H11" s="7">
+      <c r="H11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(15,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(15,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(15,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(16,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(16,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(16,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J11" s="7">
+      <c r="J11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(17,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(17,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(17,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K11" s="7">
+      <c r="K11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(18,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(18,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(18,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L11" s="7">
+      <c r="L11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(19,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(19,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(19,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M11" s="7">
+      <c r="M11" s="6">
         <f>SUMPRODUCT((((Orari!$B$6:$B$15="Addetto vendite")+(Orari!$B$6:$B$15="Vicedirettore"))&gt;0)*(((Orari!$AA$6:$AA$15&lt;=TIME(20,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(20,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(20,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2377,51 +2377,51 @@
           <t>lunedì 12 ottobre 2026</t>
         </is>
       </c>
-      <c r="B15" s="7">
+      <c r="B15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(9,30,0))*(Orari!$D$6:$D$15&gt;TIME(9,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(9,30,0))*(Orari!$F$6:$F$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C15" s="7">
+      <c r="C15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(10,30,0))*(Orari!$D$6:$D$15&gt;TIME(10,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(10,30,0))*(Orari!$F$6:$F$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D15" s="7">
+      <c r="D15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(11,30,0))*(Orari!$D$6:$D$15&gt;TIME(11,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(11,30,0))*(Orari!$F$6:$F$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E15" s="7">
+      <c r="E15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(12,30,0))*(Orari!$D$6:$D$15&gt;TIME(12,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(12,30,0))*(Orari!$F$6:$F$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F15" s="7">
+      <c r="F15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(13,30,0))*(Orari!$D$6:$D$15&gt;TIME(13,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(13,30,0))*(Orari!$F$6:$F$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G15" s="7">
+      <c r="G15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(14,30,0))*(Orari!$D$6:$D$15&gt;TIME(14,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(14,30,0))*(Orari!$F$6:$F$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H15" s="7">
+      <c r="H15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(15,30,0))*(Orari!$D$6:$D$15&gt;TIME(15,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(15,30,0))*(Orari!$F$6:$F$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I15" s="7">
+      <c r="I15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(16,30,0))*(Orari!$D$6:$D$15&gt;TIME(16,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(16,30,0))*(Orari!$F$6:$F$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J15" s="7">
+      <c r="J15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(17,30,0))*(Orari!$D$6:$D$15&gt;TIME(17,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(17,30,0))*(Orari!$F$6:$F$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K15" s="7">
+      <c r="K15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(18,30,0))*(Orari!$D$6:$D$15&gt;TIME(18,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(18,30,0))*(Orari!$F$6:$F$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L15" s="7">
+      <c r="L15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(19,30,0))*(Orari!$D$6:$D$15&gt;TIME(19,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(19,30,0))*(Orari!$F$6:$F$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M15" s="7">
+      <c r="M15" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$C$6:$C$15&lt;=TIME(20,30,0))*(Orari!$D$6:$D$15&gt;TIME(20,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(20,30,0))*(Orari!$F$6:$F$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2432,51 +2432,51 @@
           <t>martedì 13 ottobre 2026</t>
         </is>
       </c>
-      <c r="B16" s="7">
+      <c r="B16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(9,30,0))*(Orari!$H$6:$H$15&gt;TIME(9,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(9,30,0))*(Orari!$J$6:$J$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C16" s="7">
+      <c r="C16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(10,30,0))*(Orari!$H$6:$H$15&gt;TIME(10,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(10,30,0))*(Orari!$J$6:$J$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D16" s="7">
+      <c r="D16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(11,30,0))*(Orari!$H$6:$H$15&gt;TIME(11,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(11,30,0))*(Orari!$J$6:$J$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E16" s="7">
+      <c r="E16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(12,30,0))*(Orari!$H$6:$H$15&gt;TIME(12,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(12,30,0))*(Orari!$J$6:$J$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F16" s="7">
+      <c r="F16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(13,30,0))*(Orari!$H$6:$H$15&gt;TIME(13,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(13,30,0))*(Orari!$J$6:$J$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G16" s="7">
+      <c r="G16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(14,30,0))*(Orari!$H$6:$H$15&gt;TIME(14,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(14,30,0))*(Orari!$J$6:$J$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H16" s="7">
+      <c r="H16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(15,30,0))*(Orari!$H$6:$H$15&gt;TIME(15,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(15,30,0))*(Orari!$J$6:$J$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I16" s="7">
+      <c r="I16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(16,30,0))*(Orari!$H$6:$H$15&gt;TIME(16,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(16,30,0))*(Orari!$J$6:$J$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J16" s="7">
+      <c r="J16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(17,30,0))*(Orari!$H$6:$H$15&gt;TIME(17,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(17,30,0))*(Orari!$J$6:$J$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K16" s="7">
+      <c r="K16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(18,30,0))*(Orari!$H$6:$H$15&gt;TIME(18,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(18,30,0))*(Orari!$J$6:$J$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L16" s="7">
+      <c r="L16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(19,30,0))*(Orari!$H$6:$H$15&gt;TIME(19,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(19,30,0))*(Orari!$J$6:$J$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M16" s="7">
+      <c r="M16" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$G$6:$G$15&lt;=TIME(20,30,0))*(Orari!$H$6:$H$15&gt;TIME(20,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(20,30,0))*(Orari!$J$6:$J$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2487,51 +2487,51 @@
           <t>mercoledì 14 ottobre 2026</t>
         </is>
       </c>
-      <c r="B17" s="7">
+      <c r="B17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(9,30,0))*(Orari!$L$6:$L$15&gt;TIME(9,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(9,30,0))*(Orari!$N$6:$N$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C17" s="7">
+      <c r="C17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(10,30,0))*(Orari!$L$6:$L$15&gt;TIME(10,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(10,30,0))*(Orari!$N$6:$N$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D17" s="7">
+      <c r="D17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(11,30,0))*(Orari!$L$6:$L$15&gt;TIME(11,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(11,30,0))*(Orari!$N$6:$N$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E17" s="7">
+      <c r="E17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(12,30,0))*(Orari!$L$6:$L$15&gt;TIME(12,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(12,30,0))*(Orari!$N$6:$N$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F17" s="7">
+      <c r="F17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(13,30,0))*(Orari!$L$6:$L$15&gt;TIME(13,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(13,30,0))*(Orari!$N$6:$N$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G17" s="7">
+      <c r="G17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(14,30,0))*(Orari!$L$6:$L$15&gt;TIME(14,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(14,30,0))*(Orari!$N$6:$N$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H17" s="7">
+      <c r="H17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(15,30,0))*(Orari!$L$6:$L$15&gt;TIME(15,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(15,30,0))*(Orari!$N$6:$N$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I17" s="7">
+      <c r="I17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(16,30,0))*(Orari!$L$6:$L$15&gt;TIME(16,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(16,30,0))*(Orari!$N$6:$N$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J17" s="7">
+      <c r="J17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(17,30,0))*(Orari!$L$6:$L$15&gt;TIME(17,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(17,30,0))*(Orari!$N$6:$N$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K17" s="7">
+      <c r="K17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(18,30,0))*(Orari!$L$6:$L$15&gt;TIME(18,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(18,30,0))*(Orari!$N$6:$N$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L17" s="7">
+      <c r="L17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(19,30,0))*(Orari!$L$6:$L$15&gt;TIME(19,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(19,30,0))*(Orari!$N$6:$N$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M17" s="7">
+      <c r="M17" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$K$6:$K$15&lt;=TIME(20,30,0))*(Orari!$L$6:$L$15&gt;TIME(20,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(20,30,0))*(Orari!$N$6:$N$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2542,51 +2542,51 @@
           <t>giovedì 15 ottobre 2026</t>
         </is>
       </c>
-      <c r="B18" s="7">
+      <c r="B18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(9,30,0))*(Orari!$P$6:$P$15&gt;TIME(9,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(9,30,0))*(Orari!$R$6:$R$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C18" s="7">
+      <c r="C18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(10,30,0))*(Orari!$P$6:$P$15&gt;TIME(10,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(10,30,0))*(Orari!$R$6:$R$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D18" s="7">
+      <c r="D18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(11,30,0))*(Orari!$P$6:$P$15&gt;TIME(11,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(11,30,0))*(Orari!$R$6:$R$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E18" s="7">
+      <c r="E18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(12,30,0))*(Orari!$P$6:$P$15&gt;TIME(12,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(12,30,0))*(Orari!$R$6:$R$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F18" s="7">
+      <c r="F18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(13,30,0))*(Orari!$P$6:$P$15&gt;TIME(13,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(13,30,0))*(Orari!$R$6:$R$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G18" s="7">
+      <c r="G18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(14,30,0))*(Orari!$P$6:$P$15&gt;TIME(14,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(14,30,0))*(Orari!$R$6:$R$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H18" s="7">
+      <c r="H18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(15,30,0))*(Orari!$P$6:$P$15&gt;TIME(15,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(15,30,0))*(Orari!$R$6:$R$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I18" s="7">
+      <c r="I18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(16,30,0))*(Orari!$P$6:$P$15&gt;TIME(16,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(16,30,0))*(Orari!$R$6:$R$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J18" s="7">
+      <c r="J18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(17,30,0))*(Orari!$P$6:$P$15&gt;TIME(17,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(17,30,0))*(Orari!$R$6:$R$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K18" s="7">
+      <c r="K18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(18,30,0))*(Orari!$P$6:$P$15&gt;TIME(18,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(18,30,0))*(Orari!$R$6:$R$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L18" s="7">
+      <c r="L18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(19,30,0))*(Orari!$P$6:$P$15&gt;TIME(19,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(19,30,0))*(Orari!$R$6:$R$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M18" s="7">
+      <c r="M18" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$O$6:$O$15&lt;=TIME(20,30,0))*(Orari!$P$6:$P$15&gt;TIME(20,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(20,30,0))*(Orari!$R$6:$R$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2597,51 +2597,51 @@
           <t>venerdì 16 ottobre 2026</t>
         </is>
       </c>
-      <c r="B19" s="7">
+      <c r="B19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(9,30,0))*(Orari!$T$6:$T$15&gt;TIME(9,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(9,30,0))*(Orari!$V$6:$V$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C19" s="7">
+      <c r="C19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(10,30,0))*(Orari!$T$6:$T$15&gt;TIME(10,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(10,30,0))*(Orari!$V$6:$V$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D19" s="7">
+      <c r="D19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(11,30,0))*(Orari!$T$6:$T$15&gt;TIME(11,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(11,30,0))*(Orari!$V$6:$V$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E19" s="7">
+      <c r="E19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(12,30,0))*(Orari!$T$6:$T$15&gt;TIME(12,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(12,30,0))*(Orari!$V$6:$V$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F19" s="7">
+      <c r="F19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(13,30,0))*(Orari!$T$6:$T$15&gt;TIME(13,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(13,30,0))*(Orari!$V$6:$V$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G19" s="7">
+      <c r="G19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(14,30,0))*(Orari!$T$6:$T$15&gt;TIME(14,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(14,30,0))*(Orari!$V$6:$V$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H19" s="7">
+      <c r="H19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(15,30,0))*(Orari!$T$6:$T$15&gt;TIME(15,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(15,30,0))*(Orari!$V$6:$V$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I19" s="7">
+      <c r="I19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(16,30,0))*(Orari!$T$6:$T$15&gt;TIME(16,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(16,30,0))*(Orari!$V$6:$V$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J19" s="7">
+      <c r="J19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(17,30,0))*(Orari!$T$6:$T$15&gt;TIME(17,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(17,30,0))*(Orari!$V$6:$V$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K19" s="7">
+      <c r="K19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(18,30,0))*(Orari!$T$6:$T$15&gt;TIME(18,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(18,30,0))*(Orari!$V$6:$V$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L19" s="7">
+      <c r="L19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(19,30,0))*(Orari!$T$6:$T$15&gt;TIME(19,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(19,30,0))*(Orari!$V$6:$V$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M19" s="7">
+      <c r="M19" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$S$6:$S$15&lt;=TIME(20,30,0))*(Orari!$T$6:$T$15&gt;TIME(20,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(20,30,0))*(Orari!$V$6:$V$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2652,51 +2652,51 @@
           <t>sabato 17 ottobre 2026</t>
         </is>
       </c>
-      <c r="B20" s="7">
+      <c r="B20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(9,30,0))*(Orari!$X$6:$X$15&gt;TIME(9,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(9,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C20" s="7">
+      <c r="C20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(10,30,0))*(Orari!$X$6:$X$15&gt;TIME(10,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(10,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D20" s="7">
+      <c r="D20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(11,30,0))*(Orari!$X$6:$X$15&gt;TIME(11,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(11,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E20" s="7">
+      <c r="E20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(12,30,0))*(Orari!$X$6:$X$15&gt;TIME(12,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(12,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F20" s="7">
+      <c r="F20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(13,30,0))*(Orari!$X$6:$X$15&gt;TIME(13,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(13,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G20" s="7">
+      <c r="G20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(14,30,0))*(Orari!$X$6:$X$15&gt;TIME(14,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(14,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H20" s="7">
+      <c r="H20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(15,30,0))*(Orari!$X$6:$X$15&gt;TIME(15,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(15,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I20" s="7">
+      <c r="I20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(16,30,0))*(Orari!$X$6:$X$15&gt;TIME(16,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(16,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J20" s="7">
+      <c r="J20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(17,30,0))*(Orari!$X$6:$X$15&gt;TIME(17,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(17,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K20" s="7">
+      <c r="K20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(18,30,0))*(Orari!$X$6:$X$15&gt;TIME(18,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(18,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L20" s="7">
+      <c r="L20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(19,30,0))*(Orari!$X$6:$X$15&gt;TIME(19,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(19,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M20" s="7">
+      <c r="M20" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$W$6:$W$15&lt;=TIME(20,30,0))*(Orari!$X$6:$X$15&gt;TIME(20,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(20,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2707,51 +2707,51 @@
           <t>domenica 18 ottobre 2026</t>
         </is>
       </c>
-      <c r="B21" s="7">
+      <c r="B21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(9,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(9,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(9,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C21" s="7">
+      <c r="C21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(10,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(10,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(10,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D21" s="7">
+      <c r="D21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(11,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(11,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(11,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E21" s="7">
+      <c r="E21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(12,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(12,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(12,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F21" s="7">
+      <c r="F21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(13,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(13,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(13,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G21" s="7">
+      <c r="G21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(14,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(14,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(14,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H21" s="7">
+      <c r="H21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(15,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(15,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(15,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I21" s="7">
+      <c r="I21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(16,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(16,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(16,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J21" s="7">
+      <c r="J21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(17,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(17,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(17,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K21" s="7">
+      <c r="K21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(18,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(18,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(18,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L21" s="7">
+      <c r="L21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(19,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(19,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(19,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M21" s="7">
+      <c r="M21" s="6">
         <f>SUMPRODUCT((Orari!$B$6:$B$15="Cassiera")*(((Orari!$AA$6:$AA$15&lt;=TIME(20,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(20,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(20,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2836,51 +2836,51 @@
           <t>lunedì 12 ottobre 2026</t>
         </is>
       </c>
-      <c r="B25" s="7">
+      <c r="B25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(9,30,0))*(Orari!$D$6:$D$15&gt;TIME(9,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(9,30,0))*(Orari!$F$6:$F$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C25" s="7">
+      <c r="C25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(10,30,0))*(Orari!$D$6:$D$15&gt;TIME(10,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(10,30,0))*(Orari!$F$6:$F$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D25" s="7">
+      <c r="D25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(11,30,0))*(Orari!$D$6:$D$15&gt;TIME(11,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(11,30,0))*(Orari!$F$6:$F$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E25" s="7">
+      <c r="E25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(12,30,0))*(Orari!$D$6:$D$15&gt;TIME(12,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(12,30,0))*(Orari!$F$6:$F$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F25" s="7">
+      <c r="F25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(13,30,0))*(Orari!$D$6:$D$15&gt;TIME(13,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(13,30,0))*(Orari!$F$6:$F$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G25" s="7">
+      <c r="G25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(14,30,0))*(Orari!$D$6:$D$15&gt;TIME(14,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(14,30,0))*(Orari!$F$6:$F$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H25" s="7">
+      <c r="H25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(15,30,0))*(Orari!$D$6:$D$15&gt;TIME(15,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(15,30,0))*(Orari!$F$6:$F$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I25" s="7">
+      <c r="I25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(16,30,0))*(Orari!$D$6:$D$15&gt;TIME(16,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(16,30,0))*(Orari!$F$6:$F$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J25" s="7">
+      <c r="J25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(17,30,0))*(Orari!$D$6:$D$15&gt;TIME(17,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(17,30,0))*(Orari!$F$6:$F$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K25" s="7">
+      <c r="K25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(18,30,0))*(Orari!$D$6:$D$15&gt;TIME(18,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(18,30,0))*(Orari!$F$6:$F$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L25" s="7">
+      <c r="L25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(19,30,0))*(Orari!$D$6:$D$15&gt;TIME(19,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(19,30,0))*(Orari!$F$6:$F$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M25" s="7">
+      <c r="M25" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$C$6:$C$15&lt;=TIME(20,30,0))*(Orari!$D$6:$D$15&gt;TIME(20,30,0)))+((Orari!$E$6:$E$15&lt;=TIME(20,30,0))*(Orari!$F$6:$F$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2891,51 +2891,51 @@
           <t>martedì 13 ottobre 2026</t>
         </is>
       </c>
-      <c r="B26" s="7">
+      <c r="B26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(9,30,0))*(Orari!$H$6:$H$15&gt;TIME(9,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(9,30,0))*(Orari!$J$6:$J$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C26" s="7">
+      <c r="C26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(10,30,0))*(Orari!$H$6:$H$15&gt;TIME(10,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(10,30,0))*(Orari!$J$6:$J$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D26" s="7">
+      <c r="D26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(11,30,0))*(Orari!$H$6:$H$15&gt;TIME(11,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(11,30,0))*(Orari!$J$6:$J$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E26" s="7">
+      <c r="E26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(12,30,0))*(Orari!$H$6:$H$15&gt;TIME(12,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(12,30,0))*(Orari!$J$6:$J$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F26" s="7">
+      <c r="F26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(13,30,0))*(Orari!$H$6:$H$15&gt;TIME(13,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(13,30,0))*(Orari!$J$6:$J$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G26" s="7">
+      <c r="G26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(14,30,0))*(Orari!$H$6:$H$15&gt;TIME(14,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(14,30,0))*(Orari!$J$6:$J$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H26" s="7">
+      <c r="H26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(15,30,0))*(Orari!$H$6:$H$15&gt;TIME(15,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(15,30,0))*(Orari!$J$6:$J$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I26" s="7">
+      <c r="I26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(16,30,0))*(Orari!$H$6:$H$15&gt;TIME(16,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(16,30,0))*(Orari!$J$6:$J$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J26" s="7">
+      <c r="J26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(17,30,0))*(Orari!$H$6:$H$15&gt;TIME(17,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(17,30,0))*(Orari!$J$6:$J$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K26" s="7">
+      <c r="K26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(18,30,0))*(Orari!$H$6:$H$15&gt;TIME(18,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(18,30,0))*(Orari!$J$6:$J$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L26" s="7">
+      <c r="L26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(19,30,0))*(Orari!$H$6:$H$15&gt;TIME(19,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(19,30,0))*(Orari!$J$6:$J$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M26" s="7">
+      <c r="M26" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$G$6:$G$15&lt;=TIME(20,30,0))*(Orari!$H$6:$H$15&gt;TIME(20,30,0)))+((Orari!$I$6:$I$15&lt;=TIME(20,30,0))*(Orari!$J$6:$J$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -2946,51 +2946,51 @@
           <t>mercoledì 14 ottobre 2026</t>
         </is>
       </c>
-      <c r="B27" s="7">
+      <c r="B27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(9,30,0))*(Orari!$L$6:$L$15&gt;TIME(9,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(9,30,0))*(Orari!$N$6:$N$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C27" s="7">
+      <c r="C27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(10,30,0))*(Orari!$L$6:$L$15&gt;TIME(10,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(10,30,0))*(Orari!$N$6:$N$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D27" s="7">
+      <c r="D27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(11,30,0))*(Orari!$L$6:$L$15&gt;TIME(11,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(11,30,0))*(Orari!$N$6:$N$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E27" s="7">
+      <c r="E27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(12,30,0))*(Orari!$L$6:$L$15&gt;TIME(12,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(12,30,0))*(Orari!$N$6:$N$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F27" s="7">
+      <c r="F27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(13,30,0))*(Orari!$L$6:$L$15&gt;TIME(13,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(13,30,0))*(Orari!$N$6:$N$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G27" s="7">
+      <c r="G27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(14,30,0))*(Orari!$L$6:$L$15&gt;TIME(14,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(14,30,0))*(Orari!$N$6:$N$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H27" s="7">
+      <c r="H27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(15,30,0))*(Orari!$L$6:$L$15&gt;TIME(15,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(15,30,0))*(Orari!$N$6:$N$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I27" s="7">
+      <c r="I27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(16,30,0))*(Orari!$L$6:$L$15&gt;TIME(16,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(16,30,0))*(Orari!$N$6:$N$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J27" s="7">
+      <c r="J27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(17,30,0))*(Orari!$L$6:$L$15&gt;TIME(17,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(17,30,0))*(Orari!$N$6:$N$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K27" s="7">
+      <c r="K27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(18,30,0))*(Orari!$L$6:$L$15&gt;TIME(18,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(18,30,0))*(Orari!$N$6:$N$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L27" s="7">
+      <c r="L27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(19,30,0))*(Orari!$L$6:$L$15&gt;TIME(19,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(19,30,0))*(Orari!$N$6:$N$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M27" s="7">
+      <c r="M27" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$K$6:$K$15&lt;=TIME(20,30,0))*(Orari!$L$6:$L$15&gt;TIME(20,30,0)))+((Orari!$M$6:$M$15&lt;=TIME(20,30,0))*(Orari!$N$6:$N$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -3001,51 +3001,51 @@
           <t>giovedì 15 ottobre 2026</t>
         </is>
       </c>
-      <c r="B28" s="7">
+      <c r="B28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(9,30,0))*(Orari!$P$6:$P$15&gt;TIME(9,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(9,30,0))*(Orari!$R$6:$R$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C28" s="7">
+      <c r="C28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(10,30,0))*(Orari!$P$6:$P$15&gt;TIME(10,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(10,30,0))*(Orari!$R$6:$R$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D28" s="7">
+      <c r="D28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(11,30,0))*(Orari!$P$6:$P$15&gt;TIME(11,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(11,30,0))*(Orari!$R$6:$R$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E28" s="7">
+      <c r="E28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(12,30,0))*(Orari!$P$6:$P$15&gt;TIME(12,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(12,30,0))*(Orari!$R$6:$R$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F28" s="7">
+      <c r="F28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(13,30,0))*(Orari!$P$6:$P$15&gt;TIME(13,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(13,30,0))*(Orari!$R$6:$R$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G28" s="7">
+      <c r="G28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(14,30,0))*(Orari!$P$6:$P$15&gt;TIME(14,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(14,30,0))*(Orari!$R$6:$R$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H28" s="7">
+      <c r="H28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(15,30,0))*(Orari!$P$6:$P$15&gt;TIME(15,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(15,30,0))*(Orari!$R$6:$R$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I28" s="7">
+      <c r="I28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(16,30,0))*(Orari!$P$6:$P$15&gt;TIME(16,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(16,30,0))*(Orari!$R$6:$R$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J28" s="7">
+      <c r="J28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(17,30,0))*(Orari!$P$6:$P$15&gt;TIME(17,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(17,30,0))*(Orari!$R$6:$R$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K28" s="7">
+      <c r="K28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(18,30,0))*(Orari!$P$6:$P$15&gt;TIME(18,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(18,30,0))*(Orari!$R$6:$R$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L28" s="7">
+      <c r="L28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(19,30,0))*(Orari!$P$6:$P$15&gt;TIME(19,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(19,30,0))*(Orari!$R$6:$R$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M28" s="7">
+      <c r="M28" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$O$6:$O$15&lt;=TIME(20,30,0))*(Orari!$P$6:$P$15&gt;TIME(20,30,0)))+((Orari!$Q$6:$Q$15&lt;=TIME(20,30,0))*(Orari!$R$6:$R$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -3056,51 +3056,51 @@
           <t>venerdì 16 ottobre 2026</t>
         </is>
       </c>
-      <c r="B29" s="7">
+      <c r="B29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(9,30,0))*(Orari!$T$6:$T$15&gt;TIME(9,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(9,30,0))*(Orari!$V$6:$V$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C29" s="7">
+      <c r="C29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(10,30,0))*(Orari!$T$6:$T$15&gt;TIME(10,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(10,30,0))*(Orari!$V$6:$V$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D29" s="7">
+      <c r="D29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(11,30,0))*(Orari!$T$6:$T$15&gt;TIME(11,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(11,30,0))*(Orari!$V$6:$V$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E29" s="7">
+      <c r="E29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(12,30,0))*(Orari!$T$6:$T$15&gt;TIME(12,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(12,30,0))*(Orari!$V$6:$V$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F29" s="7">
+      <c r="F29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(13,30,0))*(Orari!$T$6:$T$15&gt;TIME(13,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(13,30,0))*(Orari!$V$6:$V$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G29" s="7">
+      <c r="G29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(14,30,0))*(Orari!$T$6:$T$15&gt;TIME(14,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(14,30,0))*(Orari!$V$6:$V$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H29" s="7">
+      <c r="H29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(15,30,0))*(Orari!$T$6:$T$15&gt;TIME(15,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(15,30,0))*(Orari!$V$6:$V$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I29" s="7">
+      <c r="I29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(16,30,0))*(Orari!$T$6:$T$15&gt;TIME(16,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(16,30,0))*(Orari!$V$6:$V$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J29" s="7">
+      <c r="J29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(17,30,0))*(Orari!$T$6:$T$15&gt;TIME(17,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(17,30,0))*(Orari!$V$6:$V$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K29" s="7">
+      <c r="K29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(18,30,0))*(Orari!$T$6:$T$15&gt;TIME(18,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(18,30,0))*(Orari!$V$6:$V$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L29" s="7">
+      <c r="L29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(19,30,0))*(Orari!$T$6:$T$15&gt;TIME(19,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(19,30,0))*(Orari!$V$6:$V$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M29" s="7">
+      <c r="M29" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$S$6:$S$15&lt;=TIME(20,30,0))*(Orari!$T$6:$T$15&gt;TIME(20,30,0)))+((Orari!$U$6:$U$15&lt;=TIME(20,30,0))*(Orari!$V$6:$V$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -3111,51 +3111,51 @@
           <t>sabato 17 ottobre 2026</t>
         </is>
       </c>
-      <c r="B30" s="7">
+      <c r="B30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(9,30,0))*(Orari!$X$6:$X$15&gt;TIME(9,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(9,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C30" s="7">
+      <c r="C30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(10,30,0))*(Orari!$X$6:$X$15&gt;TIME(10,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(10,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D30" s="7">
+      <c r="D30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(11,30,0))*(Orari!$X$6:$X$15&gt;TIME(11,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(11,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E30" s="7">
+      <c r="E30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(12,30,0))*(Orari!$X$6:$X$15&gt;TIME(12,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(12,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F30" s="7">
+      <c r="F30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(13,30,0))*(Orari!$X$6:$X$15&gt;TIME(13,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(13,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G30" s="7">
+      <c r="G30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(14,30,0))*(Orari!$X$6:$X$15&gt;TIME(14,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(14,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H30" s="7">
+      <c r="H30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(15,30,0))*(Orari!$X$6:$X$15&gt;TIME(15,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(15,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I30" s="7">
+      <c r="I30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(16,30,0))*(Orari!$X$6:$X$15&gt;TIME(16,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(16,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J30" s="7">
+      <c r="J30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(17,30,0))*(Orari!$X$6:$X$15&gt;TIME(17,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(17,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K30" s="7">
+      <c r="K30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(18,30,0))*(Orari!$X$6:$X$15&gt;TIME(18,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(18,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L30" s="7">
+      <c r="L30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(19,30,0))*(Orari!$X$6:$X$15&gt;TIME(19,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(19,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M30" s="7">
+      <c r="M30" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$W$6:$W$15&lt;=TIME(20,30,0))*(Orari!$X$6:$X$15&gt;TIME(20,30,0)))+((Orari!$Y$6:$Y$15&lt;=TIME(20,30,0))*(Orari!$Z$6:$Z$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>
@@ -3166,51 +3166,51 @@
           <t>domenica 18 ottobre 2026</t>
         </is>
       </c>
-      <c r="B31" s="7">
+      <c r="B31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(9,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(9,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(9,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(9,30,0)))))</f>
         <v/>
       </c>
-      <c r="C31" s="7">
+      <c r="C31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(10,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(10,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(10,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(10,30,0)))))</f>
         <v/>
       </c>
-      <c r="D31" s="7">
+      <c r="D31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(11,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(11,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(11,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(11,30,0)))))</f>
         <v/>
       </c>
-      <c r="E31" s="7">
+      <c r="E31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(12,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(12,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(12,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(12,30,0)))))</f>
         <v/>
       </c>
-      <c r="F31" s="7">
+      <c r="F31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(13,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(13,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(13,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(13,30,0)))))</f>
         <v/>
       </c>
-      <c r="G31" s="7">
+      <c r="G31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(14,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(14,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(14,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(14,30,0)))))</f>
         <v/>
       </c>
-      <c r="H31" s="7">
+      <c r="H31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(15,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(15,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(15,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(15,30,0)))))</f>
         <v/>
       </c>
-      <c r="I31" s="7">
+      <c r="I31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(16,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(16,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(16,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(16,30,0)))))</f>
         <v/>
       </c>
-      <c r="J31" s="7">
+      <c r="J31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(17,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(17,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(17,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(17,30,0)))))</f>
         <v/>
       </c>
-      <c r="K31" s="7">
+      <c r="K31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(18,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(18,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(18,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(18,30,0)))))</f>
         <v/>
       </c>
-      <c r="L31" s="7">
+      <c r="L31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(19,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(19,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(19,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(19,30,0)))))</f>
         <v/>
       </c>
-      <c r="M31" s="7">
+      <c r="M31" s="6">
         <f>SUMPRODUCT((ISNUMBER(SEARCH("🔑",Orari!$A$6:$A$15)))*(((Orari!$AA$6:$AA$15&lt;=TIME(20,30,0))*(Orari!$AB$6:$AB$15&gt;TIME(20,30,0)))+((Orari!$AC$6:$AC$15&lt;=TIME(20,30,0))*(Orari!$AD$6:$AD$15&gt;TIME(20,30,0)))))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Orari: riposi più distanziati e domenica alternata rispetto alla settimana precedente
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RgW8tUpL59m5j1P2CKTdxn
</commit_message>
<xml_diff>
--- a/orari/Orari_12-18_ottobre_2026.xlsx
+++ b/orari/Orari_12-18_ottobre_2026.xlsx
@@ -885,38 +885,38 @@
       </c>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="H6" s="7" t="n"/>
-      <c r="I6" s="7" t="n"/>
-      <c r="J6" s="7" t="n"/>
-      <c r="K6" s="6" t="n"/>
-      <c r="L6" s="6" t="n"/>
-      <c r="M6" s="5" t="n">
+      <c r="L6" s="7" t="n"/>
+      <c r="M6" s="7" t="n"/>
+      <c r="N6" s="7" t="n"/>
+      <c r="O6" s="5" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="P6" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="Q6" s="6" t="n"/>
+      <c r="R6" s="6" t="n"/>
+      <c r="S6" s="6" t="n"/>
+      <c r="T6" s="6" t="n"/>
+      <c r="U6" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="N6" s="5" t="n">
+      <c r="V6" s="5" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="O6" s="6" t="n"/>
-      <c r="P6" s="6" t="n"/>
-      <c r="Q6" s="5" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="R6" s="5" t="n">
-        <v>0.7916666666666666</v>
-      </c>
-      <c r="S6" s="5" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="T6" s="5" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="U6" s="6" t="n"/>
-      <c r="V6" s="6" t="n"/>
       <c r="W6" s="5" t="n">
         <v>0.4166666666666667</v>
       </c>
@@ -965,37 +965,37 @@
       <c r="E7" s="7" t="n"/>
       <c r="F7" s="7" t="n"/>
       <c r="G7" s="5" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.375</v>
       </c>
       <c r="H7" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="I7" s="5" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="I7" s="5" t="n">
-        <v>0.7083333333333334</v>
-      </c>
       <c r="J7" s="5" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="K7" s="7" t="inlineStr">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="O7" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="L7" s="7" t="n"/>
-      <c r="M7" s="7" t="n"/>
-      <c r="N7" s="7" t="n"/>
-      <c r="O7" s="5" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="P7" s="5" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="Q7" s="5" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-      <c r="R7" s="5" t="n">
-        <v>0.875</v>
-      </c>
+      <c r="P7" s="7" t="n"/>
+      <c r="Q7" s="7" t="n"/>
+      <c r="R7" s="7" t="n"/>
       <c r="S7" s="5" t="n">
         <v>0.375</v>
       </c>
@@ -1008,10 +1008,10 @@
         <v>0.4583333333333333</v>
       </c>
       <c r="X7" s="5" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="Y7" s="5" t="n">
-        <v>0.7083333333333334</v>
+        <v>0.625</v>
       </c>
       <c r="Z7" s="5" t="n">
         <v>0.875</v>
@@ -1058,33 +1058,33 @@
         <v>0.875</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>0.375</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="H8" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="L8" s="7" t="n"/>
+      <c r="M8" s="7" t="n"/>
+      <c r="N8" s="7" t="n"/>
+      <c r="O8" s="6" t="n"/>
+      <c r="P8" s="6" t="n"/>
+      <c r="Q8" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="I8" s="5" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="J8" s="5" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="K8" s="5" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="L8" s="5" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="M8" s="6" t="n"/>
-      <c r="N8" s="6" t="n"/>
-      <c r="O8" s="7" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="P8" s="7" t="n"/>
-      <c r="Q8" s="7" t="n"/>
-      <c r="R8" s="7" t="n"/>
+      <c r="R8" s="5" t="n">
+        <v>0.875</v>
+      </c>
       <c r="S8" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
@@ -1094,16 +1094,16 @@
       <c r="U8" s="7" t="n"/>
       <c r="V8" s="7" t="n"/>
       <c r="W8" s="5" t="n">
-        <v>0.4583333333333333</v>
+        <v>0.375</v>
       </c>
       <c r="X8" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="Y8" s="5" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="Y8" s="5" t="n">
-        <v>0.7083333333333334</v>
-      </c>
       <c r="Z8" s="5" t="n">
-        <v>0.875</v>
+        <v>0.7916666666666666</v>
       </c>
       <c r="AA8" s="5" t="n">
         <v>0.375</v>
@@ -1156,30 +1156,30 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="L9" s="5" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>0.625</v>
+        <v>0.7083333333333334</v>
       </c>
       <c r="N9" s="5" t="n">
         <v>0.875</v>
       </c>
-      <c r="O9" s="7" t="inlineStr">
+      <c r="O9" s="6" t="n"/>
+      <c r="P9" s="6" t="n"/>
+      <c r="Q9" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="R9" s="5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="S9" s="7" t="inlineStr">
         <is>
           <t>RIPOSO</t>
         </is>
       </c>
-      <c r="P9" s="7" t="n"/>
-      <c r="Q9" s="7" t="n"/>
-      <c r="R9" s="7" t="n"/>
-      <c r="S9" s="6" t="n"/>
-      <c r="T9" s="6" t="n"/>
-      <c r="U9" s="5" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="V9" s="5" t="n">
-        <v>0.875</v>
-      </c>
+      <c r="T9" s="7" t="n"/>
+      <c r="U9" s="7" t="n"/>
+      <c r="V9" s="7" t="n"/>
       <c r="W9" s="5" t="n">
         <v>0.375</v>
       </c>
@@ -1235,36 +1235,36 @@
       <c r="F10" s="5" t="n">
         <v>0.7916666666666666</v>
       </c>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="5" t="n">
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>RIPOSO</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="7" t="n"/>
+      <c r="J10" s="7" t="n"/>
+      <c r="K10" s="6" t="n"/>
+      <c r="L10" s="6" t="n"/>
+      <c r="M10" s="5" t="n">
         <v>0.625</v>
       </c>
-      <c r="J10" s="5" t="n">
+      <c r="N10" s="5" t="n">
         <v>0.875</v>
       </c>
-      <c r="K10" s="7" t="inlineStr">
-        <is>
-          <t>RIPOSO</t>
-        </is>
-      </c>
-      <c r="L10" s="7" t="n"/>
-      <c r="M10" s="7" t="n"/>
-      <c r="N10" s="7" t="n"/>
       <c r="O10" s="5" t="n">
         <v>0.375</v>
       </c>
       <c r="P10" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="Q10" s="6" t="n"/>
+      <c r="R10" s="6" t="n"/>
+      <c r="S10" s="5" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="T10" s="5" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="Q10" s="5" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="R10" s="5" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="S10" s="6" t="n"/>
-      <c r="T10" s="6" t="n"/>
       <c r="U10" s="5" t="n">
         <v>0.625</v>
       </c>
@@ -1272,16 +1272,16 @@
         <v>0.875</v>
       </c>
       <c r="W10" s="5" t="n">
-        <v>0.375</v>
+        <v>0.4583333333333333</v>
       </c>
       <c r="X10" s="5" t="n">
-        <v>0.5416666666666666</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="Y10" s="5" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.625</v>
       </c>
       <c r="Z10" s="5" t="n">
-        <v>0.7916666666666666</v>
+        <v>0.875</v>
       </c>
       <c r="AA10" s="7" t="inlineStr">
         <is>
@@ -1756,21 +1756,21 @@
   </sheetData>
   <mergeCells count="46">
     <mergeCell ref="W4:X4"/>
+    <mergeCell ref="S9:V9"/>
     <mergeCell ref="Y4:Z4"/>
     <mergeCell ref="K14:N14"/>
     <mergeCell ref="O12:R12"/>
-    <mergeCell ref="O8:R8"/>
     <mergeCell ref="AA3:AD3"/>
     <mergeCell ref="C7:F7"/>
-    <mergeCell ref="K7:N7"/>
-    <mergeCell ref="K10:N10"/>
     <mergeCell ref="AA11:AD11"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C13:F13"/>
     <mergeCell ref="E4:F4"/>
+    <mergeCell ref="K6:N6"/>
     <mergeCell ref="G9:J9"/>
     <mergeCell ref="C3:F3"/>
     <mergeCell ref="K3:N3"/>
+    <mergeCell ref="O7:R7"/>
     <mergeCell ref="O3:R3"/>
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="G11:J11"/>
@@ -1781,21 +1781,21 @@
     <mergeCell ref="Q4:R4"/>
     <mergeCell ref="AC4:AD4"/>
     <mergeCell ref="AF3:AF5"/>
-    <mergeCell ref="O9:R9"/>
     <mergeCell ref="AA13:AD13"/>
     <mergeCell ref="S3:V3"/>
     <mergeCell ref="S8:V8"/>
     <mergeCell ref="AE3:AE5"/>
     <mergeCell ref="AA6:AD6"/>
     <mergeCell ref="AA15:AD15"/>
+    <mergeCell ref="G10:J10"/>
     <mergeCell ref="S14:V14"/>
     <mergeCell ref="G4:H4"/>
-    <mergeCell ref="G6:J6"/>
     <mergeCell ref="I4:J4"/>
     <mergeCell ref="W3:Z3"/>
     <mergeCell ref="G3:J3"/>
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="K12:N12"/>
+    <mergeCell ref="K8:N8"/>
     <mergeCell ref="K4:L4"/>
     <mergeCell ref="W12:Z12"/>
     <mergeCell ref="M4:N4"/>

</xml_diff>